<commit_message>
Perbarui data SE2026 06/09/2026  8:00:23,28
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="314">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 5 Sep 2026, 06.51</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 6 Sep 2026, 07.59</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,19 +334,19 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>20,47</t>
-  </si>
-  <si>
-    <t>1,2</t>
-  </si>
-  <si>
-    <t>1,84</t>
-  </si>
-  <si>
-    <t>38,46</t>
-  </si>
-  <si>
-    <t>10,11</t>
+    <t>20,4</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>1,85</t>
+  </si>
+  <si>
+    <t>38,87</t>
+  </si>
+  <si>
+    <t>9,97</t>
   </si>
   <si>
     <t>0,19</t>
@@ -355,37 +355,40 @@
     <t>7,64</t>
   </si>
   <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>4,97</t>
-  </si>
-  <si>
-    <t>12,8</t>
+    <t>0,85</t>
+  </si>
+  <si>
+    <t>4,92</t>
+  </si>
+  <si>
+    <t>12,68</t>
   </si>
   <si>
     <t>1801</t>
@@ -406,7 +409,7 @@
     <t>0,99</t>
   </si>
   <si>
-    <t>47,84</t>
+    <t>47,85</t>
   </si>
   <si>
     <t>4,02</t>
@@ -421,9 +424,6 @@
     <t>0,01</t>
   </si>
   <si>
-    <t>0,06</t>
-  </si>
-  <si>
     <t>0,13</t>
   </si>
   <si>
@@ -433,13 +433,13 @@
     <t>0,35</t>
   </si>
   <si>
-    <t>2,8</t>
+    <t>2,79</t>
   </si>
   <si>
     <t>3,56</t>
   </si>
   <si>
-    <t>14,94</t>
+    <t>14,93</t>
   </si>
   <si>
     <t>1802</t>
@@ -448,19 +448,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>13,68</t>
+    <t>13,59</t>
   </si>
   <si>
     <t>0,5</t>
   </si>
   <si>
-    <t>0,88</t>
-  </si>
-  <si>
-    <t>27,01</t>
-  </si>
-  <si>
-    <t>30,07</t>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>27,24</t>
+  </si>
+  <si>
+    <t>30,13</t>
   </si>
   <si>
     <t>6,41</t>
@@ -475,10 +475,10 @@
     <t>0,47</t>
   </si>
   <si>
-    <t>4,71</t>
-  </si>
-  <si>
-    <t>15,8</t>
+    <t>4,65</t>
+  </si>
+  <si>
+    <t>15,86</t>
   </si>
   <si>
     <t>1803</t>
@@ -487,37 +487,40 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>16,18</t>
-  </si>
-  <si>
-    <t>2,05</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>48,61</t>
-  </si>
-  <si>
-    <t>9,05</t>
-  </si>
-  <si>
-    <t>10,55</t>
+    <t>16,12</t>
+  </si>
+  <si>
+    <t>2,03</t>
+  </si>
+  <si>
+    <t>0,39</t>
+  </si>
+  <si>
+    <t>48,75</t>
+  </si>
+  <si>
+    <t>8,93</t>
+  </si>
+  <si>
+    <t>10,53</t>
   </si>
   <si>
     <t>0,38</t>
   </si>
   <si>
-    <t>0,72</t>
-  </si>
-  <si>
-    <t>1,04</t>
-  </si>
-  <si>
-    <t>3,79</t>
-  </si>
-  <si>
-    <t>7,23</t>
+    <t>0,71</t>
+  </si>
+  <si>
+    <t>1,03</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>3,75</t>
+  </si>
+  <si>
+    <t>7,17</t>
   </si>
   <si>
     <t>1804</t>
@@ -526,412 +529,424 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>24,1</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>7,4</t>
-  </si>
-  <si>
-    <t>33,25</t>
-  </si>
-  <si>
-    <t>12,55</t>
+    <t>24,18</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>7,26</t>
+  </si>
+  <si>
+    <t>33,6</t>
+  </si>
+  <si>
+    <t>12,43</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>2,08</t>
+  </si>
+  <si>
+    <t>9,03</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,79</t>
+  </si>
+  <si>
+    <t>2,17</t>
+  </si>
+  <si>
+    <t>1,12</t>
+  </si>
+  <si>
+    <t>46,77</t>
+  </si>
+  <si>
+    <t>4,39</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>12,9</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>3,16</t>
+  </si>
+  <si>
+    <t>11,53</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,89</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>37,65</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>7,83</t>
+  </si>
+  <si>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>1,15</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>6,8</t>
+  </si>
+  <si>
+    <t>10,5</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,61</t>
+  </si>
+  <si>
+    <t>1,22</t>
+  </si>
+  <si>
+    <t>43,19</t>
+  </si>
+  <si>
+    <t>16,74</t>
+  </si>
+  <si>
+    <t>6,18</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>4,4</t>
+  </si>
+  <si>
+    <t>7,09</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,68</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>29,14</t>
+  </si>
+  <si>
+    <t>17,98</t>
+  </si>
+  <si>
+    <t>6,07</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>7,41</t>
+  </si>
+  <si>
+    <t>14,27</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,73</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>30,78</t>
+  </si>
+  <si>
+    <t>1,79</t>
+  </si>
+  <si>
+    <t>5,89</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>8,34</t>
+  </si>
+  <si>
+    <t>20,57</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,71</t>
+  </si>
+  <si>
+    <t>31,92</t>
+  </si>
+  <si>
+    <t>5,31</t>
+  </si>
+  <si>
+    <t>5,22</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>0,84</t>
+  </si>
+  <si>
+    <t>8,25</t>
+  </si>
+  <si>
+    <t>28,22</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>29,39</t>
+  </si>
+  <si>
+    <t>2,34</t>
+  </si>
+  <si>
+    <t>1,24</t>
+  </si>
+  <si>
+    <t>39,46</t>
+  </si>
+  <si>
+    <t>6,68</t>
+  </si>
+  <si>
+    <t>4,33</t>
+  </si>
+  <si>
+    <t>2,68</t>
+  </si>
+  <si>
+    <t>7,53</t>
+  </si>
+  <si>
+    <t>4,79</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>18,72</t>
+  </si>
+  <si>
+    <t>1,47</t>
+  </si>
+  <si>
+    <t>1,13</t>
+  </si>
+  <si>
+    <t>33,55</t>
+  </si>
+  <si>
+    <t>15,47</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>4,08</t>
+  </si>
+  <si>
+    <t>17,85</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,17</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>49,83</t>
+  </si>
+  <si>
+    <t>13,57</t>
+  </si>
+  <si>
+    <t>10,64</t>
+  </si>
+  <si>
+    <t>0,52</t>
+  </si>
+  <si>
+    <t>6,06</t>
+  </si>
+  <si>
+    <t>7,28</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,31</t>
+  </si>
+  <si>
+    <t>3,4</t>
+  </si>
+  <si>
+    <t>31,95</t>
+  </si>
+  <si>
+    <t>4,54</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>15,88</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>1,89</t>
+  </si>
+  <si>
+    <t>4,06</t>
+  </si>
+  <si>
+    <t>17,49</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,33</t>
+  </si>
+  <si>
+    <t>5,83</t>
+  </si>
+  <si>
+    <t>30,52</t>
+  </si>
+  <si>
+    <t>3,97</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>3,07</t>
   </si>
   <si>
     <t>0,7</t>
   </si>
   <si>
-    <t>7,12</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>1,87</t>
-  </si>
-  <si>
-    <t>2,15</t>
-  </si>
-  <si>
-    <t>9,1</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>2,2</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>46,34</t>
-  </si>
-  <si>
-    <t>4,59</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>13,01</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>3,19</t>
-  </si>
-  <si>
-    <t>11,59</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,9</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>37,69</t>
-  </si>
-  <si>
-    <t>13,96</t>
-  </si>
-  <si>
-    <t>7,83</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>1,15</t>
-  </si>
-  <si>
-    <t>6,82</t>
-  </si>
-  <si>
-    <t>10,48</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,64</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>1,24</t>
-  </si>
-  <si>
-    <t>43,12</t>
-  </si>
-  <si>
-    <t>16,74</t>
-  </si>
-  <si>
-    <t>6,18</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>4,46</t>
-  </si>
-  <si>
-    <t>7,1</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,78</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>28,48</t>
-  </si>
-  <si>
-    <t>18,25</t>
-  </si>
-  <si>
-    <t>6,11</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>7,41</t>
-  </si>
-  <si>
-    <t>14,13</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,79</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>30,67</t>
-  </si>
-  <si>
-    <t>1,79</t>
-  </si>
-  <si>
-    <t>5,82</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>8,38</t>
-  </si>
-  <si>
-    <t>20,64</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,72</t>
-  </si>
-  <si>
-    <t>31,71</t>
-  </si>
-  <si>
-    <t>5,33</t>
-  </si>
-  <si>
-    <t>5,24</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>8,29</t>
-  </si>
-  <si>
-    <t>28,33</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>29,54</t>
-  </si>
-  <si>
-    <t>2,35</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>39,23</t>
-  </si>
-  <si>
-    <t>6,74</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>4,37</t>
-  </si>
-  <si>
-    <t>2,67</t>
-  </si>
-  <si>
-    <t>7,55</t>
-  </si>
-  <si>
-    <t>4,79</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>18,6</t>
-  </si>
-  <si>
-    <t>1,47</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>33,54</t>
-  </si>
-  <si>
-    <t>15,52</t>
-  </si>
-  <si>
-    <t>6,55</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>4,07</t>
-  </si>
-  <si>
-    <t>17,91</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,3</t>
-  </si>
-  <si>
-    <t>48,09</t>
-  </si>
-  <si>
-    <t>14,57</t>
-  </si>
-  <si>
-    <t>10,84</t>
-  </si>
-  <si>
-    <t>6,32</t>
-  </si>
-  <si>
-    <t>7,79</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,27</t>
-  </si>
-  <si>
-    <t>3,3</t>
-  </si>
-  <si>
-    <t>32,05</t>
-  </si>
-  <si>
-    <t>15,83</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>4,43</t>
-  </si>
-  <si>
-    <t>17,44</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,36</t>
-  </si>
-  <si>
-    <t>5,84</t>
-  </si>
-  <si>
-    <t>30,45</t>
-  </si>
-  <si>
-    <t>3,97</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>3,08</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>0,93</t>
-  </si>
-  <si>
-    <t>3,78</t>
-  </si>
-  <si>
-    <t>33,61</t>
+    <t>1,01</t>
+  </si>
+  <si>
+    <t>3,73</t>
   </si>
   <si>
     <t/>
@@ -1911,121 +1926,121 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>122688</v>
+        <v>124095</v>
       </c>
       <c r="D6" s="6">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>25110</v>
+        <v>25314</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1473</v>
+        <v>1482</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2256</v>
+        <v>2297</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>47186</v>
+        <v>48240</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12401</v>
+        <v>12368</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>9373</v>
+        <v>9481</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="U6" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="V6" s="6">
+        <v>20</v>
+      </c>
+      <c r="W6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="V6" s="6">
-        <v>21</v>
-      </c>
-      <c r="W6" s="7" t="s">
+      <c r="X6" s="6">
+        <v>200</v>
+      </c>
+      <c r="Y6" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="X6" s="6">
-        <v>199</v>
-      </c>
-      <c r="Y6" s="7" t="s">
-        <v>116</v>
       </c>
       <c r="Z6" s="6">
         <v>26</v>
       </c>
       <c r="AA6" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AB6" s="6">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD6" s="6">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AF6" s="6">
         <v>0</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH6" s="6">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AJ6" s="6">
         <v>297</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AL6" s="6">
         <v>39</v>
       </c>
       <c r="AM6" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="AN6" s="6">
+        <v>80</v>
+      </c>
+      <c r="AO6" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="AN6" s="6">
-        <v>81</v>
-      </c>
-      <c r="AO6" s="7" t="s">
-        <v>117</v>
       </c>
       <c r="AP6" s="6">
         <v>689</v>
@@ -2037,96 +2052,96 @@
         <v>115</v>
       </c>
       <c r="AS6" s="7" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AT6" s="6">
         <v>1049</v>
       </c>
       <c r="AU6" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AV6" s="6">
-        <v>6099</v>
+        <v>6102</v>
       </c>
       <c r="AW6" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AX6" s="6">
-        <v>15703</v>
+        <v>15733</v>
       </c>
       <c r="AY6" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C7" s="9">
-        <v>7783</v>
+        <v>7781</v>
       </c>
       <c r="D7" s="9">
         <v>8</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F7" s="9">
         <v>1492</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H7" s="9">
         <v>74</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J7" s="9">
         <v>77</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L7" s="9">
         <v>3723</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N7" s="9">
         <v>313</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P7" s="9">
         <v>11</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R7" s="9">
         <v>352</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="T7" s="9">
         <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="V7" s="9">
         <v>1</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="X7" s="9">
         <v>15</v>
@@ -2138,7 +2153,7 @@
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AB7" s="9">
         <v>6</v>
@@ -2150,19 +2165,19 @@
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH7" s="9">
         <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ7" s="9">
         <v>10</v>
@@ -2174,7 +2189,7 @@
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AN7" s="9">
         <v>3</v>
@@ -2195,7 +2210,7 @@
         <v>138</v>
       </c>
       <c r="AT7" s="9">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>140</v>
@@ -2207,7 +2222,7 @@
         <v>141</v>
       </c>
       <c r="AX7" s="9">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="AY7" s="10" t="s">
         <v>142</v>
@@ -2227,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F8" s="9">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>145</v>
@@ -2242,19 +2257,19 @@
         <v>146</v>
       </c>
       <c r="J8" s="9">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>147</v>
       </c>
       <c r="L8" s="9">
-        <v>918</v>
+        <v>926</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>148</v>
       </c>
       <c r="N8" s="9">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="O8" s="10" t="s">
         <v>149</v>
@@ -2263,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R8" s="9">
         <v>218</v>
@@ -2275,13 +2290,13 @@
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X8" s="9">
         <v>6</v>
@@ -2293,31 +2308,31 @@
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
@@ -2329,13 +2344,13 @@
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
@@ -2347,22 +2362,22 @@
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="AT8" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="AV8" s="9">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="AW8" s="10" t="s">
         <v>154</v>
       </c>
       <c r="AX8" s="9">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="AY8" s="10" t="s">
         <v>155</v>
@@ -2376,16 +2391,16 @@
         <v>157</v>
       </c>
       <c r="C9" s="9">
-        <v>9593</v>
+        <v>9703</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F9" s="9">
-        <v>1552</v>
+        <v>1564</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>158</v>
@@ -2397,19 +2412,19 @@
         <v>159</v>
       </c>
       <c r="J9" s="9">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>160</v>
       </c>
       <c r="L9" s="9">
-        <v>4663</v>
+        <v>4730</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>161</v>
       </c>
       <c r="N9" s="9">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>162</v>
@@ -2418,10 +2433,10 @@
         <v>3</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R9" s="9">
-        <v>1012</v>
+        <v>1022</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>163</v>
@@ -2430,16 +2445,16 @@
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="V9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="X9" s="9">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y9" s="10" t="s">
         <v>164</v>
@@ -2448,31 +2463,31 @@
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD9" s="9">
         <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ9" s="9">
         <v>69</v>
@@ -2484,13 +2499,13 @@
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP9" s="9">
         <v>100</v>
@@ -2502,87 +2517,87 @@
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AT9" s="9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>120</v>
+        <v>167</v>
       </c>
       <c r="AV9" s="9">
         <v>364</v>
       </c>
       <c r="AW9" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AX9" s="9">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="AY9" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C10" s="9">
-        <v>20976</v>
+        <v>21204</v>
       </c>
       <c r="D10" s="9">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>151</v>
       </c>
       <c r="F10" s="9">
-        <v>5055</v>
+        <v>5128</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H10" s="9">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J10" s="9">
-        <v>1553</v>
+        <v>1539</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L10" s="9">
-        <v>6974</v>
+        <v>7125</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N10" s="9">
-        <v>2632</v>
+        <v>2636</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P10" s="9">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="R10" s="9">
-        <v>1493</v>
+        <v>1520</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="T10" s="9">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="U10" s="10" t="s">
         <v>136</v>
@@ -2591,37 +2606,37 @@
         <v>7</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="X10" s="9">
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AB10" s="9">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>136</v>
+        <v>167</v>
       </c>
       <c r="AD10" s="9">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH10" s="9">
         <v>8</v>
@@ -2633,13 +2648,13 @@
         <v>13</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AN10" s="9">
         <v>52</v>
@@ -2657,75 +2672,75 @@
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AT10" s="9">
+        <v>385</v>
+      </c>
+      <c r="AU10" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="AT10" s="9">
-        <v>392</v>
-      </c>
-      <c r="AU10" s="10" t="s">
+      <c r="AV10" s="9">
+        <v>442</v>
+      </c>
+      <c r="AW10" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="AV10" s="9">
-        <v>452</v>
-      </c>
-      <c r="AW10" s="10" t="s">
+      <c r="AX10" s="9">
+        <v>1915</v>
+      </c>
+      <c r="AY10" s="10" t="s">
         <v>181</v>
-      </c>
-      <c r="AX10" s="9">
-        <v>1909</v>
-      </c>
-      <c r="AY10" s="10" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="9">
+        <v>13578</v>
+      </c>
+      <c r="D11" s="9">
+        <v>12</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="F11" s="9">
+        <v>2144</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="C11" s="9">
-        <v>13465</v>
-      </c>
-      <c r="D11" s="9">
-        <v>11</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="F11" s="9">
-        <v>2128</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>155</v>
-      </c>
       <c r="H11" s="9">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="I11" s="10" t="s">
         <v>185</v>
       </c>
       <c r="J11" s="9">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
       <c r="L11" s="9">
-        <v>6240</v>
+        <v>6350</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>187</v>
       </c>
       <c r="N11" s="9">
-        <v>618</v>
+        <v>596</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>188</v>
       </c>
       <c r="P11" s="9">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q11" s="10" t="s">
         <v>189</v>
@@ -2764,22 +2779,22 @@
         <v>3</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD11" s="9">
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH11" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AI11" s="10" t="s">
         <v>138</v>
@@ -2788,120 +2803,120 @@
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AN11" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AP11" s="9">
         <v>86</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AT11" s="9">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AV11" s="9">
         <v>429</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AX11" s="9">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C12" s="9">
-        <v>5221</v>
+        <v>5209</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F12" s="9">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J12" s="9">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L12" s="9">
-        <v>1968</v>
+        <v>1961</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P12" s="9">
         <v>0</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R12" s="9">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V12" s="9">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X12" s="9">
         <v>26</v>
@@ -2919,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD12" s="9">
         <v>10</v>
@@ -2931,132 +2946,132 @@
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH12" s="9">
         <v>0</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ12" s="9">
         <v>31</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AN12" s="9">
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP12" s="9">
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AT12" s="9">
         <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="AV12" s="9">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C13" s="9">
-        <v>4933</v>
+        <v>4934</v>
       </c>
       <c r="D13" s="9">
         <v>1</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F13" s="9">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="J13" s="9">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L13" s="9">
-        <v>2127</v>
+        <v>2131</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="N13" s="9">
         <v>826</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P13" s="9">
         <v>5</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="R13" s="9">
         <v>305</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V13" s="9">
         <v>3</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
@@ -3068,25 +3083,25 @@
         <v>1</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH13" s="9">
         <v>2</v>
@@ -3098,7 +3113,7 @@
         <v>32</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
@@ -3110,13 +3125,13 @@
         <v>5</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AP13" s="9">
         <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
@@ -3125,93 +3140,93 @@
         <v>153</v>
       </c>
       <c r="AT13" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>189</v>
+        <v>219</v>
       </c>
       <c r="AV13" s="9">
+        <v>217</v>
+      </c>
+      <c r="AW13" s="10" t="s">
         <v>220</v>
-      </c>
-      <c r="AW13" s="10" t="s">
-        <v>218</v>
       </c>
       <c r="AX13" s="9">
         <v>350</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C14" s="9">
-        <v>4926</v>
+        <v>4956</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F14" s="9">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="J14" s="9">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="L14" s="9">
-        <v>1403</v>
+        <v>1444</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="N14" s="9">
-        <v>899</v>
+        <v>891</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="R14" s="9">
         <v>301</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X14" s="9">
         <v>9</v>
@@ -3223,210 +3238,210 @@
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ14" s="9">
         <v>16</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>228</v>
+        <v>194</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AN14" s="9">
         <v>1</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AP14" s="9">
         <v>34</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AT14" s="9">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>153</v>
+        <v>231</v>
       </c>
       <c r="AV14" s="9">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="AX14" s="9">
-        <v>696</v>
+        <v>707</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C15" s="9">
-        <v>12596</v>
+        <v>12641</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F15" s="9">
-        <v>3878</v>
+        <v>3885</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="J15" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>179</v>
+        <v>138</v>
       </c>
       <c r="L15" s="9">
-        <v>3863</v>
+        <v>3891</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="P15" s="9">
         <v>1</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="R15" s="9">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>239</v>
+        <v>194</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH15" s="9">
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AL15" s="9">
         <v>3</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AN15" s="9">
         <v>1</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AP15" s="9">
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>211</v>
+        <v>241</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
@@ -3435,33 +3450,33 @@
         <v>152</v>
       </c>
       <c r="AT15" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>179</v>
+        <v>120</v>
       </c>
       <c r="AV15" s="9">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AX15" s="9">
         <v>2600</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C16" s="9">
-        <v>5080</v>
+        <v>5100</v>
       </c>
       <c r="D16" s="9">
         <v>2</v>
@@ -3470,100 +3485,100 @@
         <v>138</v>
       </c>
       <c r="F16" s="9">
-        <v>900</v>
+        <v>903</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="J16" s="9">
         <v>8</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L16" s="9">
-        <v>1611</v>
+        <v>1628</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N16" s="9">
         <v>271</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P16" s="9">
         <v>1</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="R16" s="9">
         <v>266</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X16" s="9">
         <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="AB16" s="9">
         <v>1</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="AF16" s="9">
         <v>0</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ16" s="9">
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3575,90 +3590,90 @@
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP16" s="9">
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AT16" s="9">
         <v>33</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AV16" s="9">
         <v>421</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AX16" s="9">
         <v>1439</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C17" s="9">
-        <v>9963</v>
+        <v>10045</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>228</v>
+        <v>194</v>
       </c>
       <c r="F17" s="9">
-        <v>2943</v>
+        <v>2952</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H17" s="9">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J17" s="9">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L17" s="9">
-        <v>3908</v>
+        <v>3964</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="N17" s="9">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>260</v>
+        <v>191</v>
       </c>
       <c r="R17" s="9">
         <v>435</v>
@@ -3670,7 +3685,7 @@
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="V17" s="9">
         <v>4</v>
@@ -3694,7 +3709,7 @@
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
@@ -3706,58 +3721,58 @@
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AN17" s="9">
         <v>7</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="AR17" s="9">
         <v>9</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AT17" s="9">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="AU17" s="10" t="s">
         <v>262</v>
       </c>
       <c r="AV17" s="9">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="AW17" s="10" t="s">
         <v>263</v>
       </c>
       <c r="AX17" s="9">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="AY17" s="10" t="s">
         <v>264</v>
@@ -3771,16 +3786,16 @@
         <v>266</v>
       </c>
       <c r="C18" s="9">
-        <v>10258</v>
+        <v>10293</v>
       </c>
       <c r="D18" s="9">
         <v>2</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F18" s="9">
-        <v>1908</v>
+        <v>1927</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>267</v>
@@ -3792,13 +3807,13 @@
         <v>268</v>
       </c>
       <c r="J18" s="9">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K18" s="10" t="s">
         <v>269</v>
       </c>
       <c r="L18" s="9">
-        <v>3441</v>
+        <v>3453</v>
       </c>
       <c r="M18" s="10" t="s">
         <v>270</v>
@@ -3813,10 +3828,10 @@
         <v>1</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="R18" s="9">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="S18" s="10" t="s">
         <v>272</v>
@@ -3831,359 +3846,359 @@
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X18" s="9">
         <v>5</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AB18" s="9">
         <v>1</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AD18" s="9">
         <v>3</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AN18" s="9">
         <v>2</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AP18" s="9">
         <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>223</v>
+        <v>274</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AT18" s="9">
         <v>2</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AV18" s="9">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AX18" s="9">
         <v>1837</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C19" s="9">
-        <v>10866</v>
+        <v>11622</v>
       </c>
       <c r="D19" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F19" s="9">
-        <v>1228</v>
+        <v>1298</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="J19" s="9">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>135</v>
+        <v>281</v>
       </c>
       <c r="L19" s="9">
-        <v>5225</v>
+        <v>5791</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="N19" s="9">
-        <v>1583</v>
+        <v>1577</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R19" s="9">
-        <v>1178</v>
+        <v>1237</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X19" s="9">
         <v>18</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>274</v>
+        <v>152</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP19" s="9">
         <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>121</v>
+        <v>285</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AT19" s="9">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="AV19" s="9">
-        <v>687</v>
+        <v>704</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="AX19" s="9">
         <v>846</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C20" s="9">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="F20" s="9">
         <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J20" s="9">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="L20" s="9">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>134</v>
+        <v>293</v>
       </c>
       <c r="P20" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>249</v>
+        <v>294</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>250</v>
+        <v>123</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH20" s="9">
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
@@ -4195,13 +4210,13 @@
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
@@ -4210,51 +4225,51 @@
         <v>164</v>
       </c>
       <c r="AT20" s="9">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>237</v>
+        <v>298</v>
       </c>
       <c r="AV20" s="9">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="C21" s="9">
-        <v>2568</v>
+        <v>2572</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F21" s="9">
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="J21" s="9">
         <v>2</v>
@@ -4263,46 +4278,46 @@
         <v>106</v>
       </c>
       <c r="L21" s="9">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4314,49 +4329,49 @@
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>176</v>
+        <v>309</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
@@ -4365,147 +4380,147 @@
         <v>138</v>
       </c>
       <c r="AT21" s="9">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="AV21" s="9">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="AX21" s="9">
         <v>863</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>306</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C22" s="12">
-        <v>122688</v>
+        <v>124095</v>
       </c>
       <c r="D22" s="12">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>25110</v>
+        <v>25314</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1473</v>
+        <v>1482</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2256</v>
+        <v>2297</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>47186</v>
+        <v>48240</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12401</v>
+        <v>12368</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>9373</v>
+        <v>9481</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="U22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="V22" s="12">
+        <v>20</v>
+      </c>
+      <c r="W22" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="V22" s="12">
-        <v>21</v>
-      </c>
-      <c r="W22" s="13" t="s">
+      <c r="X22" s="12">
+        <v>200</v>
+      </c>
+      <c r="Y22" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="X22" s="12">
-        <v>199</v>
-      </c>
-      <c r="Y22" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="Z22" s="12">
         <v>26</v>
       </c>
       <c r="AA22" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AB22" s="12">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD22" s="12">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AF22" s="12">
         <v>0</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AH22" s="12">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AJ22" s="12">
         <v>297</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AL22" s="12">
         <v>39</v>
       </c>
       <c r="AM22" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="AN22" s="12">
+        <v>80</v>
+      </c>
+      <c r="AO22" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="AN22" s="12">
-        <v>81</v>
-      </c>
-      <c r="AO22" s="13" t="s">
-        <v>117</v>
       </c>
       <c r="AP22" s="12">
         <v>689</v>
@@ -4517,25 +4532,25 @@
         <v>115</v>
       </c>
       <c r="AS22" s="13" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="AT22" s="12">
         <v>1049</v>
       </c>
       <c r="AU22" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AV22" s="12">
-        <v>6099</v>
+        <v>6102</v>
       </c>
       <c r="AW22" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AX22" s="12">
-        <v>15703</v>
+        <v>15733</v>
       </c>
       <c r="AY22" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 07/09/2026 16:00:01,99
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="308">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 6 Sep 2026, 07.59</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 7 Sep 2026, 15.57</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,580 +334,568 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>20,4</t>
+    <t>20,38</t>
   </si>
   <si>
     <t>1,19</t>
   </si>
   <si>
-    <t>1,85</t>
-  </si>
-  <si>
-    <t>38,87</t>
-  </si>
-  <si>
-    <t>9,97</t>
+    <t>1,81</t>
+  </si>
+  <si>
+    <t>39,06</t>
+  </si>
+  <si>
+    <t>9,98</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>7,61</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>0,55</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,84</t>
+  </si>
+  <si>
+    <t>4,9</t>
+  </si>
+  <si>
+    <t>12,6</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>19,17</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>47,85</t>
+  </si>
+  <si>
+    <t>4,02</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,52</t>
+  </si>
+  <si>
+    <t>0,01</t>
   </si>
   <si>
     <t>0,19</t>
   </si>
   <si>
-    <t>7,64</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>0,09</t>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>2,79</t>
+  </si>
+  <si>
+    <t>3,56</t>
+  </si>
+  <si>
+    <t>14,93</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,69</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>27,21</t>
+  </si>
+  <si>
+    <t>30,09</t>
+  </si>
+  <si>
+    <t>6,41</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>4,64</t>
+  </si>
+  <si>
+    <t>15,84</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>16,11</t>
+  </si>
+  <si>
+    <t>2,01</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>49,13</t>
+  </si>
+  <si>
+    <t>8,88</t>
+  </si>
+  <si>
+    <t>10,52</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>1,02</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>3,73</t>
+  </si>
+  <si>
+    <t>7,12</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>24,28</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>7,25</t>
+  </si>
+  <si>
+    <t>33,64</t>
+  </si>
+  <si>
+    <t>12,37</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>7,15</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>2,07</t>
+  </si>
+  <si>
+    <t>8,99</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>15,8</t>
+  </si>
+  <si>
+    <t>2,15</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>46,87</t>
+  </si>
+  <si>
+    <t>4,35</t>
+  </si>
+  <si>
+    <t>12,88</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>3,14</t>
+  </si>
+  <si>
+    <t>11,52</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,89</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>37,65</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>7,83</t>
+  </si>
+  <si>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>1,15</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>6,8</t>
+  </si>
+  <si>
+    <t>10,5</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,54</t>
+  </si>
+  <si>
+    <t>1,51</t>
+  </si>
+  <si>
+    <t>43,01</t>
+  </si>
+  <si>
+    <t>16,67</t>
+  </si>
+  <si>
+    <t>6,16</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>4,38</t>
+  </si>
+  <si>
+    <t>7,06</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,67</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>29,12</t>
+  </si>
+  <si>
+    <t>17,97</t>
+  </si>
+  <si>
+    <t>6,07</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>7,42</t>
+  </si>
+  <si>
+    <t>14,26</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,7</t>
+  </si>
+  <si>
+    <t>0,43</t>
+  </si>
+  <si>
+    <t>30,8</t>
+  </si>
+  <si>
+    <t>1,79</t>
+  </si>
+  <si>
+    <t>5,89</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>8,37</t>
+  </si>
+  <si>
+    <t>20,54</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,7</t>
+  </si>
+  <si>
+    <t>31,95</t>
+  </si>
+  <si>
+    <t>5,31</t>
+  </si>
+  <si>
+    <t>5,21</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>8,25</t>
+  </si>
+  <si>
+    <t>28,2</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>29,26</t>
+  </si>
+  <si>
+    <t>2,31</t>
+  </si>
+  <si>
+    <t>1,26</t>
+  </si>
+  <si>
+    <t>39,77</t>
+  </si>
+  <si>
+    <t>6,6</t>
+  </si>
+  <si>
+    <t>4,32</t>
+  </si>
+  <si>
+    <t>2,65</t>
+  </si>
+  <si>
+    <t>7,5</t>
+  </si>
+  <si>
+    <t>4,76</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>18,85</t>
+  </si>
+  <si>
+    <t>1,46</t>
+  </si>
+  <si>
+    <t>1,12</t>
+  </si>
+  <si>
+    <t>33,66</t>
+  </si>
+  <si>
+    <t>15,45</t>
+  </si>
+  <si>
+    <t>6,5</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>4,05</t>
+  </si>
+  <si>
+    <t>17,72</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,18</t>
+  </si>
+  <si>
+    <t>50,54</t>
+  </si>
+  <si>
+    <t>13,98</t>
+  </si>
+  <si>
+    <t>10,32</t>
+  </si>
+  <si>
+    <t>0,51</t>
+  </si>
+  <si>
+    <t>5,95</t>
+  </si>
+  <si>
+    <t>7,07</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,31</t>
+  </si>
+  <si>
+    <t>3,31</t>
+  </si>
+  <si>
+    <t>4,54</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>15,88</t>
   </si>
   <si>
     <t>0,85</t>
   </si>
   <si>
-    <t>4,92</t>
-  </si>
-  <si>
-    <t>12,68</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>19,17</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>47,85</t>
-  </si>
-  <si>
-    <t>4,02</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,52</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>2,79</t>
-  </si>
-  <si>
-    <t>3,56</t>
-  </si>
-  <si>
-    <t>14,93</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,59</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>0,74</t>
-  </si>
-  <si>
-    <t>27,24</t>
-  </si>
-  <si>
-    <t>30,13</t>
-  </si>
-  <si>
-    <t>6,41</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>4,65</t>
-  </si>
-  <si>
-    <t>15,86</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>16,12</t>
-  </si>
-  <si>
-    <t>2,03</t>
-  </si>
-  <si>
-    <t>0,39</t>
-  </si>
-  <si>
-    <t>48,75</t>
-  </si>
-  <si>
-    <t>8,93</t>
-  </si>
-  <si>
-    <t>10,53</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>0,71</t>
-  </si>
-  <si>
-    <t>1,03</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>3,75</t>
-  </si>
-  <si>
-    <t>7,17</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>24,18</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>7,26</t>
-  </si>
-  <si>
-    <t>33,6</t>
-  </si>
-  <si>
-    <t>12,43</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>1,82</t>
-  </si>
-  <si>
-    <t>2,08</t>
-  </si>
-  <si>
-    <t>9,03</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,79</t>
-  </si>
-  <si>
-    <t>2,17</t>
-  </si>
-  <si>
-    <t>1,12</t>
-  </si>
-  <si>
-    <t>46,77</t>
-  </si>
-  <si>
-    <t>4,39</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>12,9</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>3,16</t>
-  </si>
-  <si>
-    <t>11,53</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,89</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>37,65</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>7,83</t>
-  </si>
-  <si>
-    <t>0,6</t>
-  </si>
-  <si>
-    <t>1,15</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>6,8</t>
-  </si>
-  <si>
-    <t>10,5</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,61</t>
-  </si>
-  <si>
-    <t>1,22</t>
-  </si>
-  <si>
-    <t>43,19</t>
-  </si>
-  <si>
-    <t>16,74</t>
-  </si>
-  <si>
-    <t>6,18</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>4,4</t>
-  </si>
-  <si>
-    <t>7,09</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,68</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>29,14</t>
-  </si>
-  <si>
-    <t>17,98</t>
-  </si>
-  <si>
-    <t>6,07</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>7,41</t>
-  </si>
-  <si>
-    <t>14,27</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,73</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>30,78</t>
-  </si>
-  <si>
-    <t>1,79</t>
-  </si>
-  <si>
-    <t>5,89</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>8,34</t>
-  </si>
-  <si>
-    <t>20,57</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,71</t>
-  </si>
-  <si>
-    <t>31,92</t>
-  </si>
-  <si>
-    <t>5,31</t>
-  </si>
-  <si>
-    <t>5,22</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>0,84</t>
-  </si>
-  <si>
-    <t>8,25</t>
-  </si>
-  <si>
-    <t>28,22</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>29,39</t>
-  </si>
-  <si>
-    <t>2,34</t>
-  </si>
-  <si>
-    <t>1,24</t>
-  </si>
-  <si>
-    <t>39,46</t>
-  </si>
-  <si>
-    <t>6,68</t>
-  </si>
-  <si>
-    <t>4,33</t>
-  </si>
-  <si>
-    <t>2,68</t>
-  </si>
-  <si>
-    <t>7,53</t>
-  </si>
-  <si>
-    <t>4,79</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>18,72</t>
-  </si>
-  <si>
-    <t>1,47</t>
-  </si>
-  <si>
-    <t>1,13</t>
-  </si>
-  <si>
-    <t>33,55</t>
-  </si>
-  <si>
-    <t>15,47</t>
-  </si>
-  <si>
-    <t>6,55</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>4,08</t>
-  </si>
-  <si>
-    <t>17,85</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,17</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>49,83</t>
-  </si>
-  <si>
-    <t>13,57</t>
-  </si>
-  <si>
-    <t>10,64</t>
-  </si>
-  <si>
-    <t>0,52</t>
-  </si>
-  <si>
-    <t>6,06</t>
-  </si>
-  <si>
-    <t>7,28</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,31</t>
-  </si>
-  <si>
-    <t>3,4</t>
-  </si>
-  <si>
-    <t>31,95</t>
-  </si>
-  <si>
-    <t>4,54</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>15,88</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
     <t>1,7</t>
   </si>
   <si>
-    <t>1,89</t>
+    <t>1,98</t>
   </si>
   <si>
     <t>4,06</t>
@@ -922,31 +910,25 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>16,33</t>
-  </si>
-  <si>
-    <t>5,83</t>
-  </si>
-  <si>
-    <t>30,52</t>
-  </si>
-  <si>
-    <t>3,97</t>
-  </si>
-  <si>
-    <t>0,31</t>
+    <t>16,3</t>
+  </si>
+  <si>
+    <t>5,82</t>
+  </si>
+  <si>
+    <t>30,51</t>
+  </si>
+  <si>
+    <t>3,96</t>
   </si>
   <si>
     <t>3,07</t>
   </si>
   <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>1,01</t>
-  </si>
-  <si>
-    <t>3,73</t>
+    <t>1,09</t>
+  </si>
+  <si>
+    <t>33,54</t>
   </si>
   <si>
     <t/>
@@ -1926,16 +1908,16 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>124095</v>
+        <v>125051</v>
       </c>
       <c r="D6" s="6">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>25314</v>
+        <v>25491</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
@@ -1947,31 +1929,31 @@
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2297</v>
+        <v>2261</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>48240</v>
+        <v>48847</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12368</v>
+        <v>12485</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>9481</v>
+        <v>9515</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -2043,31 +2025,31 @@
         <v>120</v>
       </c>
       <c r="AP6" s="6">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AR6" s="6">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AT6" s="6">
-        <v>1049</v>
+        <v>1052</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AV6" s="6">
-        <v>6102</v>
+        <v>6129</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AX6" s="6">
-        <v>15733</v>
+        <v>15754</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>125</v>
@@ -2147,7 +2129,7 @@
         <v>15</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="Z7" s="9">
         <v>2</v>
@@ -2183,7 +2165,7 @@
         <v>10</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
@@ -2195,48 +2177,48 @@
         <v>3</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AP7" s="9">
         <v>27</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AR7" s="9">
         <v>3</v>
       </c>
       <c r="AS7" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AT7" s="9">
         <v>217</v>
       </c>
       <c r="AU7" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="AV7" s="9">
         <v>277</v>
       </c>
       <c r="AW7" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AX7" s="9">
         <v>1162</v>
       </c>
       <c r="AY7" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C8" s="9">
-        <v>3399</v>
+        <v>3403</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2245,34 +2227,34 @@
         <v>117</v>
       </c>
       <c r="F8" s="9">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H8" s="9">
         <v>17</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J8" s="9">
         <v>25</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L8" s="9">
         <v>926</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="N8" s="9">
         <v>1024</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P8" s="9">
         <v>0</v>
@@ -2284,7 +2266,7 @@
         <v>218</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
@@ -2302,7 +2284,7 @@
         <v>6</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>151</v>
+        <v>112</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
@@ -2391,7 +2373,7 @@
         <v>157</v>
       </c>
       <c r="C9" s="9">
-        <v>9703</v>
+        <v>9790</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
@@ -2400,7 +2382,7 @@
         <v>117</v>
       </c>
       <c r="F9" s="9">
-        <v>1564</v>
+        <v>1577</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>158</v>
@@ -2412,31 +2394,31 @@
         <v>159</v>
       </c>
       <c r="J9" s="9">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>160</v>
       </c>
       <c r="L9" s="9">
-        <v>4730</v>
+        <v>4810</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>161</v>
       </c>
       <c r="N9" s="9">
-        <v>866</v>
+        <v>869</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>162</v>
       </c>
       <c r="P9" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="R9" s="9">
-        <v>1022</v>
+        <v>1030</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>163</v>
@@ -2526,13 +2508,13 @@
         <v>167</v>
       </c>
       <c r="AV9" s="9">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AW9" s="10" t="s">
         <v>168</v>
       </c>
       <c r="AX9" s="9">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="AY9" s="10" t="s">
         <v>169</v>
@@ -2546,16 +2528,16 @@
         <v>171</v>
       </c>
       <c r="C10" s="9">
-        <v>21204</v>
+        <v>21306</v>
       </c>
       <c r="D10" s="9">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="F10" s="9">
-        <v>5128</v>
+        <v>5173</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>172</v>
@@ -2567,19 +2549,19 @@
         <v>173</v>
       </c>
       <c r="J10" s="9">
-        <v>1539</v>
+        <v>1544</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>174</v>
       </c>
       <c r="L10" s="9">
-        <v>7125</v>
+        <v>7168</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>175</v>
       </c>
       <c r="N10" s="9">
-        <v>2636</v>
+        <v>2635</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>176</v>
@@ -2591,10 +2573,10 @@
         <v>177</v>
       </c>
       <c r="R10" s="9">
-        <v>1520</v>
+        <v>1523</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
@@ -2642,7 +2624,7 @@
         <v>8</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AJ10" s="9">
         <v>13</v>
@@ -2660,13 +2642,13 @@
         <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>178</v>
+        <v>118</v>
       </c>
       <c r="AP10" s="9">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
@@ -2675,7 +2657,7 @@
         <v>167</v>
       </c>
       <c r="AT10" s="9">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="AU10" s="10" t="s">
         <v>179</v>
@@ -2701,7 +2683,7 @@
         <v>183</v>
       </c>
       <c r="C11" s="9">
-        <v>13578</v>
+        <v>13691</v>
       </c>
       <c r="D11" s="9">
         <v>12</v>
@@ -2710,7 +2692,7 @@
         <v>122</v>
       </c>
       <c r="F11" s="9">
-        <v>2144</v>
+        <v>2163</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>184</v>
@@ -2722,13 +2704,13 @@
         <v>185</v>
       </c>
       <c r="J11" s="9">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
       <c r="L11" s="9">
-        <v>6350</v>
+        <v>6417</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>187</v>
@@ -2743,25 +2725,25 @@
         <v>30</v>
       </c>
       <c r="Q11" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="R11" s="9">
+        <v>1763</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="R11" s="9">
-        <v>1752</v>
-      </c>
-      <c r="S11" s="10" t="s">
-        <v>190</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="X11" s="9">
         <v>11</v>
@@ -2773,7 +2755,7 @@
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
@@ -2797,13 +2779,13 @@
         <v>5</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AJ11" s="9">
         <v>29</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2821,39 +2803,39 @@
         <v>86</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AT11" s="9">
         <v>43</v>
       </c>
       <c r="AU11" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="AV11" s="9">
+        <v>430</v>
+      </c>
+      <c r="AW11" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="AV11" s="9">
-        <v>429</v>
-      </c>
-      <c r="AW11" s="10" t="s">
+      <c r="AX11" s="9">
+        <v>1577</v>
+      </c>
+      <c r="AY11" s="10" t="s">
         <v>195</v>
-      </c>
-      <c r="AX11" s="9">
-        <v>1566</v>
-      </c>
-      <c r="AY11" s="10" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>197</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>198</v>
       </c>
       <c r="C12" s="9">
         <v>5209</v>
@@ -2868,31 +2850,31 @@
         <v>984</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>200</v>
+        <v>148</v>
       </c>
       <c r="J12" s="9">
         <v>52</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L12" s="9">
         <v>1961</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="P12" s="9">
         <v>0</v>
@@ -2904,7 +2886,7 @@
         <v>408</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
@@ -2922,13 +2904,13 @@
         <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
@@ -2940,7 +2922,7 @@
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
@@ -2958,7 +2940,7 @@
         <v>31</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
@@ -2976,7 +2958,7 @@
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -2988,66 +2970,66 @@
         <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="AV12" s="9">
         <v>354</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C13" s="9">
-        <v>4934</v>
+        <v>4955</v>
       </c>
       <c r="D13" s="9">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>114</v>
+        <v>205</v>
       </c>
       <c r="F13" s="9">
         <v>869</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J13" s="9">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L13" s="9">
         <v>2131</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="N13" s="9">
         <v>826</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="P13" s="9">
         <v>5</v>
@@ -3059,7 +3041,7 @@
         <v>305</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
@@ -3107,19 +3089,19 @@
         <v>2</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AJ13" s="9">
         <v>32</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="AN13" s="9">
         <v>5</v>
@@ -3131,42 +3113,42 @@
         <v>37</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>153</v>
+        <v>217</v>
       </c>
       <c r="AT13" s="9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AV13" s="9">
         <v>217</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AX13" s="9">
         <v>350</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>223</v>
-      </c>
       <c r="C14" s="9">
-        <v>4956</v>
+        <v>4958</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
@@ -3178,31 +3160,31 @@
         <v>1124</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="J14" s="9">
+        <v>16</v>
+      </c>
+      <c r="K14" s="10" t="s">
         <v>225</v>
-      </c>
-      <c r="J14" s="9">
-        <v>15</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>226</v>
       </c>
       <c r="L14" s="9">
         <v>1444</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="N14" s="9">
         <v>891</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
@@ -3214,7 +3196,7 @@
         <v>301</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
@@ -3232,7 +3214,7 @@
         <v>9</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>151</v>
+        <v>112</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3268,7 +3250,7 @@
         <v>16</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>194</v>
+        <v>225</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3286,7 +3268,7 @@
         <v>34</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3298,66 +3280,66 @@
         <v>17</v>
       </c>
       <c r="AU14" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="AV14" s="9">
+        <v>368</v>
+      </c>
+      <c r="AW14" s="10" t="s">
         <v>231</v>
-      </c>
-      <c r="AV14" s="9">
-        <v>367</v>
-      </c>
-      <c r="AW14" s="10" t="s">
-        <v>232</v>
       </c>
       <c r="AX14" s="9">
         <v>707</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="9">
+        <v>12656</v>
+      </c>
+      <c r="D15" s="9">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="9">
+        <v>3886</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>235</v>
-      </c>
-      <c r="C15" s="9">
-        <v>12641</v>
-      </c>
-      <c r="D15" s="9">
-        <v>0</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F15" s="9">
-        <v>3885</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>236</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J15" s="9">
         <v>5</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L15" s="9">
-        <v>3891</v>
+        <v>3898</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="P15" s="9">
         <v>1</v>
@@ -3366,16 +3348,16 @@
         <v>136</v>
       </c>
       <c r="R15" s="9">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>194</v>
+        <v>225</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
@@ -3387,7 +3369,7 @@
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
@@ -3441,7 +3423,7 @@
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
@@ -3456,63 +3438,63 @@
         <v>120</v>
       </c>
       <c r="AV15" s="9">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AX15" s="9">
         <v>2600</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>245</v>
-      </c>
       <c r="C16" s="9">
-        <v>5100</v>
+        <v>5102</v>
       </c>
       <c r="D16" s="9">
         <v>2</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F16" s="9">
         <v>903</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J16" s="9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="L16" s="9">
-        <v>1628</v>
+        <v>1630</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N16" s="9">
         <v>271</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P16" s="9">
         <v>1</v>
@@ -3524,7 +3506,7 @@
         <v>266</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
@@ -3542,7 +3524,7 @@
         <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
@@ -3578,7 +3560,7 @@
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3596,7 +3578,7 @@
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>251</v>
+        <v>123</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
@@ -3605,81 +3587,81 @@
         <v>134</v>
       </c>
       <c r="AT16" s="9">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>217</v>
+        <v>250</v>
       </c>
       <c r="AV16" s="9">
         <v>421</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AX16" s="9">
         <v>1439</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>255</v>
-      </c>
       <c r="C17" s="9">
-        <v>10045</v>
+        <v>10158</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>194</v>
+        <v>225</v>
       </c>
       <c r="F17" s="9">
-        <v>2952</v>
+        <v>2972</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H17" s="9">
         <v>235</v>
       </c>
       <c r="I17" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="J17" s="9">
+        <v>128</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="J17" s="9">
-        <v>125</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>4040</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="L17" s="9">
-        <v>3964</v>
-      </c>
-      <c r="M17" s="10" t="s">
+      <c r="N17" s="9">
+        <v>670</v>
+      </c>
+      <c r="O17" s="10" t="s">
         <v>259</v>
-      </c>
-      <c r="N17" s="9">
-        <v>671</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>260</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R17" s="9">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -3691,7 +3673,7 @@
         <v>4</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="X17" s="9">
         <v>8</v>
@@ -3703,7 +3685,7 @@
         <v>4</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
@@ -3715,7 +3697,7 @@
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
@@ -3751,42 +3733,42 @@
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AR17" s="9">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>122</v>
+        <v>192</v>
       </c>
       <c r="AT17" s="9">
         <v>269</v>
       </c>
       <c r="AU17" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="AV17" s="9">
+        <v>762</v>
+      </c>
+      <c r="AW17" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="AV17" s="9">
-        <v>756</v>
-      </c>
-      <c r="AW17" s="10" t="s">
+      <c r="AX17" s="9">
+        <v>484</v>
+      </c>
+      <c r="AY17" s="10" t="s">
         <v>263</v>
-      </c>
-      <c r="AX17" s="9">
-        <v>481</v>
-      </c>
-      <c r="AY17" s="10" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>266</v>
-      </c>
       <c r="C18" s="9">
-        <v>10293</v>
+        <v>10367</v>
       </c>
       <c r="D18" s="9">
         <v>2</v>
@@ -3795,34 +3777,34 @@
         <v>114</v>
       </c>
       <c r="F18" s="9">
-        <v>1927</v>
+        <v>1954</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H18" s="9">
         <v>151</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J18" s="9">
         <v>116</v>
       </c>
       <c r="K18" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="L18" s="9">
+        <v>3490</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="L18" s="9">
-        <v>3453</v>
-      </c>
-      <c r="M18" s="10" t="s">
+      <c r="N18" s="9">
+        <v>1602</v>
+      </c>
+      <c r="O18" s="10" t="s">
         <v>270</v>
-      </c>
-      <c r="N18" s="9">
-        <v>1592</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>271</v>
       </c>
       <c r="P18" s="9">
         <v>1</v>
@@ -3834,13 +3816,13 @@
         <v>674</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="T18" s="9">
         <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
@@ -3888,7 +3870,7 @@
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
@@ -3906,13 +3888,13 @@
         <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>275</v>
+        <v>115</v>
       </c>
       <c r="AT18" s="9">
         <v>2</v>
@@ -3924,72 +3906,72 @@
         <v>420</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="AX18" s="9">
         <v>1837</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" s="9">
+        <v>12041</v>
+      </c>
+      <c r="D19" s="9">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F19" s="9">
+        <v>1346</v>
+      </c>
+      <c r="G19" s="10" t="s">
         <v>278</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>279</v>
-      </c>
-      <c r="C19" s="9">
-        <v>11622</v>
-      </c>
-      <c r="D19" s="9">
-        <v>2</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" s="9">
-        <v>1298</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>137</v>
+        <v>205</v>
       </c>
       <c r="J19" s="9">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="K19" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="L19" s="9">
+        <v>6085</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="N19" s="9">
+        <v>1683</v>
+      </c>
+      <c r="O19" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="P19" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="R19" s="9">
+        <v>1243</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>281</v>
-      </c>
-      <c r="L19" s="9">
-        <v>5791</v>
-      </c>
-      <c r="M19" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="N19" s="9">
-        <v>1577</v>
-      </c>
-      <c r="O19" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="P19" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="R19" s="9">
-        <v>1237</v>
-      </c>
-      <c r="S19" s="10" t="s">
-        <v>284</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
@@ -4025,7 +4007,7 @@
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
@@ -4043,7 +4025,7 @@
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
@@ -4061,7 +4043,7 @@
         <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
@@ -4070,30 +4052,30 @@
         <v>136</v>
       </c>
       <c r="AT19" s="9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>167</v>
+        <v>136</v>
       </c>
       <c r="AV19" s="9">
-        <v>704</v>
+        <v>717</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="AX19" s="9">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C20" s="9">
         <v>1058</v>
@@ -4108,43 +4090,43 @@
         <v>162</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J20" s="9">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="L20" s="9">
         <v>338</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>292</v>
+        <v>246</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="P20" s="9">
         <v>7</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
@@ -4162,13 +4144,13 @@
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>123</v>
+        <v>292</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>296</v>
+        <v>218</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
@@ -4198,13 +4180,13 @@
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
@@ -4216,7 +4198,7 @@
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
@@ -4225,33 +4207,33 @@
         <v>164</v>
       </c>
       <c r="AT20" s="9">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="AV20" s="9">
         <v>43</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C21" s="9">
-        <v>2572</v>
+        <v>2576</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -4263,13 +4245,13 @@
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="J21" s="9">
         <v>2</v>
@@ -4278,28 +4260,28 @@
         <v>106</v>
       </c>
       <c r="L21" s="9">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>307</v>
+        <v>193</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
@@ -4317,7 +4299,7 @@
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4353,7 +4335,7 @@
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
@@ -4371,51 +4353,51 @@
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>309</v>
+        <v>165</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AT21" s="9">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>311</v>
+        <v>168</v>
       </c>
       <c r="AX21" s="9">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>270</v>
+        <v>305</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="C22" s="12">
-        <v>124095</v>
+        <v>125051</v>
       </c>
       <c r="D22" s="12">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>25314</v>
+        <v>25491</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
@@ -4427,31 +4409,31 @@
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2297</v>
+        <v>2261</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>48240</v>
+        <v>48847</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12368</v>
+        <v>12485</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>9481</v>
+        <v>9515</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4523,31 +4505,31 @@
         <v>120</v>
       </c>
       <c r="AP22" s="12">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AR22" s="12">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AT22" s="12">
-        <v>1049</v>
+        <v>1052</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AV22" s="12">
-        <v>6102</v>
+        <v>6129</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AX22" s="12">
-        <v>15733</v>
+        <v>15754</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>125</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 08/09/2026  7:19:43,20
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="309">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 7 Sep 2026, 15.57</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 8 Sep 2026, 07.18</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,25 +334,25 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>20,38</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>1,81</t>
-  </si>
-  <si>
-    <t>39,06</t>
-  </si>
-  <si>
-    <t>9,98</t>
+    <t>20,35</t>
+  </si>
+  <si>
+    <t>1,16</t>
+  </si>
+  <si>
+    <t>1,77</t>
+  </si>
+  <si>
+    <t>39,7</t>
+  </si>
+  <si>
+    <t>9,81</t>
   </si>
   <si>
     <t>0,18</t>
   </si>
   <si>
-    <t>7,61</t>
+    <t>7,52</t>
   </si>
   <si>
     <t>0,02</t>
@@ -367,6 +367,9 @@
     <t>0</t>
   </si>
   <si>
+    <t>0,01</t>
+  </si>
+  <si>
     <t>0,24</t>
   </si>
   <si>
@@ -382,427 +385,433 @@
     <t>0,09</t>
   </si>
   <si>
+    <t>0,83</t>
+  </si>
+  <si>
+    <t>4,86</t>
+  </si>
+  <si>
+    <t>12,38</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>19,22</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>0,92</t>
+  </si>
+  <si>
+    <t>47,76</t>
+  </si>
+  <si>
+    <t>4,19</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,51</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>2,77</t>
+  </si>
+  <si>
+    <t>3,55</t>
+  </si>
+  <si>
+    <t>14,92</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,77</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>27,16</t>
+  </si>
+  <si>
+    <t>30,06</t>
+  </si>
+  <si>
+    <t>6,4</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>4,64</t>
+  </si>
+  <si>
+    <t>15,83</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>16,05</t>
+  </si>
+  <si>
+    <t>1,97</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>49,7</t>
+  </si>
+  <si>
+    <t>8,65</t>
+  </si>
+  <si>
+    <t>10,4</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>3,72</t>
+  </si>
+  <si>
+    <t>7,03</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>24,4</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>7,23</t>
+  </si>
+  <si>
+    <t>33,71</t>
+  </si>
+  <si>
+    <t>12,3</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>7,1</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>2,09</t>
+  </si>
+  <si>
+    <t>8,93</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,01</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1,01</t>
+  </si>
+  <si>
+    <t>48,48</t>
+  </si>
+  <si>
+    <t>4,17</t>
+  </si>
+  <si>
+    <t>12,23</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>3,02</t>
+  </si>
+  <si>
+    <t>10,88</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,95</t>
+  </si>
+  <si>
+    <t>0,72</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>37,99</t>
+  </si>
+  <si>
+    <t>13,87</t>
+  </si>
+  <si>
+    <t>7,76</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>6,73</t>
+  </si>
+  <si>
+    <t>10,41</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,56</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>1,49</t>
+  </si>
+  <si>
+    <t>43,05</t>
+  </si>
+  <si>
+    <t>16,62</t>
+  </si>
+  <si>
+    <t>6,16</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>4,37</t>
+  </si>
+  <si>
+    <t>7,04</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,65</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>29,08</t>
+  </si>
+  <si>
+    <t>18,01</t>
+  </si>
+  <si>
+    <t>6,07</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>7,42</t>
+  </si>
+  <si>
+    <t>14,26</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,66</t>
+  </si>
+  <si>
+    <t>0,43</t>
+  </si>
+  <si>
+    <t>30,83</t>
+  </si>
+  <si>
+    <t>1,78</t>
+  </si>
+  <si>
+    <t>5,89</t>
+  </si>
+  <si>
+    <t>8,36</t>
+  </si>
+  <si>
+    <t>20,52</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,74</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>32,05</t>
+  </si>
+  <si>
+    <t>5,32</t>
+  </si>
+  <si>
+    <t>5,22</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
     <t>0,84</t>
   </si>
   <si>
-    <t>4,9</t>
-  </si>
-  <si>
-    <t>12,6</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>19,17</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>47,85</t>
-  </si>
-  <si>
-    <t>4,02</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,52</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>2,79</t>
-  </si>
-  <si>
-    <t>3,56</t>
-  </si>
-  <si>
-    <t>14,93</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,69</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>27,21</t>
-  </si>
-  <si>
-    <t>30,09</t>
-  </si>
-  <si>
-    <t>6,41</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>4,64</t>
-  </si>
-  <si>
-    <t>15,84</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>16,11</t>
-  </si>
-  <si>
-    <t>2,01</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>49,13</t>
-  </si>
-  <si>
-    <t>8,88</t>
-  </si>
-  <si>
-    <t>10,52</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>1,02</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>3,73</t>
-  </si>
-  <si>
-    <t>7,12</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>24,28</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>7,25</t>
-  </si>
-  <si>
-    <t>33,64</t>
-  </si>
-  <si>
-    <t>12,37</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>7,15</t>
-  </si>
-  <si>
-    <t>1,82</t>
-  </si>
-  <si>
-    <t>2,07</t>
-  </si>
-  <si>
-    <t>8,99</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>15,8</t>
-  </si>
-  <si>
-    <t>2,15</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>46,87</t>
-  </si>
-  <si>
-    <t>4,35</t>
-  </si>
-  <si>
-    <t>12,88</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>0,11</t>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>8,23</t>
+  </si>
+  <si>
+    <t>28,37</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
   </si>
   <si>
     <t>0,31</t>
   </si>
   <si>
-    <t>3,14</t>
-  </si>
-  <si>
-    <t>11,52</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,89</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>37,65</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>7,83</t>
-  </si>
-  <si>
-    <t>0,6</t>
-  </si>
-  <si>
-    <t>1,15</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>6,8</t>
-  </si>
-  <si>
-    <t>10,5</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,54</t>
-  </si>
-  <si>
-    <t>1,51</t>
-  </si>
-  <si>
-    <t>43,01</t>
-  </si>
-  <si>
-    <t>16,67</t>
-  </si>
-  <si>
-    <t>6,16</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>4,38</t>
-  </si>
-  <si>
-    <t>7,06</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,67</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>29,12</t>
-  </si>
-  <si>
-    <t>17,97</t>
-  </si>
-  <si>
-    <t>6,07</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>7,42</t>
-  </si>
-  <si>
-    <t>14,26</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,7</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>30,8</t>
-  </si>
-  <si>
-    <t>1,79</t>
-  </si>
-  <si>
-    <t>5,89</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>8,37</t>
-  </si>
-  <si>
-    <t>20,54</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,7</t>
-  </si>
-  <si>
-    <t>31,95</t>
-  </si>
-  <si>
-    <t>5,31</t>
-  </si>
-  <si>
-    <t>5,21</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>0,67</t>
-  </si>
-  <si>
-    <t>8,25</t>
-  </si>
-  <si>
-    <t>28,2</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>29,26</t>
-  </si>
-  <si>
-    <t>2,31</t>
-  </si>
-  <si>
-    <t>1,26</t>
-  </si>
-  <si>
-    <t>39,77</t>
+    <t>2,28</t>
+  </si>
+  <si>
+    <t>1,25</t>
+  </si>
+  <si>
+    <t>40,01</t>
   </si>
   <si>
     <t>6,6</t>
   </si>
   <si>
-    <t>4,32</t>
-  </si>
-  <si>
-    <t>2,65</t>
-  </si>
-  <si>
-    <t>7,5</t>
-  </si>
-  <si>
-    <t>4,76</t>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>2,69</t>
+  </si>
+  <si>
+    <t>7,41</t>
+  </si>
+  <si>
+    <t>4,74</t>
   </si>
   <si>
     <t>1812</t>
@@ -811,34 +820,28 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>18,85</t>
-  </si>
-  <si>
-    <t>1,46</t>
-  </si>
-  <si>
-    <t>1,12</t>
-  </si>
-  <si>
-    <t>33,66</t>
-  </si>
-  <si>
-    <t>15,45</t>
-  </si>
-  <si>
-    <t>6,5</t>
+    <t>19,01</t>
+  </si>
+  <si>
+    <t>1,44</t>
+  </si>
+  <si>
+    <t>1,1</t>
+  </si>
+  <si>
+    <t>15,39</t>
+  </si>
+  <si>
+    <t>6,48</t>
   </si>
   <si>
     <t>0,29</t>
   </si>
   <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>4,05</t>
-  </si>
-  <si>
-    <t>17,72</t>
+    <t>4,12</t>
+  </si>
+  <si>
+    <t>17,59</t>
   </si>
   <si>
     <t>1813</t>
@@ -847,25 +850,22 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>11,18</t>
-  </si>
-  <si>
-    <t>50,54</t>
-  </si>
-  <si>
-    <t>13,98</t>
-  </si>
-  <si>
-    <t>10,32</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>5,95</t>
-  </si>
-  <si>
-    <t>7,07</t>
+    <t>11,35</t>
+  </si>
+  <si>
+    <t>52,54</t>
+  </si>
+  <si>
+    <t>12,91</t>
+  </si>
+  <si>
+    <t>9,9</t>
+  </si>
+  <si>
+    <t>5,78</t>
+  </si>
+  <si>
+    <t>6,58</t>
   </si>
   <si>
     <t>1871</t>
@@ -874,34 +874,40 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>15,31</t>
-  </si>
-  <si>
-    <t>3,31</t>
-  </si>
-  <si>
-    <t>4,54</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>15,88</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>1,98</t>
-  </si>
-  <si>
-    <t>4,06</t>
-  </si>
-  <si>
-    <t>17,49</t>
+    <t>15,09</t>
+  </si>
+  <si>
+    <t>3,18</t>
+  </si>
+  <si>
+    <t>33,82</t>
+  </si>
+  <si>
+    <t>4,36</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>15,27</t>
+  </si>
+  <si>
+    <t>0,82</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>1,64</t>
+  </si>
+  <si>
+    <t>2,27</t>
+  </si>
+  <si>
+    <t>3,91</t>
+  </si>
+  <si>
+    <t>16,82</t>
   </si>
   <si>
     <t>1872</t>
@@ -910,25 +916,22 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>16,3</t>
-  </si>
-  <si>
-    <t>5,82</t>
-  </si>
-  <si>
-    <t>30,51</t>
-  </si>
-  <si>
-    <t>3,96</t>
-  </si>
-  <si>
-    <t>3,07</t>
-  </si>
-  <si>
-    <t>1,09</t>
-  </si>
-  <si>
-    <t>33,54</t>
+    <t>16,27</t>
+  </si>
+  <si>
+    <t>5,81</t>
+  </si>
+  <si>
+    <t>30,57</t>
+  </si>
+  <si>
+    <t>3,95</t>
+  </si>
+  <si>
+    <t>3,06</t>
+  </si>
+  <si>
+    <t>33,48</t>
   </si>
   <si>
     <t/>
@@ -1908,7 +1911,7 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>125051</v>
+        <v>127542</v>
       </c>
       <c r="D6" s="6">
         <v>103</v>
@@ -1917,43 +1920,43 @@
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>25491</v>
+        <v>25954</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1482</v>
+        <v>1480</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2261</v>
+        <v>2259</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>48847</v>
+        <v>50630</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12485</v>
+        <v>12513</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>9515</v>
+        <v>9596</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1971,7 +1974,7 @@
         <v>114</v>
       </c>
       <c r="X6" s="6">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>115</v>
@@ -1983,7 +1986,7 @@
         <v>114</v>
       </c>
       <c r="AB6" s="6">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AC6" s="7" t="s">
         <v>114</v>
@@ -1995,7 +1998,7 @@
         <v>116</v>
       </c>
       <c r="AF6" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG6" s="7" t="s">
         <v>117</v>
@@ -2004,126 +2007,126 @@
         <v>19</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AJ6" s="6">
-        <v>297</v>
+        <v>308</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AL6" s="6">
         <v>39</v>
       </c>
       <c r="AM6" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AO6" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AP6" s="6">
-        <v>692</v>
+        <v>703</v>
       </c>
       <c r="AQ6" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AR6" s="6">
         <v>117</v>
       </c>
       <c r="AS6" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AT6" s="6">
-        <v>1052</v>
+        <v>1064</v>
       </c>
       <c r="AU6" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AV6" s="6">
-        <v>6129</v>
+        <v>6195</v>
       </c>
       <c r="AW6" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>15754</v>
+        <v>15789</v>
       </c>
       <c r="AY6" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>7781</v>
+        <v>7801</v>
       </c>
       <c r="D7" s="9">
         <v>8</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F7" s="9">
-        <v>1492</v>
+        <v>1499</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H7" s="9">
         <v>74</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J7" s="9">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L7" s="9">
-        <v>3723</v>
+        <v>3726</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N7" s="9">
-        <v>313</v>
+        <v>327</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P7" s="9">
         <v>11</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="R7" s="9">
         <v>352</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="T7" s="9">
         <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="V7" s="9">
         <v>1</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="X7" s="9">
         <v>15</v>
@@ -2135,7 +2138,7 @@
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AB7" s="9">
         <v>6</v>
@@ -2147,7 +2150,7 @@
         <v>5</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
@@ -2171,7 +2174,7 @@
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AN7" s="9">
         <v>3</v>
@@ -2192,7 +2195,7 @@
         <v>139</v>
       </c>
       <c r="AT7" s="9">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>141</v>
@@ -2204,7 +2207,7 @@
         <v>142</v>
       </c>
       <c r="AX7" s="9">
-        <v>1162</v>
+        <v>1164</v>
       </c>
       <c r="AY7" s="10" t="s">
         <v>143</v>
@@ -2218,7 +2221,7 @@
         <v>145</v>
       </c>
       <c r="C8" s="9">
-        <v>3403</v>
+        <v>3406</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2227,7 +2230,7 @@
         <v>117</v>
       </c>
       <c r="F8" s="9">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>146</v>
@@ -2245,7 +2248,7 @@
         <v>148</v>
       </c>
       <c r="L8" s="9">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>149</v>
@@ -2302,7 +2305,7 @@
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
@@ -2344,13 +2347,13 @@
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT8" s="9">
+        <v>1</v>
+      </c>
+      <c r="AU8" s="10" t="s">
         <v>120</v>
-      </c>
-      <c r="AT8" s="9">
-        <v>0</v>
-      </c>
-      <c r="AU8" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="AV8" s="9">
         <v>158</v>
@@ -2373,7 +2376,7 @@
         <v>157</v>
       </c>
       <c r="C9" s="9">
-        <v>9790</v>
+        <v>10002</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
@@ -2382,7 +2385,7 @@
         <v>117</v>
       </c>
       <c r="F9" s="9">
-        <v>1577</v>
+        <v>1605</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>158</v>
@@ -2394,31 +2397,31 @@
         <v>159</v>
       </c>
       <c r="J9" s="9">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>160</v>
       </c>
       <c r="L9" s="9">
-        <v>4810</v>
+        <v>4971</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>161</v>
       </c>
       <c r="N9" s="9">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>162</v>
       </c>
       <c r="P9" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R9" s="9">
-        <v>1030</v>
+        <v>1040</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>163</v>
@@ -2427,7 +2430,7 @@
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
@@ -2457,7 +2460,7 @@
         <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
@@ -2472,7 +2475,7 @@
         <v>117</v>
       </c>
       <c r="AJ9" s="9">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AK9" s="10" t="s">
         <v>165</v>
@@ -2502,93 +2505,93 @@
         <v>114</v>
       </c>
       <c r="AT9" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AU9" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="AV9" s="9">
+        <v>372</v>
+      </c>
+      <c r="AW9" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="AV9" s="9">
-        <v>365</v>
-      </c>
-      <c r="AW9" s="10" t="s">
+      <c r="AX9" s="9">
+        <v>703</v>
+      </c>
+      <c r="AY9" s="10" t="s">
         <v>168</v>
-      </c>
-      <c r="AX9" s="9">
-        <v>697</v>
-      </c>
-      <c r="AY9" s="10" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>171</v>
-      </c>
       <c r="C10" s="9">
-        <v>21306</v>
+        <v>21433</v>
       </c>
       <c r="D10" s="9">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>137</v>
       </c>
       <c r="F10" s="9">
-        <v>5173</v>
+        <v>5229</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H10" s="9">
         <v>169</v>
       </c>
       <c r="I10" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="J10" s="9">
+        <v>1550</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="J10" s="9">
-        <v>1544</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="L10" s="9">
+        <v>7224</v>
+      </c>
+      <c r="M10" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="L10" s="9">
-        <v>7168</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="N10" s="9">
+        <v>2637</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="N10" s="9">
-        <v>2635</v>
-      </c>
-      <c r="O10" s="10" t="s">
+      <c r="P10" s="9">
+        <v>143</v>
+      </c>
+      <c r="Q10" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="P10" s="9">
-        <v>144</v>
-      </c>
-      <c r="Q10" s="10" t="s">
+      <c r="R10" s="9">
+        <v>1522</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>177</v>
-      </c>
-      <c r="R10" s="9">
-        <v>1523</v>
-      </c>
-      <c r="S10" s="10" t="s">
-        <v>178</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="V10" s="9">
         <v>7</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="X10" s="9">
         <v>14</v>
@@ -2600,13 +2603,13 @@
         <v>2</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AB10" s="9">
         <v>10</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="AD10" s="9">
         <v>15</v>
@@ -2630,7 +2633,7 @@
         <v>13</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
@@ -2642,28 +2645,28 @@
         <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP10" s="9">
         <v>31</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="AT10" s="9">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="AU10" s="10" t="s">
         <v>179</v>
       </c>
       <c r="AV10" s="9">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="AW10" s="10" t="s">
         <v>180</v>
@@ -2683,52 +2686,52 @@
         <v>183</v>
       </c>
       <c r="C11" s="9">
-        <v>13691</v>
+        <v>14564</v>
       </c>
       <c r="D11" s="9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F11" s="9">
-        <v>2163</v>
+        <v>2331</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>184</v>
       </c>
       <c r="H11" s="9">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="I11" s="10" t="s">
         <v>185</v>
       </c>
       <c r="J11" s="9">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
       <c r="L11" s="9">
-        <v>6417</v>
+        <v>7060</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>187</v>
       </c>
       <c r="N11" s="9">
-        <v>596</v>
+        <v>607</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>188</v>
       </c>
       <c r="P11" s="9">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>160</v>
+        <v>119</v>
       </c>
       <c r="R11" s="9">
-        <v>1763</v>
+        <v>1781</v>
       </c>
       <c r="S11" s="10" t="s">
         <v>189</v>
@@ -2737,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>138</v>
+        <v>190</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="X11" s="9">
         <v>11</v>
@@ -2755,7 +2758,7 @@
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="AB11" s="9">
         <v>3</v>
@@ -2767,7 +2770,7 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
@@ -2779,13 +2782,13 @@
         <v>5</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="AJ11" s="9">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2794,37 +2797,37 @@
         <v>114</v>
       </c>
       <c r="AN11" s="9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="AP11" s="9">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>192</v>
+        <v>129</v>
       </c>
       <c r="AT11" s="9">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="AU11" s="10" t="s">
         <v>193</v>
       </c>
       <c r="AV11" s="9">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="AW11" s="10" t="s">
         <v>194</v>
       </c>
       <c r="AX11" s="9">
-        <v>1577</v>
+        <v>1585</v>
       </c>
       <c r="AY11" s="10" t="s">
         <v>195</v>
@@ -2838,7 +2841,7 @@
         <v>197</v>
       </c>
       <c r="C12" s="9">
-        <v>5209</v>
+        <v>5257</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
@@ -2847,7 +2850,7 @@
         <v>117</v>
       </c>
       <c r="F12" s="9">
-        <v>984</v>
+        <v>996</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>198</v>
@@ -2856,25 +2859,25 @@
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>148</v>
+        <v>199</v>
       </c>
       <c r="J12" s="9">
         <v>52</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L12" s="9">
-        <v>1961</v>
+        <v>1997</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P12" s="9">
         <v>0</v>
@@ -2886,7 +2889,7 @@
         <v>408</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
@@ -2904,7 +2907,7 @@
         <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>147</v>
+        <v>204</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
@@ -2940,7 +2943,7 @@
         <v>31</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
@@ -2958,7 +2961,7 @@
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -2970,78 +2973,78 @@
         <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="AV12" s="9">
         <v>354</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C13" s="9">
-        <v>4955</v>
+        <v>4971</v>
       </c>
       <c r="D13" s="9">
         <v>6</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="F13" s="9">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="J13" s="9">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="L13" s="9">
-        <v>2131</v>
+        <v>2140</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="N13" s="9">
         <v>826</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="P13" s="9">
         <v>5</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R13" s="9">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
@@ -3053,7 +3056,7 @@
         <v>3</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
@@ -3092,63 +3095,63 @@
         <v>139</v>
       </c>
       <c r="AJ13" s="9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>215</v>
+        <v>192</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>160</v>
+        <v>218</v>
       </c>
       <c r="AN13" s="9">
         <v>5</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AP13" s="9">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="AT13" s="9">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AV13" s="9">
         <v>217</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AX13" s="9">
         <v>350</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C14" s="9">
-        <v>4958</v>
+        <v>4959</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
@@ -3157,34 +3160,34 @@
         <v>117</v>
       </c>
       <c r="F14" s="9">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="J14" s="9">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L14" s="9">
-        <v>1444</v>
+        <v>1442</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="N14" s="9">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
@@ -3196,13 +3199,13 @@
         <v>301</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
@@ -3232,7 +3235,7 @@
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
@@ -3250,7 +3253,7 @@
         <v>16</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>225</v>
+        <v>193</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3268,7 +3271,7 @@
         <v>34</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3280,30 +3283,30 @@
         <v>17</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="AV14" s="9">
         <v>368</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="AX14" s="9">
         <v>707</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C15" s="9">
-        <v>12656</v>
+        <v>12679</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -3312,52 +3315,52 @@
         <v>117</v>
       </c>
       <c r="F15" s="9">
-        <v>3886</v>
+        <v>3888</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="J15" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>139</v>
+        <v>106</v>
       </c>
       <c r="L15" s="9">
-        <v>3898</v>
+        <v>3909</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="P15" s="9">
         <v>1</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="R15" s="9">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>225</v>
+        <v>193</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
@@ -3369,7 +3372,7 @@
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
@@ -3399,13 +3402,13 @@
         <v>1</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AJ15" s="9">
         <v>11</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AL15" s="9">
         <v>3</v>
@@ -3417,13 +3420,13 @@
         <v>1</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AP15" s="9">
         <v>79</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>240</v>
+        <v>213</v>
       </c>
       <c r="AR15" s="9">
         <v>19</v>
@@ -3432,69 +3435,69 @@
         <v>152</v>
       </c>
       <c r="AT15" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AV15" s="9">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AX15" s="9">
-        <v>2600</v>
+        <v>2602</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C16" s="9">
-        <v>5102</v>
+        <v>5114</v>
       </c>
       <c r="D16" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="F16" s="9">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>191</v>
+        <v>247</v>
       </c>
       <c r="J16" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="L16" s="9">
-        <v>1630</v>
+        <v>1639</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="N16" s="9">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="P16" s="9">
         <v>1</v>
@@ -3503,10 +3506,10 @@
         <v>114</v>
       </c>
       <c r="R16" s="9">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
@@ -3524,31 +3527,31 @@
         <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AB16" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AF16" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
@@ -3560,7 +3563,7 @@
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3578,96 +3581,96 @@
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>123</v>
+        <v>252</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AT16" s="9">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AV16" s="9">
         <v>421</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="AX16" s="9">
-        <v>1439</v>
+        <v>1451</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C17" s="9">
-        <v>10158</v>
+        <v>10292</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>225</v>
+        <v>258</v>
       </c>
       <c r="F17" s="9">
-        <v>2972</v>
+        <v>2993</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>255</v>
+        <v>228</v>
       </c>
       <c r="H17" s="9">
         <v>235</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="J17" s="9">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="L17" s="9">
-        <v>4040</v>
+        <v>4118</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="N17" s="9">
-        <v>670</v>
+        <v>679</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>190</v>
+        <v>263</v>
       </c>
       <c r="R17" s="9">
-        <v>439</v>
+        <v>450</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>260</v>
+        <v>222</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="V17" s="9">
         <v>4</v>
@@ -3721,108 +3724,108 @@
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AN17" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="AT17" s="9">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AV17" s="9">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AX17" s="9">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C18" s="9">
-        <v>10367</v>
+        <v>10451</v>
       </c>
       <c r="D18" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F18" s="9">
-        <v>1954</v>
+        <v>1987</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="H18" s="9">
         <v>151</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="J18" s="9">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="L18" s="9">
-        <v>3490</v>
+        <v>3523</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>269</v>
+        <v>174</v>
       </c>
       <c r="N18" s="9">
-        <v>1602</v>
+        <v>1608</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="P18" s="9">
         <v>1</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="R18" s="9">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="T18" s="9">
         <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
@@ -3834,25 +3837,25 @@
         <v>5</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AB18" s="9">
         <v>1</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AD18" s="9">
         <v>3</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
@@ -3870,13 +3873,13 @@
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AN18" s="9">
         <v>2</v>
@@ -3888,7 +3891,7 @@
         <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>273</v>
+        <v>227</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
@@ -3897,33 +3900,33 @@
         <v>115</v>
       </c>
       <c r="AT18" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AV18" s="9">
-        <v>420</v>
+        <v>431</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AX18" s="9">
-        <v>1837</v>
+        <v>1838</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C19" s="9">
-        <v>12041</v>
+        <v>12932</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
@@ -3932,34 +3935,34 @@
         <v>117</v>
       </c>
       <c r="F19" s="9">
-        <v>1346</v>
+        <v>1468</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="J19" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="L19" s="9">
-        <v>6085</v>
+        <v>6795</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="N19" s="9">
-        <v>1683</v>
+        <v>1670</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
@@ -3968,10 +3971,10 @@
         <v>117</v>
       </c>
       <c r="R19" s="9">
-        <v>1243</v>
+        <v>1280</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
@@ -3986,7 +3989,7 @@
         <v>117</v>
       </c>
       <c r="X19" s="9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Y19" s="10" t="s">
         <v>152</v>
@@ -4025,7 +4028,7 @@
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>138</v>
+        <v>190</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
@@ -4043,22 +4046,22 @@
         <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>282</v>
+        <v>153</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="AT19" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="AV19" s="9">
-        <v>717</v>
+        <v>748</v>
       </c>
       <c r="AW19" s="10" t="s">
         <v>283</v>
@@ -4078,16 +4081,16 @@
         <v>286</v>
       </c>
       <c r="C20" s="9">
-        <v>1058</v>
+        <v>1100</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F20" s="9">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G20" s="10" t="s">
         <v>287</v>
@@ -4096,7 +4099,7 @@
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>249</v>
+        <v>122</v>
       </c>
       <c r="J20" s="9">
         <v>35</v>
@@ -4105,28 +4108,28 @@
         <v>288</v>
       </c>
       <c r="L20" s="9">
-        <v>338</v>
+        <v>372</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>246</v>
+        <v>289</v>
       </c>
       <c r="N20" s="9">
         <v>48</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P20" s="9">
         <v>7</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="R20" s="9">
         <v>168</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
@@ -4144,13 +4147,13 @@
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>218</v>
+        <v>294</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
@@ -4174,66 +4177,66 @@
         <v>1</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AJ20" s="9">
         <v>6</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>249</v>
+        <v>122</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>164</v>
+        <v>227</v>
       </c>
       <c r="AT20" s="9">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="AV20" s="9">
         <v>43</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="AX20" s="9">
         <v>185</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C21" s="9">
-        <v>2576</v>
+        <v>2581</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -4245,13 +4248,13 @@
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="J21" s="9">
         <v>2</v>
@@ -4260,28 +4263,28 @@
         <v>106</v>
       </c>
       <c r="L21" s="9">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>193</v>
+        <v>258</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
@@ -4299,7 +4302,7 @@
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>290</v>
+        <v>192</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4335,7 +4338,7 @@
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
@@ -4362,33 +4365,33 @@
         <v>139</v>
       </c>
       <c r="AT21" s="9">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>304</v>
+        <v>108</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AX21" s="9">
         <v>864</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C22" s="12">
-        <v>125051</v>
+        <v>127542</v>
       </c>
       <c r="D22" s="12">
         <v>103</v>
@@ -4397,43 +4400,43 @@
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>25491</v>
+        <v>25954</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1482</v>
+        <v>1480</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2261</v>
+        <v>2259</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>48847</v>
+        <v>50630</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12485</v>
+        <v>12513</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>9515</v>
+        <v>9596</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4451,7 +4454,7 @@
         <v>114</v>
       </c>
       <c r="X22" s="12">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>115</v>
@@ -4463,7 +4466,7 @@
         <v>114</v>
       </c>
       <c r="AB22" s="12">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AC22" s="13" t="s">
         <v>114</v>
@@ -4475,7 +4478,7 @@
         <v>116</v>
       </c>
       <c r="AF22" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG22" s="13" t="s">
         <v>117</v>
@@ -4484,55 +4487,55 @@
         <v>19</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AJ22" s="12">
-        <v>297</v>
+        <v>308</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AL22" s="12">
         <v>39</v>
       </c>
       <c r="AM22" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AO22" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AP22" s="12">
-        <v>692</v>
+        <v>703</v>
       </c>
       <c r="AQ22" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AR22" s="12">
         <v>117</v>
       </c>
       <c r="AS22" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AT22" s="12">
-        <v>1052</v>
+        <v>1064</v>
       </c>
       <c r="AU22" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AV22" s="12">
-        <v>6129</v>
+        <v>6195</v>
       </c>
       <c r="AW22" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>15754</v>
+        <v>15789</v>
       </c>
       <c r="AY22" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 09/09/2026  8:18:38,42
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="310">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 8 Sep 2026, 07.18</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 9 Sep 2026, 08.17</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,604 +334,607 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>20,35</t>
-  </si>
-  <si>
-    <t>1,16</t>
+    <t>20,32</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>1,74</t>
+  </si>
+  <si>
+    <t>40,22</t>
+  </si>
+  <si>
+    <t>9,63</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>7,54</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,81</t>
+  </si>
+  <si>
+    <t>4,82</t>
+  </si>
+  <si>
+    <t>12,18</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>19,24</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>0,92</t>
+  </si>
+  <si>
+    <t>47,76</t>
+  </si>
+  <si>
+    <t>4,19</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,51</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>2,74</t>
+  </si>
+  <si>
+    <t>3,55</t>
+  </si>
+  <si>
+    <t>14,95</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,73</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>27,28</t>
+  </si>
+  <si>
+    <t>29,98</t>
+  </si>
+  <si>
+    <t>6,44</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>4,63</t>
+  </si>
+  <si>
+    <t>15,78</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>15,96</t>
+  </si>
+  <si>
+    <t>1,94</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>50,15</t>
+  </si>
+  <si>
+    <t>8,48</t>
+  </si>
+  <si>
+    <t>10,34</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>3,69</t>
+  </si>
+  <si>
+    <t>6,92</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>24,38</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>7,19</t>
+  </si>
+  <si>
+    <t>33,86</t>
+  </si>
+  <si>
+    <t>12,24</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>7,09</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>1,83</t>
+  </si>
+  <si>
+    <t>2,08</t>
+  </si>
+  <si>
+    <t>8,91</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,01</t>
+  </si>
+  <si>
+    <t>1,97</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>48,72</t>
+  </si>
+  <si>
+    <t>3,99</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>12,5</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>2,95</t>
+  </si>
+  <si>
+    <t>10,64</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,55</t>
+  </si>
+  <si>
+    <t>0,94</t>
+  </si>
+  <si>
+    <t>40,21</t>
+  </si>
+  <si>
+    <t>13,18</t>
+  </si>
+  <si>
+    <t>7,49</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>1,08</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>6,56</t>
+  </si>
+  <si>
+    <t>9,89</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,7</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>1,46</t>
+  </si>
+  <si>
+    <t>43,21</t>
+  </si>
+  <si>
+    <t>16,5</t>
+  </si>
+  <si>
+    <t>6,11</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>4,35</t>
+  </si>
+  <si>
+    <t>7,01</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,64</t>
+  </si>
+  <si>
+    <t>29,09</t>
+  </si>
+  <si>
+    <t>6,07</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>7,42</t>
+  </si>
+  <si>
+    <t>14,25</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,51</t>
+  </si>
+  <si>
+    <t>0,43</t>
+  </si>
+  <si>
+    <t>31,02</t>
   </si>
   <si>
     <t>1,77</t>
   </si>
   <si>
-    <t>39,7</t>
-  </si>
-  <si>
-    <t>9,81</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>7,52</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,06</t>
+    <t>5,87</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>8,34</t>
+  </si>
+  <si>
+    <t>20,45</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,41</t>
+  </si>
+  <si>
+    <t>0,61</t>
+  </si>
+  <si>
+    <t>33,85</t>
+  </si>
+  <si>
+    <t>4,8</t>
+  </si>
+  <si>
+    <t>5,14</t>
   </si>
   <si>
     <t>0,55</t>
   </si>
   <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,83</t>
-  </si>
-  <si>
-    <t>4,86</t>
-  </si>
-  <si>
-    <t>12,38</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>19,22</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>47,76</t>
-  </si>
-  <si>
-    <t>4,19</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,51</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>2,77</t>
-  </si>
-  <si>
-    <t>3,55</t>
-  </si>
-  <si>
-    <t>14,92</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,77</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>27,16</t>
-  </si>
-  <si>
-    <t>30,06</t>
-  </si>
-  <si>
-    <t>6,4</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>4,64</t>
-  </si>
-  <si>
-    <t>15,83</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>16,05</t>
-  </si>
-  <si>
-    <t>1,97</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>49,7</t>
-  </si>
-  <si>
-    <t>8,65</t>
-  </si>
-  <si>
-    <t>10,4</t>
-  </si>
-  <si>
-    <t>0,37</t>
+    <t>0,82</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>8,12</t>
+  </si>
+  <si>
+    <t>27,73</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>28,96</t>
+  </si>
+  <si>
+    <t>2,27</t>
+  </si>
+  <si>
+    <t>1,25</t>
+  </si>
+  <si>
+    <t>40,18</t>
+  </si>
+  <si>
+    <t>6,59</t>
+  </si>
+  <si>
+    <t>4,39</t>
+  </si>
+  <si>
+    <t>2,67</t>
+  </si>
+  <si>
+    <t>7,4</t>
+  </si>
+  <si>
+    <t>4,73</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>20,17</t>
+  </si>
+  <si>
+    <t>1,4</t>
+  </si>
+  <si>
+    <t>0,9</t>
+  </si>
+  <si>
+    <t>34,01</t>
+  </si>
+  <si>
+    <t>14,96</t>
+  </si>
+  <si>
+    <t>6,62</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>4,14</t>
+  </si>
+  <si>
+    <t>16,66</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,28</t>
+  </si>
+  <si>
+    <t>53,96</t>
+  </si>
+  <si>
+    <t>12,3</t>
+  </si>
+  <si>
+    <t>9,68</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>5,62</t>
+  </si>
+  <si>
+    <t>6,3</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,1</t>
+  </si>
+  <si>
+    <t>2,32</t>
+  </si>
+  <si>
+    <t>35,12</t>
+  </si>
+  <si>
+    <t>4,47</t>
+  </si>
+  <si>
+    <t>15,19</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>1,61</t>
+  </si>
+  <si>
+    <t>3,84</t>
+  </si>
+  <si>
+    <t>17,78</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,27</t>
+  </si>
+  <si>
+    <t>5,81</t>
+  </si>
+  <si>
+    <t>30,56</t>
+  </si>
+  <si>
+    <t>3,95</t>
+  </si>
+  <si>
+    <t>3,06</t>
   </si>
   <si>
     <t>0,7</t>
   </si>
   <si>
-    <t>1</t>
+    <t>1,2</t>
   </si>
   <si>
     <t>3,72</t>
   </si>
   <si>
-    <t>7,03</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>24,4</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>7,23</t>
-  </si>
-  <si>
-    <t>33,71</t>
-  </si>
-  <si>
-    <t>12,3</t>
-  </si>
-  <si>
-    <t>0,67</t>
-  </si>
-  <si>
-    <t>7,1</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>1,82</t>
-  </si>
-  <si>
-    <t>2,09</t>
-  </si>
-  <si>
-    <t>8,93</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>16,01</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>1,01</t>
-  </si>
-  <si>
-    <t>48,48</t>
-  </si>
-  <si>
-    <t>4,17</t>
-  </si>
-  <si>
-    <t>12,23</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>3,02</t>
-  </si>
-  <si>
-    <t>10,88</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,95</t>
-  </si>
-  <si>
-    <t>0,72</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>37,99</t>
-  </si>
-  <si>
-    <t>13,87</t>
-  </si>
-  <si>
-    <t>7,76</t>
-  </si>
-  <si>
-    <t>0,49</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>6,73</t>
-  </si>
-  <si>
-    <t>10,41</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,56</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>1,49</t>
-  </si>
-  <si>
-    <t>43,05</t>
-  </si>
-  <si>
-    <t>16,62</t>
-  </si>
-  <si>
-    <t>6,16</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>4,37</t>
-  </si>
-  <si>
-    <t>7,04</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,65</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>29,08</t>
-  </si>
-  <si>
-    <t>18,01</t>
-  </si>
-  <si>
-    <t>6,07</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>7,42</t>
-  </si>
-  <si>
-    <t>14,26</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,66</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>30,83</t>
-  </si>
-  <si>
-    <t>1,78</t>
-  </si>
-  <si>
-    <t>5,89</t>
-  </si>
-  <si>
-    <t>8,36</t>
-  </si>
-  <si>
-    <t>20,52</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,74</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>32,05</t>
-  </si>
-  <si>
-    <t>5,32</t>
-  </si>
-  <si>
-    <t>5,22</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>0,84</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>8,23</t>
-  </si>
-  <si>
-    <t>28,37</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>2,28</t>
-  </si>
-  <si>
-    <t>1,25</t>
-  </si>
-  <si>
-    <t>40,01</t>
-  </si>
-  <si>
-    <t>6,6</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>2,69</t>
-  </si>
-  <si>
-    <t>7,41</t>
-  </si>
-  <si>
-    <t>4,74</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>19,01</t>
-  </si>
-  <si>
-    <t>1,44</t>
-  </si>
-  <si>
-    <t>1,1</t>
-  </si>
-  <si>
-    <t>15,39</t>
-  </si>
-  <si>
-    <t>6,48</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>4,12</t>
-  </si>
-  <si>
-    <t>17,59</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,35</t>
-  </si>
-  <si>
-    <t>52,54</t>
-  </si>
-  <si>
-    <t>12,91</t>
-  </si>
-  <si>
-    <t>9,9</t>
-  </si>
-  <si>
-    <t>5,78</t>
-  </si>
-  <si>
-    <t>6,58</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,09</t>
-  </si>
-  <si>
-    <t>3,18</t>
-  </si>
-  <si>
-    <t>33,82</t>
-  </si>
-  <si>
-    <t>4,36</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>15,27</t>
-  </si>
-  <si>
-    <t>0,82</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>1,64</t>
-  </si>
-  <si>
-    <t>2,27</t>
-  </si>
-  <si>
-    <t>3,91</t>
-  </si>
-  <si>
-    <t>16,82</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,27</t>
-  </si>
-  <si>
-    <t>5,81</t>
-  </si>
-  <si>
-    <t>30,57</t>
-  </si>
-  <si>
-    <t>3,95</t>
-  </si>
-  <si>
-    <t>3,06</t>
-  </si>
-  <si>
-    <t>33,48</t>
+    <t>33,46</t>
   </si>
   <si>
     <t/>
@@ -1911,40 +1914,40 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>127542</v>
+        <v>130015</v>
       </c>
       <c r="D6" s="6">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>25954</v>
+        <v>26420</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1480</v>
+        <v>1486</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2259</v>
+        <v>2257</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>50630</v>
+        <v>52295</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12513</v>
+        <v>12522</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
@@ -1956,7 +1959,7 @@
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>9596</v>
+        <v>9804</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1974,7 +1977,7 @@
         <v>114</v>
       </c>
       <c r="X6" s="6">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>115</v>
@@ -1986,13 +1989,13 @@
         <v>114</v>
       </c>
       <c r="AB6" s="6">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AC6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="AD6" s="6">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AE6" s="7" t="s">
         <v>116</v>
@@ -2004,55 +2007,55 @@
         <v>117</v>
       </c>
       <c r="AH6" s="6">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AI6" s="7" t="s">
         <v>118</v>
       </c>
       <c r="AJ6" s="6">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="AK6" s="7" t="s">
         <v>119</v>
       </c>
       <c r="AL6" s="6">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AM6" s="7" t="s">
         <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AP6" s="6">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AR6" s="6">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AT6" s="6">
-        <v>1064</v>
+        <v>1056</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AV6" s="6">
-        <v>6195</v>
+        <v>6263</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>15789</v>
+        <v>15842</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>126</v>
@@ -2066,7 +2069,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>7801</v>
+        <v>7808</v>
       </c>
       <c r="D7" s="9">
         <v>8</v>
@@ -2075,7 +2078,7 @@
         <v>129</v>
       </c>
       <c r="F7" s="9">
-        <v>1499</v>
+        <v>1502</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>130</v>
@@ -2093,7 +2096,7 @@
         <v>132</v>
       </c>
       <c r="L7" s="9">
-        <v>3726</v>
+        <v>3729</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>133</v>
@@ -2195,7 +2198,7 @@
         <v>139</v>
       </c>
       <c r="AT7" s="9">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>141</v>
@@ -2207,7 +2210,7 @@
         <v>142</v>
       </c>
       <c r="AX7" s="9">
-        <v>1164</v>
+        <v>1167</v>
       </c>
       <c r="AY7" s="10" t="s">
         <v>143</v>
@@ -2221,7 +2224,7 @@
         <v>145</v>
       </c>
       <c r="C8" s="9">
-        <v>3406</v>
+        <v>3416</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2248,7 +2251,7 @@
         <v>148</v>
       </c>
       <c r="L8" s="9">
-        <v>925</v>
+        <v>932</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>149</v>
@@ -2266,7 +2269,7 @@
         <v>117</v>
       </c>
       <c r="R8" s="9">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="S8" s="10" t="s">
         <v>151</v>
@@ -2350,10 +2353,10 @@
         <v>121</v>
       </c>
       <c r="AT8" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AV8" s="9">
         <v>158</v>
@@ -2376,7 +2379,7 @@
         <v>157</v>
       </c>
       <c r="C9" s="9">
-        <v>10002</v>
+        <v>10171</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
@@ -2385,7 +2388,7 @@
         <v>117</v>
       </c>
       <c r="F9" s="9">
-        <v>1605</v>
+        <v>1623</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>158</v>
@@ -2397,31 +2400,31 @@
         <v>159</v>
       </c>
       <c r="J9" s="9">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>160</v>
       </c>
       <c r="L9" s="9">
-        <v>4971</v>
+        <v>5101</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>161</v>
       </c>
       <c r="N9" s="9">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>162</v>
       </c>
       <c r="P9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R9" s="9">
-        <v>1040</v>
+        <v>1052</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>163</v>
@@ -2505,19 +2508,19 @@
         <v>114</v>
       </c>
       <c r="AT9" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="AV9" s="9">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="AW9" s="10" t="s">
         <v>167</v>
       </c>
       <c r="AX9" s="9">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="AY9" s="10" t="s">
         <v>168</v>
@@ -2531,55 +2534,55 @@
         <v>170</v>
       </c>
       <c r="C10" s="9">
-        <v>21433</v>
+        <v>21515</v>
       </c>
       <c r="D10" s="9">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>137</v>
+        <v>171</v>
       </c>
       <c r="F10" s="9">
-        <v>5229</v>
+        <v>5245</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H10" s="9">
         <v>169</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J10" s="9">
-        <v>1550</v>
+        <v>1547</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L10" s="9">
-        <v>7224</v>
+        <v>7285</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N10" s="9">
-        <v>2637</v>
+        <v>2633</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P10" s="9">
         <v>143</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="R10" s="9">
-        <v>1522</v>
+        <v>1526</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
@@ -2606,16 +2609,16 @@
         <v>118</v>
       </c>
       <c r="AB10" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>178</v>
+        <v>139</v>
       </c>
       <c r="AD10" s="9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
@@ -2657,36 +2660,36 @@
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AT10" s="9">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AV10" s="9">
         <v>447</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AX10" s="9">
-        <v>1915</v>
+        <v>1917</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C11" s="9">
-        <v>14564</v>
+        <v>14931</v>
       </c>
       <c r="D11" s="9">
         <v>13</v>
@@ -2695,52 +2698,52 @@
         <v>123</v>
       </c>
       <c r="F11" s="9">
-        <v>2331</v>
+        <v>2390</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H11" s="9">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J11" s="9">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L11" s="9">
-        <v>7060</v>
+        <v>7275</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="N11" s="9">
-        <v>607</v>
+        <v>596</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="P11" s="9">
         <v>35</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>119</v>
+        <v>190</v>
       </c>
       <c r="R11" s="9">
-        <v>1781</v>
+        <v>1867</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
@@ -2752,7 +2755,7 @@
         <v>11</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
@@ -2779,7 +2782,7 @@
         <v>117</v>
       </c>
       <c r="AH11" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AI11" s="10" t="s">
         <v>120</v>
@@ -2788,7 +2791,7 @@
         <v>38</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2797,16 +2800,16 @@
         <v>114</v>
       </c>
       <c r="AN11" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="AP11" s="9">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="AR11" s="9">
         <v>15</v>
@@ -2815,33 +2818,33 @@
         <v>129</v>
       </c>
       <c r="AT11" s="9">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AV11" s="9">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AX11" s="9">
-        <v>1585</v>
+        <v>1588</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C12" s="9">
-        <v>5257</v>
+        <v>5531</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
@@ -2850,16 +2853,16 @@
         <v>117</v>
       </c>
       <c r="F12" s="9">
-        <v>996</v>
+        <v>1026</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>199</v>
+        <v>165</v>
       </c>
       <c r="J12" s="9">
         <v>52</v>
@@ -2868,7 +2871,7 @@
         <v>200</v>
       </c>
       <c r="L12" s="9">
-        <v>1997</v>
+        <v>2224</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>201</v>
@@ -2880,13 +2883,13 @@
         <v>202</v>
       </c>
       <c r="P12" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="R12" s="9">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>203</v>
@@ -2907,7 +2910,7 @@
         <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>204</v>
+        <v>153</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
@@ -2925,7 +2928,7 @@
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
@@ -2943,7 +2946,7 @@
         <v>31</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
@@ -2961,7 +2964,7 @@
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -2973,66 +2976,66 @@
         <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="AV12" s="9">
+        <v>363</v>
+      </c>
+      <c r="AW12" s="10" t="s">
         <v>207</v>
-      </c>
-      <c r="AV12" s="9">
-        <v>354</v>
-      </c>
-      <c r="AW12" s="10" t="s">
-        <v>208</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>211</v>
-      </c>
       <c r="C13" s="9">
-        <v>4971</v>
+        <v>5006</v>
       </c>
       <c r="D13" s="9">
         <v>6</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F13" s="9">
-        <v>873</v>
+        <v>886</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="J13" s="9">
+        <v>73</v>
+      </c>
+      <c r="K13" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="J13" s="9">
-        <v>74</v>
-      </c>
-      <c r="K13" s="10" t="s">
+      <c r="L13" s="9">
+        <v>2163</v>
+      </c>
+      <c r="M13" s="10" t="s">
         <v>214</v>
-      </c>
-      <c r="L13" s="9">
-        <v>2140</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>215</v>
       </c>
       <c r="N13" s="9">
         <v>826</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P13" s="9">
         <v>5</v>
@@ -3044,7 +3047,7 @@
         <v>306</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
@@ -3098,13 +3101,13 @@
         <v>33</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AN13" s="9">
         <v>5</v>
@@ -3116,42 +3119,42 @@
         <v>38</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="AT13" s="9">
+        <v>13</v>
+      </c>
+      <c r="AU13" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="AT13" s="9">
-        <v>15</v>
-      </c>
-      <c r="AU13" s="10" t="s">
+      <c r="AV13" s="9">
+        <v>218</v>
+      </c>
+      <c r="AW13" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AV13" s="9">
-        <v>217</v>
-      </c>
-      <c r="AW13" s="10" t="s">
+      <c r="AX13" s="9">
+        <v>351</v>
+      </c>
+      <c r="AY13" s="10" t="s">
         <v>222</v>
-      </c>
-      <c r="AX13" s="9">
-        <v>350</v>
-      </c>
-      <c r="AY13" s="10" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>225</v>
-      </c>
       <c r="C14" s="9">
-        <v>4959</v>
+        <v>4960</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
@@ -3163,31 +3166,31 @@
         <v>1123</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>227</v>
+        <v>164</v>
       </c>
       <c r="J14" s="9">
         <v>18</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>227</v>
+        <v>164</v>
       </c>
       <c r="L14" s="9">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="N14" s="9">
         <v>893</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>229</v>
+        <v>104</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
@@ -3199,7 +3202,7 @@
         <v>301</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
@@ -3253,7 +3256,7 @@
         <v>16</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3271,7 +3274,7 @@
         <v>34</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>231</v>
+        <v>165</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3283,30 +3286,30 @@
         <v>17</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AV14" s="9">
         <v>368</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AX14" s="9">
         <v>707</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C15" s="9">
-        <v>12679</v>
+        <v>12775</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -3315,52 +3318,52 @@
         <v>117</v>
       </c>
       <c r="F15" s="9">
-        <v>3888</v>
+        <v>3898</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="J15" s="9">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>106</v>
+        <v>190</v>
       </c>
       <c r="L15" s="9">
-        <v>3909</v>
+        <v>3963</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="P15" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R15" s="9">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
@@ -3372,7 +3375,7 @@
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
@@ -3399,69 +3402,69 @@
         <v>117</v>
       </c>
       <c r="AH15" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AJ15" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="AL15" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AM15" s="10" t="s">
         <v>114</v>
       </c>
       <c r="AN15" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AP15" s="9">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="AR15" s="9">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="AT15" s="9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="AV15" s="9">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="AX15" s="9">
-        <v>2602</v>
+        <v>2612</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C16" s="9">
-        <v>5114</v>
+        <v>5273</v>
       </c>
       <c r="D16" s="9">
         <v>1</v>
@@ -3470,16 +3473,16 @@
         <v>114</v>
       </c>
       <c r="F16" s="9">
-        <v>907</v>
+        <v>918</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="J16" s="9">
         <v>4</v>
@@ -3488,16 +3491,16 @@
         <v>106</v>
       </c>
       <c r="L16" s="9">
-        <v>1639</v>
+        <v>1785</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="N16" s="9">
-        <v>272</v>
+        <v>253</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="P16" s="9">
         <v>1</v>
@@ -3506,10 +3509,10 @@
         <v>114</v>
       </c>
       <c r="R16" s="9">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
@@ -3527,7 +3530,7 @@
         <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
@@ -3563,7 +3566,7 @@
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3581,90 +3584,90 @@
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AT16" s="9">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AU16" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="AV16" s="9">
+        <v>428</v>
+      </c>
+      <c r="AW16" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="AX16" s="9">
+        <v>1462</v>
+      </c>
+      <c r="AY16" s="10" t="s">
         <v>253</v>
-      </c>
-      <c r="AV16" s="9">
-        <v>421</v>
-      </c>
-      <c r="AW16" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="AX16" s="9">
-        <v>1451</v>
-      </c>
-      <c r="AY16" s="10" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C17" s="9">
-        <v>10292</v>
+        <v>10335</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F17" s="9">
         <v>2993</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="H17" s="9">
         <v>235</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J17" s="9">
         <v>129</v>
       </c>
       <c r="K17" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="L17" s="9">
+        <v>4153</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="L17" s="9">
-        <v>4118</v>
-      </c>
-      <c r="M17" s="10" t="s">
+      <c r="N17" s="9">
+        <v>681</v>
+      </c>
+      <c r="O17" s="10" t="s">
         <v>261</v>
-      </c>
-      <c r="N17" s="9">
-        <v>679</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>262</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>263</v>
+        <v>171</v>
       </c>
       <c r="R17" s="9">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>222</v>
+        <v>262</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -3718,7 +3721,7 @@
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
@@ -3736,75 +3739,75 @@
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AT17" s="9">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="AU17" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="AV17" s="9">
+        <v>765</v>
+      </c>
+      <c r="AW17" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="AV17" s="9">
-        <v>763</v>
-      </c>
-      <c r="AW17" s="10" t="s">
+      <c r="AX17" s="9">
+        <v>489</v>
+      </c>
+      <c r="AY17" s="10" t="s">
         <v>265</v>
-      </c>
-      <c r="AX17" s="9">
-        <v>488</v>
-      </c>
-      <c r="AY17" s="10" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="C18" s="9">
+        <v>11077</v>
+      </c>
+      <c r="D18" s="9">
+        <v>2</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F18" s="9">
+        <v>2234</v>
+      </c>
+      <c r="G18" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="C18" s="9">
-        <v>10451</v>
-      </c>
-      <c r="D18" s="9">
-        <v>1</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F18" s="9">
-        <v>1987</v>
-      </c>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="9">
+        <v>155</v>
+      </c>
+      <c r="I18" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="H18" s="9">
-        <v>151</v>
-      </c>
-      <c r="I18" s="10" t="s">
+      <c r="J18" s="9">
+        <v>100</v>
+      </c>
+      <c r="K18" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="J18" s="9">
-        <v>115</v>
-      </c>
-      <c r="K18" s="10" t="s">
+      <c r="L18" s="9">
+        <v>3767</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="L18" s="9">
-        <v>3523</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>174</v>
-      </c>
       <c r="N18" s="9">
-        <v>1608</v>
+        <v>1657</v>
       </c>
       <c r="O18" s="10" t="s">
         <v>272</v>
@@ -3816,7 +3819,7 @@
         <v>118</v>
       </c>
       <c r="R18" s="9">
-        <v>677</v>
+        <v>733</v>
       </c>
       <c r="S18" s="10" t="s">
         <v>273</v>
@@ -3834,10 +3837,10 @@
         <v>117</v>
       </c>
       <c r="X18" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>178</v>
+        <v>123</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
@@ -3873,13 +3876,13 @@
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>207</v>
+        <v>129</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="AN18" s="9">
         <v>2</v>
@@ -3891,13 +3894,13 @@
         <v>38</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="AT18" s="9">
         <v>1</v>
@@ -3906,13 +3909,13 @@
         <v>118</v>
       </c>
       <c r="AV18" s="9">
-        <v>431</v>
+        <v>459</v>
       </c>
       <c r="AW18" s="10" t="s">
         <v>275</v>
       </c>
       <c r="AX18" s="9">
-        <v>1838</v>
+        <v>1845</v>
       </c>
       <c r="AY18" s="10" t="s">
         <v>276</v>
@@ -3926,16 +3929,16 @@
         <v>278</v>
       </c>
       <c r="C19" s="9">
-        <v>12932</v>
+        <v>13516</v>
       </c>
       <c r="D19" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F19" s="9">
-        <v>1468</v>
+        <v>1524</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>279</v>
@@ -3944,22 +3947,22 @@
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="J19" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L19" s="9">
-        <v>6795</v>
+        <v>7293</v>
       </c>
       <c r="M19" s="10" t="s">
         <v>280</v>
       </c>
       <c r="N19" s="9">
-        <v>1670</v>
+        <v>1663</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>281</v>
@@ -3971,7 +3974,7 @@
         <v>117</v>
       </c>
       <c r="R19" s="9">
-        <v>1280</v>
+        <v>1309</v>
       </c>
       <c r="S19" s="10" t="s">
         <v>282</v>
@@ -3992,7 +3995,7 @@
         <v>19</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
@@ -4028,7 +4031,7 @@
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
@@ -4046,7 +4049,7 @@
         <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>153</v>
+        <v>283</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
@@ -4055,33 +4058,33 @@
         <v>118</v>
       </c>
       <c r="AT19" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AV19" s="9">
-        <v>748</v>
+        <v>759</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AX19" s="9">
         <v>851</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C20" s="9">
-        <v>1100</v>
+        <v>1119</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
@@ -4090,10 +4093,10 @@
         <v>123</v>
       </c>
       <c r="F20" s="9">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
@@ -4102,31 +4105,31 @@
         <v>122</v>
       </c>
       <c r="J20" s="9">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L20" s="9">
-        <v>372</v>
+        <v>393</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="N20" s="9">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="P20" s="9">
         <v>7</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>291</v>
+        <v>239</v>
       </c>
       <c r="R20" s="9">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S20" s="10" t="s">
         <v>292</v>
@@ -4153,7 +4156,7 @@
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
@@ -4174,16 +4177,16 @@
         <v>117</v>
       </c>
       <c r="AH20" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="AJ20" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>122</v>
+        <v>239</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
@@ -4201,42 +4204,42 @@
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>227</v>
+        <v>164</v>
       </c>
       <c r="AT20" s="9">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>296</v>
+        <v>166</v>
       </c>
       <c r="AV20" s="9">
         <v>43</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="AX20" s="9">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C21" s="9">
-        <v>2581</v>
+        <v>2582</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -4248,13 +4251,13 @@
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J21" s="9">
         <v>2</v>
@@ -4266,25 +4269,25 @@
         <v>789</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
@@ -4302,7 +4305,7 @@
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4338,7 +4341,7 @@
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
@@ -4356,7 +4359,7 @@
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>165</v>
+        <v>304</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
@@ -4365,66 +4368,66 @@
         <v>139</v>
       </c>
       <c r="AT21" s="9">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>108</v>
+        <v>305</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>167</v>
+        <v>306</v>
       </c>
       <c r="AX21" s="9">
         <v>864</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C22" s="12">
-        <v>127542</v>
+        <v>130015</v>
       </c>
       <c r="D22" s="12">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>25954</v>
+        <v>26420</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1480</v>
+        <v>1486</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2259</v>
+        <v>2257</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>50630</v>
+        <v>52295</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12513</v>
+        <v>12522</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
@@ -4436,7 +4439,7 @@
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>9596</v>
+        <v>9804</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4454,7 +4457,7 @@
         <v>114</v>
       </c>
       <c r="X22" s="12">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>115</v>
@@ -4466,13 +4469,13 @@
         <v>114</v>
       </c>
       <c r="AB22" s="12">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AC22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="AD22" s="12">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AE22" s="13" t="s">
         <v>116</v>
@@ -4484,55 +4487,55 @@
         <v>117</v>
       </c>
       <c r="AH22" s="12">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AI22" s="13" t="s">
         <v>118</v>
       </c>
       <c r="AJ22" s="12">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="AK22" s="13" t="s">
         <v>119</v>
       </c>
       <c r="AL22" s="12">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AM22" s="13" t="s">
         <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AP22" s="12">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AR22" s="12">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AT22" s="12">
-        <v>1064</v>
+        <v>1056</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AV22" s="12">
-        <v>6195</v>
+        <v>6263</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>15789</v>
+        <v>15842</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>126</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 10/09/2026  8:09:17,49
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="307">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 9 Sep 2026, 08.17</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 10 Sep 2026, 08.07</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,42 +334,42 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>20,32</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>1,74</t>
-  </si>
-  <si>
-    <t>40,22</t>
-  </si>
-  <si>
-    <t>9,63</t>
+    <t>20,23</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>1,66</t>
+  </si>
+  <si>
+    <t>40,95</t>
+  </si>
+  <si>
+    <t>9,39</t>
   </si>
   <si>
     <t>0,18</t>
   </si>
   <si>
-    <t>7,54</t>
+    <t>7,56</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,16</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
     <t>0</t>
   </si>
   <si>
-    <t>0,01</t>
-  </si>
-  <si>
     <t>0,24</t>
   </si>
   <si>
@@ -385,13 +385,13 @@
     <t>0,09</t>
   </si>
   <si>
-    <t>0,81</t>
-  </si>
-  <si>
-    <t>4,82</t>
-  </si>
-  <si>
-    <t>12,18</t>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>4,77</t>
+  </si>
+  <si>
+    <t>11,96</t>
   </si>
   <si>
     <t>1801</t>
@@ -403,25 +403,25 @@
     <t>0,1</t>
   </si>
   <si>
-    <t>19,24</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>47,76</t>
-  </si>
-  <si>
-    <t>4,19</t>
+    <t>19,18</t>
+  </si>
+  <si>
+    <t>0,94</t>
+  </si>
+  <si>
+    <t>0,9</t>
+  </si>
+  <si>
+    <t>47,73</t>
+  </si>
+  <si>
+    <t>4,17</t>
   </si>
   <si>
     <t>0,14</t>
   </si>
   <si>
-    <t>4,51</t>
+    <t>4,49</t>
   </si>
   <si>
     <t>0,19</t>
@@ -433,16 +433,16 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>2,74</t>
-  </si>
-  <si>
-    <t>3,55</t>
-  </si>
-  <si>
-    <t>14,95</t>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>2,56</t>
+  </si>
+  <si>
+    <t>3,53</t>
+  </si>
+  <si>
+    <t>15,27</t>
   </si>
   <si>
     <t>1802</t>
@@ -451,22 +451,25 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>13,73</t>
+    <t>13,75</t>
   </si>
   <si>
     <t>0,5</t>
   </si>
   <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>27,28</t>
-  </si>
-  <si>
-    <t>29,98</t>
-  </si>
-  <si>
-    <t>6,44</t>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>27,29</t>
+  </si>
+  <si>
+    <t>30,04</t>
+  </si>
+  <si>
+    <t>6,48</t>
+  </si>
+  <si>
+    <t>0,2</t>
   </si>
   <si>
     <t>0,15</t>
@@ -475,10 +478,10 @@
     <t>0,47</t>
   </si>
   <si>
-    <t>4,63</t>
-  </si>
-  <si>
-    <t>15,78</t>
+    <t>4,61</t>
+  </si>
+  <si>
+    <t>15,73</t>
   </si>
   <si>
     <t>1803</t>
@@ -487,454 +490,442 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>15,96</t>
-  </si>
-  <si>
-    <t>1,94</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>50,15</t>
-  </si>
-  <si>
-    <t>8,48</t>
+    <t>15,91</t>
+  </si>
+  <si>
+    <t>1,87</t>
+  </si>
+  <si>
+    <t>50,69</t>
+  </si>
+  <si>
+    <t>8,26</t>
   </si>
   <si>
     <t>10,34</t>
   </si>
   <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>3,68</t>
+  </si>
+  <si>
+    <t>6,83</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>24,37</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>7,16</t>
+  </si>
+  <si>
+    <t>33,91</t>
+  </si>
+  <si>
+    <t>12,21</t>
+  </si>
+  <si>
+    <t>7,12</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>1,84</t>
+  </si>
+  <si>
+    <t>2,07</t>
+  </si>
+  <si>
+    <t>8,88</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,3</t>
+  </si>
+  <si>
+    <t>1,83</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>49,82</t>
+  </si>
+  <si>
+    <t>3,6</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>2,87</t>
+  </si>
+  <si>
+    <t>10,17</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>18,13</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>0,91</t>
+  </si>
+  <si>
+    <t>41,87</t>
+  </si>
+  <si>
+    <t>12,7</t>
+  </si>
+  <si>
+    <t>7,23</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>1,05</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>9,53</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,65</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>1,41</t>
+  </si>
+  <si>
+    <t>43,31</t>
+  </si>
+  <si>
+    <t>16,49</t>
+  </si>
+  <si>
+    <t>6,16</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>4,34</t>
+  </si>
+  <si>
+    <t>6,99</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,54</t>
+  </si>
+  <si>
     <t>0,36</t>
   </si>
   <si>
+    <t>29,22</t>
+  </si>
+  <si>
+    <t>17,91</t>
+  </si>
+  <si>
+    <t>6,1</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>7,38</t>
+  </si>
+  <si>
+    <t>14,18</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,4</t>
+  </si>
+  <si>
+    <t>0,43</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>31,38</t>
+  </si>
+  <si>
+    <t>1,75</t>
+  </si>
+  <si>
+    <t>5,84</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>8,3</t>
+  </si>
+  <si>
+    <t>20,29</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,49</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>34,26</t>
+  </si>
+  <si>
+    <t>4,69</t>
+  </si>
+  <si>
+    <t>5,1</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>7,99</t>
+  </si>
+  <si>
+    <t>27,86</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>28,75</t>
+  </si>
+  <si>
+    <t>2,27</t>
+  </si>
+  <si>
+    <t>1,25</t>
+  </si>
+  <si>
+    <t>40,41</t>
+  </si>
+  <si>
+    <t>6,54</t>
+  </si>
+  <si>
+    <t>4,4</t>
+  </si>
+  <si>
+    <t>2,62</t>
+  </si>
+  <si>
+    <t>7,43</t>
+  </si>
+  <si>
+    <t>4,8</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>20,26</t>
+  </si>
+  <si>
+    <t>34,69</t>
+  </si>
+  <si>
+    <t>14,88</t>
+  </si>
+  <si>
+    <t>6,6</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>4,12</t>
+  </si>
+  <si>
+    <t>16,45</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,63</t>
+  </si>
+  <si>
+    <t>55,41</t>
+  </si>
+  <si>
+    <t>11,17</t>
+  </si>
+  <si>
+    <t>9,87</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>5,36</t>
+  </si>
+  <si>
+    <t>5,7</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,1</t>
+  </si>
+  <si>
+    <t>2,23</t>
+  </si>
+  <si>
+    <t>35,21</t>
+  </si>
+  <si>
+    <t>4,47</t>
+  </si>
+  <si>
+    <t>15,28</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>1,61</t>
+  </si>
+  <si>
+    <t>3,84</t>
+  </si>
+  <si>
+    <t>17,78</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,15</t>
+  </si>
+  <si>
+    <t>5,77</t>
+  </si>
+  <si>
+    <t>30,42</t>
+  </si>
+  <si>
+    <t>3,92</t>
+  </si>
+  <si>
+    <t>3,04</t>
+  </si>
+  <si>
     <t>0,69</t>
   </si>
   <si>
-    <t>0,98</t>
+    <t>1,81</t>
   </si>
   <si>
     <t>3,69</t>
   </si>
   <si>
-    <t>6,92</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>24,38</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>7,19</t>
-  </si>
-  <si>
-    <t>33,86</t>
-  </si>
-  <si>
-    <t>12,24</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>7,09</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>1,83</t>
-  </si>
-  <si>
-    <t>2,08</t>
-  </si>
-  <si>
-    <t>8,91</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>16,01</t>
-  </si>
-  <si>
-    <t>1,97</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>48,72</t>
-  </si>
-  <si>
-    <t>3,99</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>12,5</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>2,95</t>
-  </si>
-  <si>
-    <t>10,64</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,55</t>
-  </si>
-  <si>
-    <t>0,94</t>
-  </si>
-  <si>
-    <t>40,21</t>
-  </si>
-  <si>
-    <t>13,18</t>
-  </si>
-  <si>
-    <t>7,49</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>1,08</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>6,56</t>
-  </si>
-  <si>
-    <t>9,89</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,7</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>1,46</t>
-  </si>
-  <si>
-    <t>43,21</t>
-  </si>
-  <si>
-    <t>16,5</t>
-  </si>
-  <si>
-    <t>6,11</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>4,35</t>
-  </si>
-  <si>
-    <t>7,01</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,64</t>
-  </si>
-  <si>
-    <t>29,09</t>
-  </si>
-  <si>
-    <t>6,07</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>7,42</t>
-  </si>
-  <si>
-    <t>14,25</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,51</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>31,02</t>
-  </si>
-  <si>
-    <t>1,77</t>
-  </si>
-  <si>
-    <t>5,87</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>8,34</t>
-  </si>
-  <si>
-    <t>20,45</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,41</t>
-  </si>
-  <si>
-    <t>0,61</t>
-  </si>
-  <si>
-    <t>33,85</t>
-  </si>
-  <si>
-    <t>4,8</t>
-  </si>
-  <si>
-    <t>5,14</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>0,82</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>8,12</t>
-  </si>
-  <si>
-    <t>27,73</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>28,96</t>
-  </si>
-  <si>
-    <t>2,27</t>
-  </si>
-  <si>
-    <t>1,25</t>
-  </si>
-  <si>
-    <t>40,18</t>
-  </si>
-  <si>
-    <t>6,59</t>
-  </si>
-  <si>
-    <t>4,39</t>
-  </si>
-  <si>
-    <t>2,67</t>
-  </si>
-  <si>
-    <t>7,4</t>
-  </si>
-  <si>
-    <t>4,73</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>20,17</t>
-  </si>
-  <si>
-    <t>1,4</t>
-  </si>
-  <si>
-    <t>0,9</t>
-  </si>
-  <si>
-    <t>34,01</t>
-  </si>
-  <si>
-    <t>14,96</t>
-  </si>
-  <si>
-    <t>6,62</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>4,14</t>
-  </si>
-  <si>
-    <t>16,66</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,28</t>
-  </si>
-  <si>
-    <t>53,96</t>
-  </si>
-  <si>
-    <t>12,3</t>
-  </si>
-  <si>
-    <t>9,68</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>5,62</t>
-  </si>
-  <si>
-    <t>6,3</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,1</t>
-  </si>
-  <si>
-    <t>2,32</t>
-  </si>
-  <si>
-    <t>35,12</t>
-  </si>
-  <si>
-    <t>4,47</t>
-  </si>
-  <si>
-    <t>15,19</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>1,61</t>
-  </si>
-  <si>
-    <t>3,84</t>
-  </si>
-  <si>
-    <t>17,78</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,27</t>
-  </si>
-  <si>
-    <t>5,81</t>
-  </si>
-  <si>
-    <t>30,56</t>
-  </si>
-  <si>
-    <t>3,95</t>
-  </si>
-  <si>
-    <t>3,06</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>1,2</t>
-  </si>
-  <si>
-    <t>3,72</t>
-  </si>
-  <si>
-    <t>33,46</t>
+    <t>33,23</t>
   </si>
   <si>
     <t/>
@@ -1914,52 +1905,52 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>130015</v>
+        <v>133133</v>
       </c>
       <c r="D6" s="6">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>26420</v>
+        <v>26935</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1486</v>
+        <v>1483</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2257</v>
+        <v>2206</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>52295</v>
+        <v>54514</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12522</v>
+        <v>12507</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>9804</v>
+        <v>10067</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1968,52 +1959,52 @@
         <v>98</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Z6" s="6">
         <v>26</v>
       </c>
       <c r="AA6" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AD6" s="6">
         <v>93</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="AF6" s="6">
         <v>1</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH6" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ6" s="6">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="AK6" s="7" t="s">
         <v>119</v>
@@ -2025,37 +2016,37 @@
         <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AP6" s="6">
-        <v>707</v>
+        <v>722</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AR6" s="6">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AT6" s="6">
-        <v>1056</v>
+        <v>1048</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AV6" s="6">
-        <v>6263</v>
+        <v>6349</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>15842</v>
+        <v>15929</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>126</v>
@@ -2069,7 +2060,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>7808</v>
+        <v>7848</v>
       </c>
       <c r="D7" s="9">
         <v>8</v>
@@ -2078,7 +2069,7 @@
         <v>129</v>
       </c>
       <c r="F7" s="9">
-        <v>1502</v>
+        <v>1505</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>130</v>
@@ -2090,13 +2081,13 @@
         <v>131</v>
       </c>
       <c r="J7" s="9">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>132</v>
       </c>
       <c r="L7" s="9">
-        <v>3729</v>
+        <v>3746</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>133</v>
@@ -2126,7 +2117,7 @@
         <v>120</v>
       </c>
       <c r="V7" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7" s="10" t="s">
         <v>118</v>
@@ -2159,13 +2150,13 @@
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH7" s="9">
         <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ7" s="9">
         <v>10</v>
@@ -2177,7 +2168,7 @@
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN7" s="9">
         <v>3</v>
@@ -2186,7 +2177,7 @@
         <v>139</v>
       </c>
       <c r="AP7" s="9">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="AQ7" s="10" t="s">
         <v>140</v>
@@ -2198,7 +2189,7 @@
         <v>139</v>
       </c>
       <c r="AT7" s="9">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>141</v>
@@ -2210,7 +2201,7 @@
         <v>142</v>
       </c>
       <c r="AX7" s="9">
-        <v>1167</v>
+        <v>1198</v>
       </c>
       <c r="AY7" s="10" t="s">
         <v>143</v>
@@ -2224,16 +2215,16 @@
         <v>145</v>
       </c>
       <c r="C8" s="9">
-        <v>3416</v>
+        <v>3426</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F8" s="9">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>146</v>
@@ -2245,19 +2236,19 @@
         <v>147</v>
       </c>
       <c r="J8" s="9">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>148</v>
       </c>
       <c r="L8" s="9">
-        <v>932</v>
+        <v>935</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>149</v>
       </c>
       <c r="N8" s="9">
-        <v>1024</v>
+        <v>1029</v>
       </c>
       <c r="O8" s="10" t="s">
         <v>150</v>
@@ -2266,10 +2257,10 @@
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R8" s="9">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="S8" s="10" t="s">
         <v>151</v>
@@ -2278,31 +2269,31 @@
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X8" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
@@ -2314,37 +2305,37 @@
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
@@ -2362,69 +2353,69 @@
         <v>158</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="AX8" s="9">
         <v>539</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C9" s="9">
-        <v>10171</v>
+        <v>10406</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F9" s="9">
-        <v>1623</v>
+        <v>1656</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H9" s="9">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J9" s="9">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="L9" s="9">
-        <v>5101</v>
+        <v>5275</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>161</v>
       </c>
       <c r="N9" s="9">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>162</v>
       </c>
       <c r="P9" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="R9" s="9">
-        <v>1052</v>
+        <v>1076</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>163</v>
@@ -2433,16 +2424,16 @@
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X9" s="9">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y9" s="10" t="s">
         <v>164</v>
@@ -2451,13 +2442,13 @@
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD9" s="9">
         <v>9</v>
@@ -2469,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ9" s="9">
         <v>70</v>
@@ -2487,16 +2478,16 @@
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP9" s="9">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AQ9" s="10" t="s">
         <v>166</v>
@@ -2505,22 +2496,22 @@
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AT9" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="AV9" s="9">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="AW9" s="10" t="s">
         <v>167</v>
       </c>
       <c r="AX9" s="9">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="AY9" s="10" t="s">
         <v>168</v>
@@ -2534,61 +2525,61 @@
         <v>170</v>
       </c>
       <c r="C10" s="9">
-        <v>21515</v>
+        <v>21580</v>
       </c>
       <c r="D10" s="9">
         <v>43</v>
       </c>
       <c r="E10" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F10" s="9">
+        <v>5260</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="F10" s="9">
-        <v>5245</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="H10" s="9">
         <v>172</v>
       </c>
-      <c r="H10" s="9">
-        <v>169</v>
-      </c>
       <c r="I10" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="J10" s="9">
+        <v>1545</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="J10" s="9">
-        <v>1547</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="L10" s="9">
+        <v>7317</v>
+      </c>
+      <c r="M10" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="L10" s="9">
-        <v>7285</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="N10" s="9">
+        <v>2634</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="N10" s="9">
-        <v>2633</v>
-      </c>
-      <c r="O10" s="10" t="s">
+      <c r="P10" s="9">
+        <v>144</v>
+      </c>
+      <c r="Q10" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="R10" s="9">
+        <v>1536</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>176</v>
-      </c>
-      <c r="P10" s="9">
-        <v>143</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="R10" s="9">
-        <v>1526</v>
-      </c>
-      <c r="S10" s="10" t="s">
-        <v>178</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V10" s="9">
         <v>7</v>
@@ -2600,13 +2591,13 @@
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AB10" s="9">
         <v>9</v>
@@ -2624,10 +2615,10 @@
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH10" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AI10" s="10" t="s">
         <v>139</v>
@@ -2642,13 +2633,13 @@
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN10" s="9">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>119</v>
+        <v>177</v>
       </c>
       <c r="AP10" s="9">
         <v>31</v>
@@ -2660,90 +2651,90 @@
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="AT10" s="9">
+        <v>397</v>
+      </c>
+      <c r="AU10" s="10" t="s">
         <v>179</v>
-      </c>
-      <c r="AT10" s="9">
-        <v>394</v>
-      </c>
-      <c r="AU10" s="10" t="s">
-        <v>180</v>
       </c>
       <c r="AV10" s="9">
         <v>447</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AX10" s="9">
         <v>1917</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>184</v>
-      </c>
       <c r="C11" s="9">
-        <v>14931</v>
+        <v>15619</v>
       </c>
       <c r="D11" s="9">
         <v>13</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="F11" s="9">
-        <v>2390</v>
+        <v>2546</v>
       </c>
       <c r="G11" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="H11" s="9">
+        <v>286</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="H11" s="9">
-        <v>294</v>
-      </c>
-      <c r="I11" s="10" t="s">
+      <c r="J11" s="9">
+        <v>155</v>
+      </c>
+      <c r="K11" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="J11" s="9">
-        <v>148</v>
-      </c>
-      <c r="K11" s="10" t="s">
+      <c r="L11" s="9">
+        <v>7782</v>
+      </c>
+      <c r="M11" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="L11" s="9">
-        <v>7275</v>
-      </c>
-      <c r="M11" s="10" t="s">
+      <c r="N11" s="9">
+        <v>563</v>
+      </c>
+      <c r="O11" s="10" t="s">
         <v>188</v>
-      </c>
-      <c r="N11" s="9">
-        <v>596</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>189</v>
       </c>
       <c r="P11" s="9">
         <v>35</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="R11" s="9">
-        <v>1867</v>
+        <v>1907</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
@@ -2755,7 +2746,7 @@
         <v>11</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
@@ -2767,19 +2758,19 @@
         <v>3</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AD11" s="9">
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH11" s="9">
         <v>4</v>
@@ -2788,81 +2779,81 @@
         <v>120</v>
       </c>
       <c r="AJ11" s="9">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AN11" s="9">
         <v>3</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AP11" s="9">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="AR11" s="9">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="AT11" s="9">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="AU11" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="AV11" s="9">
+        <v>449</v>
+      </c>
+      <c r="AW11" s="10" t="s">
         <v>194</v>
-      </c>
-      <c r="AV11" s="9">
-        <v>441</v>
-      </c>
-      <c r="AW11" s="10" t="s">
-        <v>195</v>
       </c>
       <c r="AX11" s="9">
         <v>1588</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="9">
+        <v>5741</v>
+      </c>
+      <c r="D12" s="9">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="9">
+        <v>1041</v>
+      </c>
+      <c r="G12" s="10" t="s">
         <v>198</v>
-      </c>
-      <c r="C12" s="9">
-        <v>5531</v>
-      </c>
-      <c r="D12" s="9">
-        <v>0</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F12" s="9">
-        <v>1026</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>199</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="J12" s="9">
         <v>52</v>
@@ -2871,7 +2862,7 @@
         <v>200</v>
       </c>
       <c r="L12" s="9">
-        <v>2224</v>
+        <v>2404</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>201</v>
@@ -2886,10 +2877,10 @@
         <v>2</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="R12" s="9">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>203</v>
@@ -2898,144 +2889,144 @@
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V12" s="9">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X12" s="9">
         <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>153</v>
+        <v>204</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD12" s="9">
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>112</v>
+        <v>205</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH12" s="9">
         <v>0</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ12" s="9">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN12" s="9">
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP12" s="9">
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AT12" s="9">
         <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>206</v>
+        <v>129</v>
       </c>
       <c r="AV12" s="9">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C13" s="9">
-        <v>5006</v>
+        <v>5020</v>
       </c>
       <c r="D13" s="9">
         <v>6</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F13" s="9">
         <v>886</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J13" s="9">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L13" s="9">
-        <v>2163</v>
+        <v>2174</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N13" s="9">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P13" s="9">
         <v>5</v>
@@ -3044,16 +3035,16 @@
         <v>129</v>
       </c>
       <c r="R13" s="9">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V13" s="9">
         <v>3</v>
@@ -3071,25 +3062,25 @@
         <v>1</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH13" s="9">
         <v>2</v>
@@ -3101,13 +3092,13 @@
         <v>33</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>217</v>
+        <v>189</v>
       </c>
       <c r="AN13" s="9">
         <v>5</v>
@@ -3131,57 +3122,57 @@
         <v>13</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>220</v>
+        <v>191</v>
       </c>
       <c r="AV13" s="9">
         <v>218</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AX13" s="9">
         <v>351</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="9">
+        <v>4986</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1124</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>224</v>
-      </c>
-      <c r="C14" s="9">
-        <v>4960</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1123</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>225</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="J14" s="9">
         <v>18</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="L14" s="9">
-        <v>1443</v>
+        <v>1457</v>
       </c>
       <c r="M14" s="10" t="s">
         <v>226</v>
@@ -3190,19 +3181,19 @@
         <v>893</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>104</v>
+        <v>227</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="R14" s="9">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
@@ -3214,7 +3205,7 @@
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X14" s="9">
         <v>9</v>
@@ -3226,13 +3217,13 @@
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
@@ -3244,43 +3235,43 @@
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ14" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>228</v>
+        <v>140</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AN14" s="9">
         <v>1</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AP14" s="9">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>165</v>
+        <v>218</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AT14" s="9">
         <v>17</v>
@@ -3309,16 +3300,16 @@
         <v>233</v>
       </c>
       <c r="C15" s="9">
-        <v>12775</v>
+        <v>12883</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F15" s="9">
-        <v>3898</v>
+        <v>3917</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>234</v>
@@ -3330,82 +3321,82 @@
         <v>235</v>
       </c>
       <c r="J15" s="9">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="L15" s="9">
-        <v>3963</v>
+        <v>4043</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="N15" s="9">
         <v>226</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P15" s="9">
         <v>0</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R15" s="9">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH15" s="9">
         <v>0</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ15" s="9">
         <v>13</v>
@@ -3417,19 +3408,19 @@
         <v>2</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AN15" s="9">
         <v>0</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP15" s="9">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>239</v>
+        <v>148</v>
       </c>
       <c r="AR15" s="9">
         <v>18</v>
@@ -3438,99 +3429,99 @@
         <v>135</v>
       </c>
       <c r="AT15" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AV15" s="9">
-        <v>1066</v>
+        <v>1069</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AX15" s="9">
-        <v>2612</v>
+        <v>2614</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C16" s="9">
-        <v>5273</v>
+        <v>5391</v>
       </c>
       <c r="D16" s="9">
         <v>1</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F16" s="9">
-        <v>918</v>
+        <v>943</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J16" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="L16" s="9">
-        <v>1785</v>
+        <v>1847</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N16" s="9">
         <v>253</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P16" s="9">
         <v>1</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="R16" s="9">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X16" s="9">
         <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>206</v>
+        <v>250</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
@@ -3542,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
@@ -3554,37 +3545,37 @@
         <v>1</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ16" s="9">
         <v>29</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>249</v>
+        <v>122</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AN16" s="9">
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP16" s="9">
         <v>43</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>250</v>
+        <v>172</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
@@ -3593,87 +3584,87 @@
         <v>138</v>
       </c>
       <c r="AT16" s="9">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="AU16" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AV16" s="9">
+        <v>431</v>
+      </c>
+      <c r="AW16" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="AV16" s="9">
-        <v>428</v>
-      </c>
-      <c r="AW16" s="10" t="s">
+      <c r="AX16" s="9">
+        <v>1502</v>
+      </c>
+      <c r="AY16" s="10" t="s">
         <v>252</v>
-      </c>
-      <c r="AX16" s="9">
-        <v>1462</v>
-      </c>
-      <c r="AY16" s="10" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>255</v>
-      </c>
       <c r="C17" s="9">
-        <v>10335</v>
+        <v>10412</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F17" s="9">
         <v>2993</v>
       </c>
       <c r="G17" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H17" s="9">
+        <v>236</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="H17" s="9">
-        <v>235</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="J17" s="9">
+        <v>130</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="J17" s="9">
-        <v>129</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>4207</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>259</v>
-      </c>
-      <c r="L17" s="9">
-        <v>4153</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>260</v>
       </c>
       <c r="N17" s="9">
         <v>681</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="R17" s="9">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V17" s="9">
         <v>4</v>
@@ -3697,7 +3688,7 @@
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
@@ -3709,19 +3700,19 @@
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
@@ -3739,117 +3730,117 @@
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>235</v>
+        <v>193</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>206</v>
+        <v>250</v>
       </c>
       <c r="AT17" s="9">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="AU17" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="AV17" s="9">
+        <v>774</v>
+      </c>
+      <c r="AW17" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="AV17" s="9">
-        <v>765</v>
-      </c>
-      <c r="AW17" s="10" t="s">
+      <c r="AX17" s="9">
+        <v>500</v>
+      </c>
+      <c r="AY17" s="10" t="s">
         <v>264</v>
-      </c>
-      <c r="AX17" s="9">
-        <v>489</v>
-      </c>
-      <c r="AY17" s="10" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="C18" s="9">
+        <v>11207</v>
+      </c>
+      <c r="D18" s="9">
+        <v>0</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="9">
+        <v>2271</v>
+      </c>
+      <c r="G18" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="C18" s="9">
-        <v>11077</v>
-      </c>
-      <c r="D18" s="9">
-        <v>2</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="F18" s="9">
-        <v>2234</v>
-      </c>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="9">
+        <v>158</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="J18" s="9">
+        <v>52</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="L18" s="9">
+        <v>3888</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="H18" s="9">
-        <v>155</v>
-      </c>
-      <c r="I18" s="10" t="s">
+      <c r="N18" s="9">
+        <v>1668</v>
+      </c>
+      <c r="O18" s="10" t="s">
         <v>269</v>
-      </c>
-      <c r="J18" s="9">
-        <v>100</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="L18" s="9">
-        <v>3767</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="N18" s="9">
-        <v>1657</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>272</v>
       </c>
       <c r="P18" s="9">
         <v>1</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R18" s="9">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="T18" s="9">
         <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X18" s="9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AB18" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC18" s="10" t="s">
         <v>118</v>
@@ -3864,13 +3855,13 @@
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
@@ -3888,7 +3879,7 @@
         <v>2</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AP18" s="9">
         <v>38</v>
@@ -3900,188 +3891,188 @@
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AT18" s="9">
         <v>1</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AV18" s="9">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="AX18" s="9">
-        <v>1845</v>
+        <v>1843</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C19" s="9">
-        <v>13516</v>
+        <v>14895</v>
       </c>
       <c r="D19" s="9">
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F19" s="9">
-        <v>1524</v>
+        <v>1733</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="H19" s="9">
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>206</v>
+        <v>129</v>
       </c>
       <c r="J19" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L19" s="9">
-        <v>7293</v>
+        <v>8254</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="N19" s="9">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="P19" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="R19" s="9">
-        <v>1309</v>
+        <v>1470</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X19" s="9">
         <v>19</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD19" s="9">
         <v>3</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AF19" s="9">
         <v>0</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ19" s="9">
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>192</v>
+        <v>250</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP19" s="9">
         <v>61</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AT19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU19" s="10" t="s">
         <v>118</v>
       </c>
       <c r="AV19" s="9">
-        <v>759</v>
+        <v>798</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="AX19" s="9">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C20" s="9">
         <v>1119</v>
@@ -4096,7 +4087,7 @@
         <v>169</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
@@ -4105,88 +4096,88 @@
         <v>122</v>
       </c>
       <c r="J20" s="9">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="L20" s="9">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="N20" s="9">
         <v>50</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="P20" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>239</v>
+        <v>122</v>
       </c>
       <c r="R20" s="9">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>293</v>
+        <v>172</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH20" s="9">
         <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ20" s="9">
         <v>7</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>239</v>
+        <v>290</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
@@ -4204,13 +4195,13 @@
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="AT20" s="9">
         <v>11</v>
@@ -4222,42 +4213,42 @@
         <v>43</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="AX20" s="9">
         <v>199</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C21" s="9">
-        <v>2582</v>
+        <v>2600</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F21" s="9">
         <v>420</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="H21" s="9">
         <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="J21" s="9">
         <v>2</v>
@@ -4266,46 +4257,46 @@
         <v>106</v>
       </c>
       <c r="L21" s="9">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4317,49 +4308,49 @@
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP21" s="9">
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
@@ -4368,78 +4359,78 @@
         <v>139</v>
       </c>
       <c r="AT21" s="9">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="AX21" s="9">
         <v>864</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C22" s="12">
-        <v>130015</v>
+        <v>133133</v>
       </c>
       <c r="D22" s="12">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>26420</v>
+        <v>26935</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1486</v>
+        <v>1483</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2257</v>
+        <v>2206</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>52295</v>
+        <v>54514</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12522</v>
+        <v>12507</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>9804</v>
+        <v>10067</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4448,52 +4439,52 @@
         <v>98</v>
       </c>
       <c r="U22" s="13" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="W22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="Y22" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Z22" s="12">
         <v>26</v>
       </c>
       <c r="AA22" s="13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AD22" s="12">
         <v>93</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="AF22" s="12">
         <v>1</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AH22" s="12">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ22" s="12">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="AK22" s="13" t="s">
         <v>119</v>
@@ -4505,37 +4496,37 @@
         <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AP22" s="12">
-        <v>707</v>
+        <v>722</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AR22" s="12">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AT22" s="12">
-        <v>1056</v>
+        <v>1048</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AV22" s="12">
-        <v>6263</v>
+        <v>6349</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>15842</v>
+        <v>15929</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>126</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 11/09/2026  7:33:49,24
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="308">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 10 Sep 2026, 08.07</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 11 Sep 2026, 07.31</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,598 +334,601 @@
     <t>0,08</t>
   </si>
   <si>
+    <t>19,98</t>
+  </si>
+  <si>
+    <t>1,07</t>
+  </si>
+  <si>
+    <t>1,57</t>
+  </si>
+  <si>
+    <t>42,06</t>
+  </si>
+  <si>
+    <t>9,07</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>7,62</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>4,74</t>
+  </si>
+  <si>
+    <t>11,57</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>19,16</t>
+  </si>
+  <si>
+    <t>0,93</t>
+  </si>
+  <si>
+    <t>0,81</t>
+  </si>
+  <si>
+    <t>47,58</t>
+  </si>
+  <si>
+    <t>4,25</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,49</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>2,39</t>
+  </si>
+  <si>
+    <t>3,64</t>
+  </si>
+  <si>
+    <t>15,29</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,75</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>0,55</t>
+  </si>
+  <si>
+    <t>27,32</t>
+  </si>
+  <si>
+    <t>30,06</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>4,6</t>
+  </si>
+  <si>
+    <t>15,7</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>15,64</t>
+  </si>
+  <si>
+    <t>1,81</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>51,7</t>
+  </si>
+  <si>
+    <t>7,89</t>
+  </si>
+  <si>
+    <t>10,29</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>0,67</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>6,66</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>24,36</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>7,27</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>12,12</t>
+  </si>
+  <si>
+    <t>7,09</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>1,85</t>
+  </si>
+  <si>
+    <t>2,06</t>
+  </si>
+  <si>
+    <t>8,83</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,39</t>
+  </si>
+  <si>
+    <t>1,74</t>
+  </si>
+  <si>
+    <t>50,74</t>
+  </si>
+  <si>
+    <t>3,42</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>12,11</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>2,89</t>
+  </si>
+  <si>
+    <t>9,65</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>17,7</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>0,87</t>
+  </si>
+  <si>
+    <t>43,95</t>
+  </si>
+  <si>
+    <t>12,15</t>
+  </si>
+  <si>
+    <t>6,92</t>
+  </si>
+  <si>
+    <t>0,43</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>6,32</t>
+  </si>
+  <si>
+    <t>9,12</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>17,77</t>
+  </si>
+  <si>
+    <t>0,61</t>
+  </si>
+  <si>
+    <t>1,42</t>
+  </si>
+  <si>
+    <t>43,57</t>
+  </si>
+  <si>
+    <t>16,3</t>
+  </si>
+  <si>
+    <t>6,15</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>4,29</t>
+  </si>
+  <si>
+    <t>6,9</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,46</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>29,44</t>
+  </si>
+  <si>
+    <t>17,68</t>
+  </si>
+  <si>
+    <t>6,46</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>7,41</t>
+  </si>
+  <si>
+    <t>13,9</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,29</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>31,6</t>
+  </si>
+  <si>
+    <t>1,73</t>
+  </si>
+  <si>
+    <t>5,91</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>8,27</t>
+  </si>
+  <si>
+    <t>20,18</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,48</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>34,59</t>
+  </si>
+  <si>
+    <t>4,89</t>
+  </si>
+  <si>
+    <t>5,16</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>7,95</t>
+  </si>
+  <si>
+    <t>27,45</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>28,58</t>
+  </si>
+  <si>
+    <t>2,21</t>
+  </si>
+  <si>
+    <t>1,21</t>
+  </si>
+  <si>
+    <t>40,77</t>
+  </si>
+  <si>
+    <t>6,49</t>
+  </si>
+  <si>
+    <t>4,42</t>
+  </si>
+  <si>
+    <t>2,58</t>
+  </si>
+  <si>
+    <t>7,45</t>
+  </si>
+  <si>
+    <t>4,77</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
     <t>20,23</t>
   </si>
   <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>1,66</t>
-  </si>
-  <si>
-    <t>40,95</t>
-  </si>
-  <si>
-    <t>9,39</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>7,56</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>4,77</t>
-  </si>
-  <si>
-    <t>11,96</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>19,18</t>
-  </si>
-  <si>
-    <t>0,94</t>
-  </si>
-  <si>
-    <t>0,9</t>
-  </si>
-  <si>
-    <t>47,73</t>
-  </si>
-  <si>
-    <t>4,17</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,49</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>2,56</t>
-  </si>
-  <si>
-    <t>3,53</t>
-  </si>
-  <si>
-    <t>15,27</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,75</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>27,29</t>
-  </si>
-  <si>
-    <t>30,04</t>
-  </si>
-  <si>
-    <t>6,48</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>4,61</t>
-  </si>
-  <si>
-    <t>15,73</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>15,91</t>
-  </si>
-  <si>
-    <t>1,87</t>
-  </si>
-  <si>
-    <t>50,69</t>
-  </si>
-  <si>
-    <t>8,26</t>
-  </si>
-  <si>
-    <t>10,34</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>0,67</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>3,68</t>
-  </si>
-  <si>
-    <t>6,83</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>24,37</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>7,16</t>
-  </si>
-  <si>
-    <t>33,91</t>
-  </si>
-  <si>
-    <t>12,21</t>
-  </si>
-  <si>
-    <t>7,12</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>1,84</t>
-  </si>
-  <si>
-    <t>2,07</t>
-  </si>
-  <si>
-    <t>8,88</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>16,3</t>
-  </si>
-  <si>
-    <t>1,83</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>49,82</t>
-  </si>
-  <si>
-    <t>3,6</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>2,87</t>
-  </si>
-  <si>
-    <t>10,17</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>18,13</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>0,91</t>
-  </si>
-  <si>
-    <t>41,87</t>
-  </si>
-  <si>
-    <t>12,7</t>
-  </si>
-  <si>
-    <t>7,23</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>1,05</t>
-  </si>
-  <si>
-    <t>6,55</t>
-  </si>
-  <si>
-    <t>9,53</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,65</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>1,41</t>
-  </si>
-  <si>
-    <t>43,31</t>
-  </si>
-  <si>
-    <t>16,49</t>
-  </si>
-  <si>
-    <t>6,16</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>4,34</t>
-  </si>
-  <si>
-    <t>6,99</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,54</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>29,22</t>
-  </si>
-  <si>
-    <t>17,91</t>
-  </si>
-  <si>
-    <t>6,1</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>7,38</t>
-  </si>
-  <si>
-    <t>14,18</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,4</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>31,38</t>
-  </si>
-  <si>
-    <t>1,75</t>
-  </si>
-  <si>
-    <t>5,84</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>8,3</t>
-  </si>
-  <si>
-    <t>20,29</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,49</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>34,26</t>
-  </si>
-  <si>
-    <t>4,69</t>
-  </si>
-  <si>
-    <t>5,1</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>7,99</t>
-  </si>
-  <si>
-    <t>27,86</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
+    <t>1,4</t>
+  </si>
+  <si>
+    <t>35,78</t>
+  </si>
+  <si>
+    <t>14,43</t>
+  </si>
+  <si>
+    <t>6,57</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>4,1</t>
+  </si>
+  <si>
+    <t>16,38</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>11,5</t>
+  </si>
+  <si>
+    <t>58,15</t>
+  </si>
+  <si>
+    <t>9,69</t>
+  </si>
+  <si>
+    <t>9,92</t>
+  </si>
+  <si>
+    <t>5,19</t>
+  </si>
+  <si>
+    <t>4,8</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>15,02</t>
+  </si>
+  <si>
+    <t>0,53</t>
+  </si>
+  <si>
+    <t>2,22</t>
+  </si>
+  <si>
+    <t>35,38</t>
+  </si>
+  <si>
+    <t>4,44</t>
+  </si>
+  <si>
+    <t>15,2</t>
+  </si>
+  <si>
+    <t>1,6</t>
+  </si>
+  <si>
+    <t>1,16</t>
+  </si>
+  <si>
+    <t>3,82</t>
+  </si>
+  <si>
+    <t>17,69</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,17</t>
+  </si>
+  <si>
+    <t>5,72</t>
+  </si>
+  <si>
+    <t>30,41</t>
+  </si>
+  <si>
+    <t>3,92</t>
   </si>
   <si>
     <t>0,31</t>
   </si>
   <si>
-    <t>28,75</t>
-  </si>
-  <si>
-    <t>2,27</t>
-  </si>
-  <si>
-    <t>1,25</t>
-  </si>
-  <si>
-    <t>40,41</t>
-  </si>
-  <si>
-    <t>6,54</t>
-  </si>
-  <si>
-    <t>4,4</t>
-  </si>
-  <si>
-    <t>2,62</t>
-  </si>
-  <si>
-    <t>7,43</t>
-  </si>
-  <si>
-    <t>4,8</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>20,26</t>
-  </si>
-  <si>
-    <t>34,69</t>
-  </si>
-  <si>
-    <t>14,88</t>
-  </si>
-  <si>
-    <t>6,6</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>4,12</t>
-  </si>
-  <si>
-    <t>16,45</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,63</t>
-  </si>
-  <si>
-    <t>55,41</t>
-  </si>
-  <si>
-    <t>11,17</t>
-  </si>
-  <si>
-    <t>9,87</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>5,36</t>
-  </si>
-  <si>
-    <t>5,7</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,1</t>
-  </si>
-  <si>
-    <t>2,23</t>
-  </si>
-  <si>
-    <t>35,21</t>
-  </si>
-  <si>
-    <t>4,47</t>
-  </si>
-  <si>
-    <t>15,28</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>1,61</t>
-  </si>
-  <si>
-    <t>3,84</t>
-  </si>
-  <si>
-    <t>17,78</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,15</t>
-  </si>
-  <si>
-    <t>5,77</t>
-  </si>
-  <si>
-    <t>30,42</t>
-  </si>
-  <si>
-    <t>3,92</t>
-  </si>
-  <si>
-    <t>3,04</t>
+    <t>3,03</t>
   </si>
   <si>
     <t>0,69</t>
   </si>
   <si>
-    <t>1,81</t>
+    <t>1,92</t>
   </si>
   <si>
     <t>3,69</t>
   </si>
   <si>
-    <t>33,23</t>
+    <t>33,18</t>
   </si>
   <si>
     <t/>
@@ -1905,52 +1908,52 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>133133</v>
+        <v>137675</v>
       </c>
       <c r="D6" s="6">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>26935</v>
+        <v>27506</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1483</v>
+        <v>1477</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2206</v>
+        <v>2167</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>54514</v>
+        <v>57903</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12507</v>
+        <v>12494</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>10067</v>
+        <v>10494</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1968,7 +1971,7 @@
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
@@ -1980,31 +1983,31 @@
         <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD6" s="6">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="AE6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="AF6" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AG6" s="7" t="s">
         <v>118</v>
       </c>
       <c r="AH6" s="6">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AI6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="AJ6" s="6">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="AK6" s="7" t="s">
         <v>119</v>
@@ -2016,19 +2019,19 @@
         <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AP6" s="6">
-        <v>722</v>
+        <v>739</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AR6" s="6">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>123</v>
@@ -2040,13 +2043,13 @@
         <v>124</v>
       </c>
       <c r="AV6" s="6">
-        <v>6349</v>
+        <v>6519</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>15929</v>
+        <v>15934</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>126</v>
@@ -2060,7 +2063,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>7848</v>
+        <v>7944</v>
       </c>
       <c r="D7" s="9">
         <v>8</v>
@@ -2069,7 +2072,7 @@
         <v>129</v>
       </c>
       <c r="F7" s="9">
-        <v>1505</v>
+        <v>1522</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>130</v>
@@ -2081,19 +2084,19 @@
         <v>131</v>
       </c>
       <c r="J7" s="9">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>132</v>
       </c>
       <c r="L7" s="9">
-        <v>3746</v>
+        <v>3780</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>133</v>
       </c>
       <c r="N7" s="9">
-        <v>327</v>
+        <v>338</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>134</v>
@@ -2105,7 +2108,7 @@
         <v>135</v>
       </c>
       <c r="R7" s="9">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="S7" s="10" t="s">
         <v>136</v>
@@ -2123,7 +2126,7 @@
         <v>118</v>
       </c>
       <c r="X7" s="9">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Y7" s="10" t="s">
         <v>137</v>
@@ -2135,16 +2138,16 @@
         <v>120</v>
       </c>
       <c r="AB7" s="9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AD7" s="9">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
@@ -2159,10 +2162,10 @@
         <v>118</v>
       </c>
       <c r="AJ7" s="9">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
@@ -2171,99 +2174,99 @@
         <v>115</v>
       </c>
       <c r="AN7" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO7" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="AP7" s="9">
+        <v>38</v>
+      </c>
+      <c r="AQ7" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="AP7" s="9">
-        <v>31</v>
-      </c>
-      <c r="AQ7" s="10" t="s">
+      <c r="AR7" s="9">
+        <v>7</v>
+      </c>
+      <c r="AS7" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="AT7" s="9">
+        <v>190</v>
+      </c>
+      <c r="AU7" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="AR7" s="9">
-        <v>3</v>
-      </c>
-      <c r="AS7" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="AT7" s="9">
-        <v>201</v>
-      </c>
-      <c r="AU7" s="10" t="s">
+      <c r="AV7" s="9">
+        <v>289</v>
+      </c>
+      <c r="AW7" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="AV7" s="9">
-        <v>277</v>
-      </c>
-      <c r="AW7" s="10" t="s">
+      <c r="AX7" s="9">
+        <v>1215</v>
+      </c>
+      <c r="AY7" s="10" t="s">
         <v>142</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>1198</v>
-      </c>
-      <c r="AY7" s="10" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="9">
+        <v>3433</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F8" s="9">
+        <v>472</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>145</v>
-      </c>
-      <c r="C8" s="9">
-        <v>3426</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F8" s="9">
-        <v>471</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>146</v>
       </c>
       <c r="H8" s="9">
         <v>17</v>
       </c>
       <c r="I8" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J8" s="9">
+        <v>19</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="J8" s="9">
-        <v>22</v>
-      </c>
-      <c r="K8" s="10" t="s">
+      <c r="L8" s="9">
+        <v>938</v>
+      </c>
+      <c r="M8" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="L8" s="9">
-        <v>935</v>
-      </c>
-      <c r="M8" s="10" t="s">
+      <c r="N8" s="9">
+        <v>1032</v>
+      </c>
+      <c r="O8" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="N8" s="9">
-        <v>1029</v>
-      </c>
-      <c r="O8" s="10" t="s">
+      <c r="P8" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R8" s="9">
+        <v>225</v>
+      </c>
+      <c r="S8" s="10" t="s">
         <v>150</v>
-      </c>
-      <c r="P8" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R8" s="9">
-        <v>222</v>
-      </c>
-      <c r="S8" s="10" t="s">
-        <v>151</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
@@ -2281,7 +2284,7 @@
         <v>7</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
@@ -2317,7 +2320,7 @@
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>153</v>
+        <v>116</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
@@ -2335,90 +2338,90 @@
         <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="AT8" s="9">
         <v>2</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="AV8" s="9">
         <v>158</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AX8" s="9">
         <v>539</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="C9" s="9">
+        <v>10773</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" s="9">
+        <v>1685</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>157</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="9">
-        <v>10406</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1656</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="H9" s="9">
         <v>195</v>
       </c>
       <c r="I9" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="J9" s="9">
+        <v>19</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="L9" s="9">
+        <v>5570</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="J9" s="9">
-        <v>21</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="L9" s="9">
-        <v>5275</v>
-      </c>
-      <c r="M9" s="10" t="s">
+      <c r="N9" s="9">
+        <v>850</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="N9" s="9">
-        <v>860</v>
-      </c>
-      <c r="O9" s="10" t="s">
+      <c r="P9" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R9" s="9">
+        <v>1109</v>
+      </c>
+      <c r="S9" s="10" t="s">
         <v>162</v>
-      </c>
-      <c r="P9" s="9">
-        <v>3</v>
-      </c>
-      <c r="Q9" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="R9" s="9">
-        <v>1076</v>
-      </c>
-      <c r="S9" s="10" t="s">
-        <v>163</v>
       </c>
       <c r="T9" s="9">
         <v>1</v>
@@ -2436,7 +2439,7 @@
         <v>38</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
@@ -2454,7 +2457,7 @@
         <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
@@ -2469,28 +2472,28 @@
         <v>118</v>
       </c>
       <c r="AJ9" s="9">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="AK9" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="AL9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AN9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AP9" s="9">
+        <v>108</v>
+      </c>
+      <c r="AQ9" s="10" t="s">
         <v>165</v>
-      </c>
-      <c r="AL9" s="9">
-        <v>0</v>
-      </c>
-      <c r="AM9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AN9" s="9">
-        <v>0</v>
-      </c>
-      <c r="AO9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AP9" s="9">
-        <v>102</v>
-      </c>
-      <c r="AQ9" s="10" t="s">
-        <v>166</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
@@ -2499,81 +2502,81 @@
         <v>117</v>
       </c>
       <c r="AT9" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="AV9" s="9">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="AW9" s="10" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="AX9" s="9">
-        <v>711</v>
+        <v>718</v>
       </c>
       <c r="AY9" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="C10" s="9">
+        <v>21731</v>
+      </c>
+      <c r="D10" s="9">
+        <v>44</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="9">
+        <v>5293</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="C10" s="9">
-        <v>21580</v>
-      </c>
-      <c r="D10" s="9">
-        <v>43</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="F10" s="9">
-        <v>5260</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>171</v>
       </c>
       <c r="H10" s="9">
         <v>172</v>
       </c>
       <c r="I10" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="J10" s="9">
+        <v>1579</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="L10" s="9">
+        <v>7389</v>
+      </c>
+      <c r="M10" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="J10" s="9">
-        <v>1545</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="N10" s="9">
+        <v>2633</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="L10" s="9">
-        <v>7317</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="P10" s="9">
+        <v>145</v>
+      </c>
+      <c r="Q10" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="R10" s="9">
+        <v>1540</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>174</v>
-      </c>
-      <c r="N10" s="9">
-        <v>2634</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="P10" s="9">
-        <v>144</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="R10" s="9">
-        <v>1536</v>
-      </c>
-      <c r="S10" s="10" t="s">
-        <v>176</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
@@ -2591,7 +2594,7 @@
         <v>14</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="Z10" s="9">
         <v>2</v>
@@ -2603,7 +2606,7 @@
         <v>9</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="AD10" s="9">
         <v>17</v>
@@ -2621,13 +2624,13 @@
         <v>9</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="AJ10" s="9">
         <v>13</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
@@ -2639,7 +2642,7 @@
         <v>53</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>177</v>
+        <v>119</v>
       </c>
       <c r="AP10" s="9">
         <v>31</v>
@@ -2651,90 +2654,90 @@
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>178</v>
+        <v>121</v>
       </c>
       <c r="AT10" s="9">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="AV10" s="9">
         <v>447</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AX10" s="9">
-        <v>1917</v>
+        <v>1919</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C11" s="9">
+        <v>16408</v>
+      </c>
+      <c r="D11" s="9">
+        <v>16</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F11" s="9">
+        <v>2689</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="9">
+        <v>285</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="J11" s="9">
+        <v>153</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="L11" s="9">
+        <v>8325</v>
+      </c>
+      <c r="M11" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="C11" s="9">
-        <v>15619</v>
-      </c>
-      <c r="D11" s="9">
-        <v>13</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="F11" s="9">
-        <v>2546</v>
-      </c>
-      <c r="G11" s="10" t="s">
+      <c r="N11" s="9">
+        <v>561</v>
+      </c>
+      <c r="O11" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="H11" s="9">
-        <v>286</v>
-      </c>
-      <c r="I11" s="10" t="s">
+      <c r="P11" s="9">
+        <v>36</v>
+      </c>
+      <c r="Q11" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="J11" s="9">
-        <v>155</v>
-      </c>
-      <c r="K11" s="10" t="s">
+      <c r="R11" s="9">
+        <v>1987</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="L11" s="9">
-        <v>7782</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="N11" s="9">
-        <v>563</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="P11" s="9">
-        <v>35</v>
-      </c>
-      <c r="Q11" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="R11" s="9">
-        <v>1907</v>
-      </c>
-      <c r="S11" s="10" t="s">
-        <v>175</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
@@ -2743,10 +2746,10 @@
         <v>120</v>
       </c>
       <c r="X11" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
@@ -2764,7 +2767,7 @@
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>135</v>
+        <v>187</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
@@ -2773,7 +2776,7 @@
         <v>118</v>
       </c>
       <c r="AH11" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AI11" s="10" t="s">
         <v>120</v>
@@ -2782,7 +2785,7 @@
         <v>40</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>191</v>
+        <v>119</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
@@ -2797,10 +2800,10 @@
         <v>117</v>
       </c>
       <c r="AP11" s="9">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="AR11" s="9">
         <v>13</v>
@@ -2809,33 +2812,33 @@
         <v>106</v>
       </c>
       <c r="AT11" s="9">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="AV11" s="9">
-        <v>449</v>
+        <v>474</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="AX11" s="9">
-        <v>1588</v>
+        <v>1583</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C12" s="9">
-        <v>5741</v>
+        <v>6000</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
@@ -2844,34 +2847,34 @@
         <v>118</v>
       </c>
       <c r="F12" s="9">
-        <v>1041</v>
+        <v>1062</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="H12" s="9">
         <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J12" s="9">
         <v>52</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="L12" s="9">
-        <v>2404</v>
+        <v>2637</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="P12" s="9">
         <v>2</v>
@@ -2883,7 +2886,7 @@
         <v>415</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
@@ -2901,7 +2904,7 @@
         <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
@@ -2919,7 +2922,7 @@
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>205</v>
+        <v>112</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
@@ -2934,10 +2937,10 @@
         <v>118</v>
       </c>
       <c r="AJ12" s="9">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
@@ -2955,7 +2958,7 @@
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>207</v>
+        <v>165</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
@@ -2970,63 +2973,63 @@
         <v>129</v>
       </c>
       <c r="AV12" s="9">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C13" s="9">
-        <v>5020</v>
+        <v>5086</v>
       </c>
       <c r="D13" s="9">
         <v>6</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="F13" s="9">
-        <v>886</v>
+        <v>904</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="H13" s="9">
         <v>31</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="J13" s="9">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="L13" s="9">
-        <v>2174</v>
+        <v>2216</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="N13" s="9">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="P13" s="9">
         <v>5</v>
@@ -3035,10 +3038,10 @@
         <v>129</v>
       </c>
       <c r="R13" s="9">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
@@ -3050,7 +3053,7 @@
         <v>3</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
@@ -3074,7 +3077,7 @@
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>116</v>
+        <v>213</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
@@ -3086,19 +3089,19 @@
         <v>2</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="AJ13" s="9">
         <v>33</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AN13" s="9">
         <v>5</v>
@@ -3110,78 +3113,78 @@
         <v>38</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AR13" s="9">
         <v>23</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="AT13" s="9">
         <v>13</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>191</v>
+        <v>217</v>
       </c>
       <c r="AV13" s="9">
         <v>218</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="AX13" s="9">
         <v>351</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C14" s="9">
+        <v>5044</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1133</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>222</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="C14" s="9">
-        <v>4986</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1124</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="J14" s="9">
         <v>18</v>
       </c>
       <c r="K14" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="L14" s="9">
+        <v>1485</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="N14" s="9">
+        <v>892</v>
+      </c>
+      <c r="O14" s="10" t="s">
         <v>225</v>
-      </c>
-      <c r="L14" s="9">
-        <v>1457</v>
-      </c>
-      <c r="M14" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="N14" s="9">
-        <v>893</v>
-      </c>
-      <c r="O14" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
@@ -3190,16 +3193,16 @@
         <v>117</v>
       </c>
       <c r="R14" s="9">
-        <v>304</v>
+        <v>326</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
@@ -3211,7 +3214,7 @@
         <v>9</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>112</v>
+        <v>159</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
@@ -3247,7 +3250,7 @@
         <v>20</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>140</v>
+        <v>227</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
@@ -3265,7 +3268,7 @@
         <v>38</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
@@ -3277,84 +3280,84 @@
         <v>17</v>
       </c>
       <c r="AU14" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="AV14" s="9">
+        <v>374</v>
+      </c>
+      <c r="AW14" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="AV14" s="9">
-        <v>368</v>
-      </c>
-      <c r="AW14" s="10" t="s">
+      <c r="AX14" s="9">
+        <v>701</v>
+      </c>
+      <c r="AY14" s="10" t="s">
         <v>230</v>
-      </c>
-      <c r="AX14" s="9">
-        <v>707</v>
-      </c>
-      <c r="AY14" s="10" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="9">
+        <v>12956</v>
+      </c>
+      <c r="D15" s="9">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" s="9">
+        <v>3924</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>233</v>
-      </c>
-      <c r="C15" s="9">
-        <v>12883</v>
-      </c>
-      <c r="D15" s="9">
-        <v>0</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="9">
-        <v>3917</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>234</v>
       </c>
       <c r="H15" s="9">
         <v>55</v>
       </c>
       <c r="I15" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="J15" s="9">
+        <v>27</v>
+      </c>
+      <c r="K15" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="J15" s="9">
-        <v>29</v>
-      </c>
-      <c r="K15" s="10" t="s">
+      <c r="L15" s="9">
+        <v>4094</v>
+      </c>
+      <c r="M15" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="L15" s="9">
-        <v>4043</v>
-      </c>
-      <c r="M15" s="10" t="s">
+      <c r="N15" s="9">
+        <v>224</v>
+      </c>
+      <c r="O15" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="N15" s="9">
-        <v>226</v>
-      </c>
-      <c r="O15" s="10" t="s">
+      <c r="P15" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R15" s="9">
+        <v>766</v>
+      </c>
+      <c r="S15" s="10" t="s">
         <v>238</v>
-      </c>
-      <c r="P15" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R15" s="9">
-        <v>753</v>
-      </c>
-      <c r="S15" s="10" t="s">
-        <v>239</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
@@ -3366,7 +3369,7 @@
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
@@ -3420,7 +3423,7 @@
         <v>82</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>148</v>
+        <v>195</v>
       </c>
       <c r="AR15" s="9">
         <v>18</v>
@@ -3429,81 +3432,81 @@
         <v>135</v>
       </c>
       <c r="AT15" s="9">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="AV15" s="9">
-        <v>1069</v>
+        <v>1071</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AX15" s="9">
         <v>2614</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="C16" s="9">
+        <v>5482</v>
+      </c>
+      <c r="D16" s="9">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F16" s="9">
+        <v>958</v>
+      </c>
+      <c r="G16" s="10" t="s">
         <v>244</v>
-      </c>
-      <c r="C16" s="9">
-        <v>5391</v>
-      </c>
-      <c r="D16" s="9">
-        <v>1</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F16" s="9">
-        <v>943</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>245</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="J16" s="9">
+        <v>2</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="L16" s="9">
+        <v>1896</v>
+      </c>
+      <c r="M16" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="J16" s="9">
-        <v>3</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="L16" s="9">
-        <v>1847</v>
-      </c>
-      <c r="M16" s="10" t="s">
+      <c r="N16" s="9">
+        <v>268</v>
+      </c>
+      <c r="O16" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="N16" s="9">
-        <v>253</v>
-      </c>
-      <c r="O16" s="10" t="s">
+      <c r="P16" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R16" s="9">
+        <v>283</v>
+      </c>
+      <c r="S16" s="10" t="s">
         <v>248</v>
-      </c>
-      <c r="P16" s="9">
-        <v>1</v>
-      </c>
-      <c r="Q16" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="R16" s="9">
-        <v>275</v>
-      </c>
-      <c r="S16" s="10" t="s">
-        <v>249</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
@@ -3521,7 +3524,7 @@
         <v>6</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>250</v>
+        <v>138</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
@@ -3554,10 +3557,10 @@
         <v>118</v>
       </c>
       <c r="AJ16" s="9">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3572,93 +3575,93 @@
         <v>118</v>
       </c>
       <c r="AP16" s="9">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>172</v>
+        <v>249</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="AT16" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="AV16" s="9">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="AW16" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="AX16" s="9">
+        <v>1505</v>
+      </c>
+      <c r="AY16" s="10" t="s">
         <v>251</v>
-      </c>
-      <c r="AX16" s="9">
-        <v>1502</v>
-      </c>
-      <c r="AY16" s="10" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>254</v>
-      </c>
       <c r="C17" s="9">
-        <v>10412</v>
+        <v>10499</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="F17" s="9">
+        <v>3001</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="F17" s="9">
-        <v>2993</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="H17" s="9">
+        <v>232</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="H17" s="9">
-        <v>236</v>
-      </c>
-      <c r="I17" s="10" t="s">
+      <c r="J17" s="9">
+        <v>127</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="J17" s="9">
-        <v>130</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>4280</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="L17" s="9">
-        <v>4207</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>259</v>
       </c>
       <c r="N17" s="9">
         <v>681</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="R17" s="9">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
@@ -3670,7 +3673,7 @@
         <v>4</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="X17" s="9">
         <v>8</v>
@@ -3682,7 +3685,7 @@
         <v>4</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
@@ -3694,7 +3697,7 @@
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
@@ -3712,7 +3715,7 @@
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>153</v>
+        <v>116</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
@@ -3730,87 +3733,87 @@
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>193</v>
+        <v>234</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>250</v>
+        <v>129</v>
       </c>
       <c r="AT17" s="9">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AU17" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="AV17" s="9">
+        <v>782</v>
+      </c>
+      <c r="AW17" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="AV17" s="9">
-        <v>774</v>
-      </c>
-      <c r="AW17" s="10" t="s">
+      <c r="AX17" s="9">
+        <v>501</v>
+      </c>
+      <c r="AY17" s="10" t="s">
         <v>263</v>
-      </c>
-      <c r="AX17" s="9">
-        <v>500</v>
-      </c>
-      <c r="AY17" s="10" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="C18" s="9">
+        <v>11279</v>
+      </c>
+      <c r="D18" s="9">
+        <v>0</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="9">
+        <v>2282</v>
+      </c>
+      <c r="G18" s="10" t="s">
         <v>266</v>
-      </c>
-      <c r="C18" s="9">
-        <v>11207</v>
-      </c>
-      <c r="D18" s="9">
-        <v>0</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F18" s="9">
-        <v>2271</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>267</v>
       </c>
       <c r="H18" s="9">
         <v>158</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>214</v>
+        <v>267</v>
       </c>
       <c r="J18" s="9">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>219</v>
+        <v>118</v>
       </c>
       <c r="L18" s="9">
-        <v>3888</v>
+        <v>4036</v>
       </c>
       <c r="M18" s="10" t="s">
         <v>268</v>
       </c>
       <c r="N18" s="9">
-        <v>1668</v>
+        <v>1627</v>
       </c>
       <c r="O18" s="10" t="s">
         <v>269</v>
       </c>
       <c r="P18" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="R18" s="9">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="S18" s="10" t="s">
         <v>270</v>
@@ -3846,10 +3849,10 @@
         <v>118</v>
       </c>
       <c r="AD18" s="9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
@@ -3876,28 +3879,28 @@
         <v>123</v>
       </c>
       <c r="AN18" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AP18" s="9">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>229</v>
+        <v>163</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>153</v>
+        <v>116</v>
       </c>
       <c r="AT18" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AV18" s="9">
         <v>462</v>
@@ -3906,7 +3909,7 @@
         <v>272</v>
       </c>
       <c r="AX18" s="9">
-        <v>1843</v>
+        <v>1847</v>
       </c>
       <c r="AY18" s="10" t="s">
         <v>273</v>
@@ -3920,7 +3923,7 @@
         <v>275</v>
       </c>
       <c r="C19" s="9">
-        <v>14895</v>
+        <v>17311</v>
       </c>
       <c r="D19" s="9">
         <v>1</v>
@@ -3929,7 +3932,7 @@
         <v>115</v>
       </c>
       <c r="F19" s="9">
-        <v>1733</v>
+        <v>1991</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>276</v>
@@ -3938,22 +3941,22 @@
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J19" s="9">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="L19" s="9">
-        <v>8254</v>
+        <v>10067</v>
       </c>
       <c r="M19" s="10" t="s">
         <v>277</v>
       </c>
       <c r="N19" s="9">
-        <v>1664</v>
+        <v>1678</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>278</v>
@@ -3965,7 +3968,7 @@
         <v>115</v>
       </c>
       <c r="R19" s="9">
-        <v>1470</v>
+        <v>1718</v>
       </c>
       <c r="S19" s="10" t="s">
         <v>279</v>
@@ -3983,10 +3986,10 @@
         <v>118</v>
       </c>
       <c r="X19" s="9">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>138</v>
+        <v>206</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
@@ -4001,16 +4004,16 @@
         <v>118</v>
       </c>
       <c r="AD19" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AF19" s="9">
         <v>3</v>
       </c>
-      <c r="AE19" s="10" t="s">
+      <c r="AG19" s="10" t="s">
         <v>117</v>
-      </c>
-      <c r="AF19" s="9">
-        <v>0</v>
-      </c>
-      <c r="AG19" s="10" t="s">
-        <v>118</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
@@ -4022,7 +4025,7 @@
         <v>16</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>250</v>
+        <v>123</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
@@ -4037,10 +4040,10 @@
         <v>118</v>
       </c>
       <c r="AP19" s="9">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>280</v>
+        <v>223</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
@@ -4055,27 +4058,27 @@
         <v>118</v>
       </c>
       <c r="AV19" s="9">
-        <v>798</v>
+        <v>898</v>
       </c>
       <c r="AW19" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="AX19" s="9">
+        <v>831</v>
+      </c>
+      <c r="AY19" s="10" t="s">
         <v>281</v>
-      </c>
-      <c r="AX19" s="9">
-        <v>849</v>
-      </c>
-      <c r="AY19" s="10" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>284</v>
-      </c>
       <c r="C20" s="9">
-        <v>1119</v>
+        <v>1125</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
@@ -4087,13 +4090,13 @@
         <v>169</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>122</v>
+        <v>285</v>
       </c>
       <c r="J20" s="9">
         <v>25</v>
@@ -4102,7 +4105,7 @@
         <v>286</v>
       </c>
       <c r="L20" s="9">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="M20" s="10" t="s">
         <v>287</v>
@@ -4117,7 +4120,7 @@
         <v>6</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>122</v>
+        <v>285</v>
       </c>
       <c r="R20" s="9">
         <v>171</v>
@@ -4141,7 +4144,7 @@
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>172</v>
+        <v>249</v>
       </c>
       <c r="Z20" s="9">
         <v>3</v>
@@ -4177,13 +4180,13 @@
         <v>7</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>290</v>
+        <v>188</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>112</v>
+        <v>159</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
@@ -4195,19 +4198,19 @@
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AR20" s="9">
         <v>4</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AT20" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>166</v>
+        <v>291</v>
       </c>
       <c r="AV20" s="9">
         <v>43</v>
@@ -4230,7 +4233,7 @@
         <v>295</v>
       </c>
       <c r="C21" s="9">
-        <v>2600</v>
+        <v>2604</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -4239,13 +4242,13 @@
         <v>118</v>
       </c>
       <c r="F21" s="9">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G21" s="10" t="s">
         <v>296</v>
       </c>
       <c r="H21" s="9">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>297</v>
@@ -4257,7 +4260,7 @@
         <v>106</v>
       </c>
       <c r="L21" s="9">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="M21" s="10" t="s">
         <v>298</v>
@@ -4272,13 +4275,13 @@
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>255</v>
+        <v>300</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
@@ -4296,7 +4299,7 @@
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
@@ -4332,7 +4335,7 @@
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
@@ -4350,87 +4353,87 @@
         <v>18</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="AT21" s="9">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="AV21" s="9">
         <v>96</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="AX21" s="9">
         <v>864</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C22" s="12">
-        <v>133133</v>
+        <v>137675</v>
       </c>
       <c r="D22" s="12">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>26935</v>
+        <v>27506</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1483</v>
+        <v>1477</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2206</v>
+        <v>2167</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>54514</v>
+        <v>57903</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12507</v>
+        <v>12494</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>10067</v>
+        <v>10494</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4448,7 +4451,7 @@
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
@@ -4460,31 +4463,31 @@
         <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD22" s="12">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="AE22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="AF22" s="12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AG22" s="13" t="s">
         <v>118</v>
       </c>
       <c r="AH22" s="12">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AI22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="AJ22" s="12">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="AK22" s="13" t="s">
         <v>119</v>
@@ -4496,19 +4499,19 @@
         <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AP22" s="12">
-        <v>722</v>
+        <v>739</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AR22" s="12">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>123</v>
@@ -4520,13 +4523,13 @@
         <v>124</v>
       </c>
       <c r="AV22" s="12">
-        <v>6349</v>
+        <v>6519</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>15929</v>
+        <v>15934</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>126</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 13/09/2026 14:37:22,03
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="307">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 11 Sep 2026, 07.31</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 13 Sep 2026, 14.36</t>
   </si>
   <si>
     <t>Kode</t>
@@ -331,508 +331,508 @@
     <t>LAMPUNG</t>
   </si>
   <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>19,8</t>
+  </si>
+  <si>
+    <t>1,02</t>
+  </si>
+  <si>
+    <t>1,43</t>
+  </si>
+  <si>
+    <t>43,36</t>
+  </si>
+  <si>
+    <t>8,65</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>7,77</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>19,98</t>
-  </si>
-  <si>
-    <t>1,07</t>
-  </si>
-  <si>
-    <t>1,57</t>
-  </si>
-  <si>
-    <t>42,06</t>
-  </si>
-  <si>
-    <t>9,07</t>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>4,69</t>
+  </si>
+  <si>
+    <t>11,07</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>19,16</t>
+  </si>
+  <si>
+    <t>0,93</t>
+  </si>
+  <si>
+    <t>0,81</t>
+  </si>
+  <si>
+    <t>47,6</t>
+  </si>
+  <si>
+    <t>4,25</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>4,49</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>2,38</t>
+  </si>
+  <si>
+    <t>3,65</t>
+  </si>
+  <si>
+    <t>15,31</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>13,72</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>0,55</t>
+  </si>
+  <si>
+    <t>27,3</t>
+  </si>
+  <si>
+    <t>30,13</t>
+  </si>
+  <si>
+    <t>6,54</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>4,59</t>
+  </si>
+  <si>
+    <t>15,67</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>15,51</t>
+  </si>
+  <si>
+    <t>1,71</t>
+  </si>
+  <si>
+    <t>52,77</t>
+  </si>
+  <si>
+    <t>7,63</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>10,08</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>0,97</t>
+  </si>
+  <si>
+    <t>3,61</t>
+  </si>
+  <si>
+    <t>6,47</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>24,71</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>7,02</t>
+  </si>
+  <si>
+    <t>34,49</t>
+  </si>
+  <si>
+    <t>11,86</t>
+  </si>
+  <si>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>7,2</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>1,81</t>
+  </si>
+  <si>
+    <t>2,02</t>
+  </si>
+  <si>
+    <t>8,55</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,6</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>51,11</t>
+  </si>
+  <si>
+    <t>3,37</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>12,01</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>2,84</t>
+  </si>
+  <si>
+    <t>9,47</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>17,68</t>
+  </si>
+  <si>
+    <t>0,87</t>
+  </si>
+  <si>
+    <t>43,95</t>
+  </si>
+  <si>
+    <t>12,15</t>
+  </si>
+  <si>
+    <t>6,92</t>
+  </si>
+  <si>
+    <t>0,43</t>
   </si>
   <si>
     <t>0,17</t>
   </si>
   <si>
-    <t>7,62</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>4,74</t>
-  </si>
-  <si>
-    <t>11,57</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>19,16</t>
-  </si>
-  <si>
-    <t>0,93</t>
-  </si>
-  <si>
-    <t>0,81</t>
-  </si>
-  <si>
-    <t>47,58</t>
-  </si>
-  <si>
-    <t>4,25</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,49</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>2,39</t>
-  </si>
-  <si>
-    <t>3,64</t>
-  </si>
-  <si>
-    <t>15,29</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,75</t>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>6,32</t>
+  </si>
+  <si>
+    <t>9,12</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>17,99</t>
+  </si>
+  <si>
+    <t>43,11</t>
+  </si>
+  <si>
+    <t>17,02</t>
+  </si>
+  <si>
+    <t>6,81</t>
+  </si>
+  <si>
+    <t>0,78</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>1,19</t>
   </si>
   <si>
     <t>0,5</t>
   </si>
   <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>27,32</t>
-  </si>
-  <si>
-    <t>30,06</t>
-  </si>
-  <si>
-    <t>6,55</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>4,6</t>
-  </si>
-  <si>
-    <t>15,7</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>15,64</t>
-  </si>
-  <si>
-    <t>1,81</t>
-  </si>
-  <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>51,7</t>
-  </si>
-  <si>
-    <t>7,89</t>
-  </si>
-  <si>
-    <t>10,29</t>
+    <t>4,31</t>
+  </si>
+  <si>
+    <t>6,66</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>22,2</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>31,04</t>
+  </si>
+  <si>
+    <t>17,3</t>
+  </si>
+  <si>
+    <t>6,26</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>7,33</t>
+  </si>
+  <si>
+    <t>13,45</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,21</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>32,12</t>
+  </si>
+  <si>
+    <t>1,5</t>
+  </si>
+  <si>
+    <t>5,9</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>8,2</t>
+  </si>
+  <si>
+    <t>20,04</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,33</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>35,07</t>
+  </si>
+  <si>
+    <t>5,03</t>
+  </si>
+  <si>
+    <t>5,17</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>7,85</t>
+  </si>
+  <si>
+    <t>27,17</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>28,57</t>
+  </si>
+  <si>
+    <t>2,21</t>
+  </si>
+  <si>
+    <t>1,24</t>
+  </si>
+  <si>
+    <t>40,77</t>
+  </si>
+  <si>
+    <t>6,48</t>
+  </si>
+  <si>
+    <t>4,42</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>2,57</t>
+  </si>
+  <si>
+    <t>7,45</t>
+  </si>
+  <si>
+    <t>4,77</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>20,22</t>
+  </si>
+  <si>
+    <t>1,4</t>
+  </si>
+  <si>
+    <t>35,8</t>
+  </si>
+  <si>
+    <t>14,42</t>
+  </si>
+  <si>
+    <t>6,58</t>
   </si>
   <si>
     <t>0,35</t>
   </si>
   <si>
-    <t>0,67</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>6,66</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>24,36</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>7,27</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>12,12</t>
-  </si>
-  <si>
-    <t>7,09</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>1,85</t>
-  </si>
-  <si>
-    <t>2,06</t>
-  </si>
-  <si>
-    <t>8,83</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>16,39</t>
-  </si>
-  <si>
-    <t>1,74</t>
-  </si>
-  <si>
-    <t>50,74</t>
-  </si>
-  <si>
-    <t>3,42</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>12,11</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>2,89</t>
-  </si>
-  <si>
-    <t>9,65</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>17,7</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>0,87</t>
-  </si>
-  <si>
-    <t>43,95</t>
-  </si>
-  <si>
-    <t>12,15</t>
-  </si>
-  <si>
-    <t>6,92</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>6,32</t>
-  </si>
-  <si>
-    <t>9,12</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>17,77</t>
-  </si>
-  <si>
-    <t>0,61</t>
-  </si>
-  <si>
-    <t>1,42</t>
-  </si>
-  <si>
-    <t>43,57</t>
-  </si>
-  <si>
-    <t>16,3</t>
-  </si>
-  <si>
-    <t>6,15</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>4,29</t>
-  </si>
-  <si>
-    <t>6,9</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,46</t>
-  </si>
-  <si>
-    <t>0,36</t>
-  </si>
-  <si>
-    <t>29,44</t>
-  </si>
-  <si>
-    <t>17,68</t>
-  </si>
-  <si>
-    <t>6,46</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>7,41</t>
-  </si>
-  <si>
-    <t>13,9</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,29</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>31,6</t>
-  </si>
-  <si>
-    <t>1,73</t>
-  </si>
-  <si>
-    <t>5,91</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>8,27</t>
-  </si>
-  <si>
-    <t>20,18</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,48</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>34,59</t>
-  </si>
-  <si>
-    <t>4,89</t>
-  </si>
-  <si>
-    <t>5,16</t>
-  </si>
-  <si>
-    <t>0,8</t>
-  </si>
-  <si>
-    <t>7,95</t>
-  </si>
-  <si>
-    <t>27,45</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>28,58</t>
-  </si>
-  <si>
-    <t>2,21</t>
-  </si>
-  <si>
-    <t>1,21</t>
-  </si>
-  <si>
-    <t>40,77</t>
-  </si>
-  <si>
-    <t>6,49</t>
-  </si>
-  <si>
-    <t>4,42</t>
-  </si>
-  <si>
-    <t>2,58</t>
-  </si>
-  <si>
-    <t>7,45</t>
-  </si>
-  <si>
-    <t>4,77</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>20,23</t>
-  </si>
-  <si>
-    <t>1,4</t>
-  </si>
-  <si>
-    <t>35,78</t>
-  </si>
-  <si>
-    <t>14,43</t>
-  </si>
-  <si>
-    <t>6,57</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>4,1</t>
-  </si>
-  <si>
-    <t>16,38</t>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>16,37</t>
   </si>
   <si>
     <t>1813</t>
@@ -841,22 +841,25 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>11,5</t>
-  </si>
-  <si>
-    <t>58,15</t>
-  </si>
-  <si>
-    <t>9,69</t>
-  </si>
-  <si>
-    <t>9,92</t>
-  </si>
-  <si>
-    <t>5,19</t>
-  </si>
-  <si>
-    <t>4,8</t>
+    <t>11,63</t>
+  </si>
+  <si>
+    <t>61,46</t>
+  </si>
+  <si>
+    <t>7,12</t>
+  </si>
+  <si>
+    <t>10,39</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>5,07</t>
+  </si>
+  <si>
+    <t>3,67</t>
   </si>
   <si>
     <t>1871</t>
@@ -865,34 +868,34 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>15,02</t>
-  </si>
-  <si>
-    <t>0,53</t>
-  </si>
-  <si>
-    <t>2,22</t>
-  </si>
-  <si>
-    <t>35,38</t>
-  </si>
-  <si>
-    <t>4,44</t>
-  </si>
-  <si>
-    <t>15,2</t>
-  </si>
-  <si>
-    <t>1,6</t>
-  </si>
-  <si>
-    <t>1,16</t>
-  </si>
-  <si>
-    <t>3,82</t>
-  </si>
-  <si>
-    <t>17,69</t>
+    <t>15,06</t>
+  </si>
+  <si>
+    <t>0,51</t>
+  </si>
+  <si>
+    <t>2,13</t>
+  </si>
+  <si>
+    <t>37,19</t>
+  </si>
+  <si>
+    <t>4,26</t>
+  </si>
+  <si>
+    <t>14,64</t>
+  </si>
+  <si>
+    <t>0,77</t>
+  </si>
+  <si>
+    <t>1,53</t>
+  </si>
+  <si>
+    <t>3,83</t>
+  </si>
+  <si>
+    <t>17,45</t>
   </si>
   <si>
     <t>1872</t>
@@ -901,34 +904,28 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>16,17</t>
-  </si>
-  <si>
-    <t>5,72</t>
-  </si>
-  <si>
-    <t>30,41</t>
-  </si>
-  <si>
-    <t>3,92</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>3,03</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>1,92</t>
-  </si>
-  <si>
-    <t>3,69</t>
-  </si>
-  <si>
-    <t>33,18</t>
+    <t>16,05</t>
+  </si>
+  <si>
+    <t>5,57</t>
+  </si>
+  <si>
+    <t>31,34</t>
+  </si>
+  <si>
+    <t>3,84</t>
+  </si>
+  <si>
+    <t>2,98</t>
+  </si>
+  <si>
+    <t>0,72</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>34,09</t>
   </si>
   <si>
     <t/>
@@ -1908,40 +1905,40 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>137675</v>
+        <v>144340</v>
       </c>
       <c r="D6" s="6">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>27506</v>
+        <v>28573</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2167</v>
+        <v>2063</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>57903</v>
+        <v>62588</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12494</v>
+        <v>12488</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
@@ -1953,7 +1950,7 @@
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>10494</v>
+        <v>11218</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1962,559 +1959,559 @@
         <v>98</v>
       </c>
       <c r="U6" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="V6" s="6">
+        <v>11</v>
+      </c>
+      <c r="W6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="V6" s="6">
+      <c r="X6" s="6">
+        <v>227</v>
+      </c>
+      <c r="Y6" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z6" s="6">
+        <v>33</v>
+      </c>
+      <c r="AA6" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB6" s="6">
         <v>19</v>
       </c>
-      <c r="W6" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="X6" s="6">
-        <v>213</v>
-      </c>
-      <c r="Y6" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="Z6" s="6">
-        <v>26</v>
-      </c>
-      <c r="AA6" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="AB6" s="6">
-        <v>18</v>
-      </c>
       <c r="AC6" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD6" s="6">
         <v>97</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AF6" s="6">
         <v>4</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH6" s="6">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AJ6" s="6">
-        <v>329</v>
+        <v>345</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AL6" s="6">
         <v>38</v>
       </c>
       <c r="AM6" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="AN6" s="6">
+        <v>66</v>
+      </c>
+      <c r="AO6" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="AP6" s="6">
+        <v>775</v>
+      </c>
+      <c r="AQ6" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="AN6" s="6">
-        <v>72</v>
-      </c>
-      <c r="AO6" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="AP6" s="6">
-        <v>739</v>
-      </c>
-      <c r="AQ6" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="AR6" s="6">
         <v>118</v>
       </c>
       <c r="AS6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT6" s="6">
+        <v>1016</v>
+      </c>
+      <c r="AU6" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="AV6" s="6">
+        <v>6769</v>
+      </c>
+      <c r="AW6" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="AT6" s="6">
-        <v>1048</v>
-      </c>
-      <c r="AU6" s="7" t="s">
+      <c r="AX6" s="6">
+        <v>15973</v>
+      </c>
+      <c r="AY6" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="AV6" s="6">
-        <v>6519</v>
-      </c>
-      <c r="AW6" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="AX6" s="6">
-        <v>15934</v>
-      </c>
-      <c r="AY6" s="7" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="9">
+        <v>7950</v>
+      </c>
+      <c r="D7" s="9">
+        <v>7</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="F7" s="9">
+        <v>1523</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="C7" s="9">
-        <v>7944</v>
-      </c>
-      <c r="D7" s="9">
-        <v>8</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="F7" s="9">
-        <v>1522</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="H7" s="9">
         <v>74</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J7" s="9">
         <v>64</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L7" s="9">
-        <v>3780</v>
+        <v>3784</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="N7" s="9">
         <v>338</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="P7" s="9">
         <v>11</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="R7" s="9">
         <v>357</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="T7" s="9">
         <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="V7" s="9">
         <v>0</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X7" s="9">
         <v>16</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Z7" s="9">
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AB7" s="9">
         <v>4</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="AD7" s="9">
         <v>9</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AF7" s="9">
         <v>0</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH7" s="9">
         <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ7" s="9">
         <v>16</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AN7" s="9">
         <v>1</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AP7" s="9">
         <v>38</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AR7" s="9">
         <v>7</v>
       </c>
       <c r="AS7" s="10" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="AT7" s="9">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AU7" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AV7" s="9">
+        <v>290</v>
+      </c>
+      <c r="AW7" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="AX7" s="9">
+        <v>1217</v>
+      </c>
+      <c r="AY7" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="AV7" s="9">
-        <v>289</v>
-      </c>
-      <c r="AW7" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>1215</v>
-      </c>
-      <c r="AY7" s="10" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C8" s="9">
-        <v>3433</v>
+        <v>3439</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F8" s="9">
         <v>472</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H8" s="9">
         <v>17</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J8" s="9">
         <v>19</v>
       </c>
       <c r="K8" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="L8" s="9">
+        <v>939</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="N8" s="9">
+        <v>1036</v>
+      </c>
+      <c r="O8" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="L8" s="9">
-        <v>938</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="N8" s="9">
-        <v>1032</v>
-      </c>
-      <c r="O8" s="10" t="s">
-        <v>149</v>
-      </c>
       <c r="P8" s="9">
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="R8" s="9">
         <v>225</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X8" s="9">
         <v>7</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AT8" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="AV8" s="9">
         <v>158</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AX8" s="9">
         <v>539</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="9">
+        <v>11136</v>
+      </c>
+      <c r="D9" s="9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F9" s="9">
+        <v>1727</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="C9" s="9">
-        <v>10773</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1685</v>
-      </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="9">
+        <v>190</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="H9" s="9">
-        <v>195</v>
-      </c>
-      <c r="I9" s="10" t="s">
+      <c r="J9" s="9">
+        <v>7</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="L9" s="9">
+        <v>5876</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="J9" s="9">
-        <v>19</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="L9" s="9">
-        <v>5570</v>
-      </c>
-      <c r="M9" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="N9" s="9">
         <v>850</v>
       </c>
       <c r="O9" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="P9" s="9">
+        <v>4</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="R9" s="9">
+        <v>1123</v>
+      </c>
+      <c r="S9" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="P9" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R9" s="9">
-        <v>1109</v>
-      </c>
-      <c r="S9" s="10" t="s">
-        <v>162</v>
       </c>
       <c r="T9" s="9">
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X9" s="9">
         <v>38</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Z9" s="9">
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD9" s="9">
         <v>9</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ9" s="9">
         <v>72</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP9" s="9">
         <v>108</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AT9" s="9">
         <v>5</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="AV9" s="9">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="AW9" s="10" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="AX9" s="9">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="AY9" s="10" t="s">
         <v>166</v>
@@ -2528,16 +2525,16 @@
         <v>168</v>
       </c>
       <c r="C10" s="9">
-        <v>21731</v>
+        <v>22513</v>
       </c>
       <c r="D10" s="9">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F10" s="9">
-        <v>5293</v>
+        <v>5563</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>169</v>
@@ -2549,293 +2546,293 @@
         <v>170</v>
       </c>
       <c r="J10" s="9">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>171</v>
       </c>
       <c r="L10" s="9">
-        <v>7389</v>
+        <v>7765</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>172</v>
       </c>
       <c r="N10" s="9">
-        <v>2633</v>
+        <v>2671</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>173</v>
       </c>
       <c r="P10" s="9">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="R10" s="9">
-        <v>1540</v>
+        <v>1620</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V10" s="9">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="X10" s="9">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="Z10" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AB10" s="9">
         <v>9</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="AD10" s="9">
         <v>17</v>
       </c>
       <c r="AE10" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG10" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH10" s="9">
+        <v>8</v>
+      </c>
+      <c r="AI10" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="AJ10" s="9">
+        <v>16</v>
+      </c>
+      <c r="AK10" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="AF10" s="9">
-        <v>0</v>
-      </c>
-      <c r="AG10" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH10" s="9">
-        <v>9</v>
-      </c>
-      <c r="AI10" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="AJ10" s="9">
-        <v>13</v>
-      </c>
-      <c r="AK10" s="10" t="s">
-        <v>152</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AN10" s="9">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>119</v>
+        <v>176</v>
       </c>
       <c r="AP10" s="9">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="AT10" s="9">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AV10" s="9">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AX10" s="9">
-        <v>1919</v>
+        <v>1924</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C11" s="9">
-        <v>16408</v>
+        <v>16744</v>
       </c>
       <c r="D11" s="9">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="F11" s="9">
-        <v>2689</v>
+        <v>2780</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H11" s="9">
         <v>285</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J11" s="9">
-        <v>153</v>
+        <v>110</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="L11" s="9">
-        <v>8325</v>
+        <v>8558</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="N11" s="9">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="P11" s="9">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="R11" s="9">
-        <v>1987</v>
+        <v>2011</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="X11" s="9">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>106</v>
+        <v>189</v>
       </c>
       <c r="Z11" s="9">
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AB11" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD11" s="9">
         <v>22</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH11" s="9">
         <v>5</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AJ11" s="9">
         <v>40</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AN11" s="9">
         <v>3</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AP11" s="9">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AR11" s="9">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>106</v>
+        <v>151</v>
       </c>
       <c r="AT11" s="9">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>189</v>
+        <v>137</v>
       </c>
       <c r="AV11" s="9">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AX11" s="9">
-        <v>1583</v>
+        <v>1585</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C12" s="9">
         <v>6000</v>
@@ -2844,201 +2841,201 @@
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F12" s="9">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H12" s="9">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="J12" s="9">
         <v>52</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L12" s="9">
         <v>2637</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N12" s="9">
         <v>729</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P12" s="9">
         <v>2</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="R12" s="9">
         <v>415</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="T12" s="9">
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V12" s="9">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X12" s="9">
         <v>26</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD12" s="9">
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>112</v>
+        <v>202</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH12" s="9">
         <v>0</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ12" s="9">
         <v>34</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AN12" s="9">
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP12" s="9">
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>165</v>
+        <v>204</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AT12" s="9">
         <v>6</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="AV12" s="9">
         <v>379</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AX12" s="9">
         <v>547</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C13" s="9">
-        <v>5086</v>
+        <v>5358</v>
       </c>
       <c r="D13" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>206</v>
+        <v>127</v>
       </c>
       <c r="F13" s="9">
-        <v>904</v>
+        <v>964</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H13" s="9">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>208</v>
+        <v>174</v>
       </c>
       <c r="J13" s="9">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="L13" s="9">
-        <v>2216</v>
+        <v>2310</v>
       </c>
       <c r="M13" s="10" t="s">
         <v>210</v>
       </c>
       <c r="N13" s="9">
-        <v>829</v>
+        <v>912</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>211</v>
       </c>
       <c r="P13" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="R13" s="9">
-        <v>313</v>
+        <v>365</v>
       </c>
       <c r="S13" s="10" t="s">
         <v>212</v>
@@ -3047,13 +3044,13 @@
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V13" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>152</v>
+        <v>115</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
@@ -3062,380 +3059,380 @@
         <v>106</v>
       </c>
       <c r="Z13" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="AF13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG13" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AJ13" s="9">
+        <v>42</v>
+      </c>
+      <c r="AK13" s="10" t="s">
         <v>213</v>
-      </c>
-      <c r="AF13" s="9">
-        <v>0</v>
-      </c>
-      <c r="AG13" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH13" s="9">
-        <v>2</v>
-      </c>
-      <c r="AI13" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="AJ13" s="9">
-        <v>33</v>
-      </c>
-      <c r="AK13" s="10" t="s">
-        <v>214</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>185</v>
+        <v>214</v>
       </c>
       <c r="AN13" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="AP13" s="9">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="AQ13" s="10" t="s">
         <v>215</v>
       </c>
       <c r="AR13" s="9">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="AS13" s="10" t="s">
         <v>216</v>
       </c>
       <c r="AT13" s="9">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="AU13" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="AV13" s="9">
+        <v>231</v>
+      </c>
+      <c r="AW13" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="AV13" s="9">
+      <c r="AX13" s="9">
+        <v>357</v>
+      </c>
+      <c r="AY13" s="10" t="s">
         <v>218</v>
-      </c>
-      <c r="AW13" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="AX13" s="9">
-        <v>351</v>
-      </c>
-      <c r="AY13" s="10" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="9">
+        <v>5225</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1160</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="C14" s="9">
-        <v>5044</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1133</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>222</v>
       </c>
       <c r="H14" s="9">
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="J14" s="9">
+        <v>14</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="L14" s="9">
+        <v>1622</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="J14" s="9">
-        <v>18</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="L14" s="9">
-        <v>1485</v>
-      </c>
-      <c r="M14" s="10" t="s">
+      <c r="N14" s="9">
+        <v>904</v>
+      </c>
+      <c r="O14" s="10" t="s">
         <v>224</v>
-      </c>
-      <c r="N14" s="9">
-        <v>892</v>
-      </c>
-      <c r="O14" s="10" t="s">
-        <v>225</v>
       </c>
       <c r="P14" s="9">
         <v>1</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="R14" s="9">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X14" s="9">
         <v>9</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>159</v>
+        <v>202</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ14" s="9">
         <v>20</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AN14" s="9">
         <v>1</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AP14" s="9">
         <v>38</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AT14" s="9">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="AU14" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="AV14" s="9">
+        <v>383</v>
+      </c>
+      <c r="AW14" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="AV14" s="9">
-        <v>374</v>
-      </c>
-      <c r="AW14" s="10" t="s">
+      <c r="AX14" s="9">
+        <v>703</v>
+      </c>
+      <c r="AY14" s="10" t="s">
         <v>229</v>
-      </c>
-      <c r="AX14" s="9">
-        <v>701</v>
-      </c>
-      <c r="AY14" s="10" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="9">
+        <v>13061</v>
+      </c>
+      <c r="D15" s="9">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F15" s="9">
+        <v>3946</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="C15" s="9">
-        <v>12956</v>
-      </c>
-      <c r="D15" s="9">
-        <v>0</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="9">
-        <v>3924</v>
-      </c>
-      <c r="G15" s="10" t="s">
+      <c r="H15" s="9">
+        <v>52</v>
+      </c>
+      <c r="I15" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="H15" s="9">
-        <v>55</v>
-      </c>
-      <c r="I15" s="10" t="s">
+      <c r="J15" s="9">
+        <v>30</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="L15" s="9">
+        <v>4195</v>
+      </c>
+      <c r="M15" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="J15" s="9">
-        <v>27</v>
-      </c>
-      <c r="K15" s="10" t="s">
+      <c r="N15" s="9">
+        <v>196</v>
+      </c>
+      <c r="O15" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="L15" s="9">
-        <v>4094</v>
-      </c>
-      <c r="M15" s="10" t="s">
+      <c r="P15" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="R15" s="9">
+        <v>771</v>
+      </c>
+      <c r="S15" s="10" t="s">
         <v>236</v>
-      </c>
-      <c r="N15" s="9">
-        <v>224</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="P15" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R15" s="9">
-        <v>766</v>
-      </c>
-      <c r="S15" s="10" t="s">
-        <v>238</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="V15" s="9">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>206</v>
+        <v>136</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH15" s="9">
         <v>0</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ15" s="9">
         <v>13</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="AL15" s="9">
         <v>2</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AN15" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="AP15" s="9">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>195</v>
+        <v>238</v>
       </c>
       <c r="AR15" s="9">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>135</v>
+        <v>239</v>
       </c>
       <c r="AT15" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>121</v>
+        <v>151</v>
       </c>
       <c r="AV15" s="9">
         <v>1071</v>
@@ -3444,7 +3441,7 @@
         <v>240</v>
       </c>
       <c r="AX15" s="9">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="AY15" s="10" t="s">
         <v>241</v>
@@ -3458,16 +3455,16 @@
         <v>243</v>
       </c>
       <c r="C16" s="9">
-        <v>5482</v>
+        <v>5551</v>
       </c>
       <c r="D16" s="9">
         <v>0</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F16" s="9">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>244</v>
@@ -3479,19 +3476,19 @@
         <v>245</v>
       </c>
       <c r="J16" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>175</v>
+        <v>116</v>
       </c>
       <c r="L16" s="9">
-        <v>1896</v>
+        <v>1947</v>
       </c>
       <c r="M16" s="10" t="s">
         <v>246</v>
       </c>
       <c r="N16" s="9">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="O16" s="10" t="s">
         <v>247</v>
@@ -3500,10 +3497,10 @@
         <v>0</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="R16" s="9">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S16" s="10" t="s">
         <v>248</v>
@@ -3512,67 +3509,67 @@
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X16" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>138</v>
+        <v>190</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="AB16" s="9">
         <v>0</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="AF16" s="9">
         <v>1</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ16" s="9">
         <v>30</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AN16" s="9">
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP16" s="9">
         <v>44</v>
@@ -3584,13 +3581,13 @@
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="AT16" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AV16" s="9">
         <v>436</v>
@@ -3599,7 +3596,7 @@
         <v>250</v>
       </c>
       <c r="AX16" s="9">
-        <v>1505</v>
+        <v>1508</v>
       </c>
       <c r="AY16" s="10" t="s">
         <v>251</v>
@@ -3613,136 +3610,136 @@
         <v>253</v>
       </c>
       <c r="C17" s="9">
-        <v>10499</v>
+        <v>10503</v>
       </c>
       <c r="D17" s="9">
         <v>32</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>254</v>
+        <v>187</v>
       </c>
       <c r="F17" s="9">
         <v>3001</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H17" s="9">
         <v>232</v>
       </c>
       <c r="I17" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="J17" s="9">
+        <v>130</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="J17" s="9">
-        <v>127</v>
-      </c>
-      <c r="K17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>4282</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>257</v>
-      </c>
-      <c r="L17" s="9">
-        <v>4280</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>258</v>
       </c>
       <c r="N17" s="9">
         <v>681</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="P17" s="9">
         <v>21</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="R17" s="9">
         <v>464</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V17" s="9">
         <v>4</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="X17" s="9">
         <v>8</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="Z17" s="9">
         <v>4</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AN17" s="9">
         <v>8</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>234</v>
+        <v>260</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="AT17" s="9">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AU17" s="10" t="s">
         <v>261</v>
@@ -3768,13 +3765,13 @@
         <v>265</v>
       </c>
       <c r="C18" s="9">
-        <v>11279</v>
+        <v>11285</v>
       </c>
       <c r="D18" s="9">
         <v>0</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F18" s="9">
         <v>2282</v>
@@ -3792,10 +3789,10 @@
         <v>0</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="L18" s="9">
-        <v>4036</v>
+        <v>4040</v>
       </c>
       <c r="M18" s="10" t="s">
         <v>268</v>
@@ -3810,10 +3807,10 @@
         <v>0</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="R18" s="9">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="S18" s="10" t="s">
         <v>270</v>
@@ -3822,85 +3819,85 @@
         <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>271</v>
+        <v>222</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X18" s="9">
         <v>11</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AB18" s="9">
         <v>0</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD18" s="9">
         <v>6</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="AN18" s="9">
         <v>0</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP18" s="9">
         <v>40</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>163</v>
+        <v>271</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="AT18" s="9">
         <v>0</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AV18" s="9">
         <v>462</v>
@@ -3923,16 +3920,16 @@
         <v>275</v>
       </c>
       <c r="C19" s="9">
-        <v>17311</v>
+        <v>21745</v>
       </c>
       <c r="D19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F19" s="9">
-        <v>1991</v>
+        <v>2529</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>276</v>
@@ -3941,34 +3938,34 @@
         <v>15</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="J19" s="9">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="L19" s="9">
-        <v>10067</v>
+        <v>13364</v>
       </c>
       <c r="M19" s="10" t="s">
         <v>277</v>
       </c>
       <c r="N19" s="9">
-        <v>1678</v>
+        <v>1549</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>278</v>
       </c>
       <c r="P19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="R19" s="9">
-        <v>1718</v>
+        <v>2259</v>
       </c>
       <c r="S19" s="10" t="s">
         <v>279</v>
@@ -3977,305 +3974,305 @@
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X19" s="9">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>206</v>
+        <v>136</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD19" s="9">
         <v>0</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AF19" s="9">
         <v>3</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ19" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP19" s="9">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>223</v>
+        <v>280</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AT19" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="AV19" s="9">
-        <v>898</v>
+        <v>1103</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AX19" s="9">
-        <v>831</v>
+        <v>797</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C20" s="9">
-        <v>1125</v>
+        <v>1175</v>
       </c>
       <c r="D20" s="9">
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F20" s="9">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="J20" s="9">
         <v>25</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="L20" s="9">
-        <v>398</v>
+        <v>437</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="N20" s="9">
         <v>50</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="P20" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>285</v>
+        <v>201</v>
       </c>
       <c r="R20" s="9">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>249</v>
+        <v>291</v>
       </c>
       <c r="Z20" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>271</v>
+        <v>162</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH20" s="9">
         <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ20" s="9">
         <v>7</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>159</v>
+        <v>202</v>
       </c>
       <c r="AN20" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="AR20" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="AT20" s="9">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>291</v>
+        <v>174</v>
       </c>
       <c r="AV20" s="9">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="AX20" s="9">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C21" s="9">
-        <v>2604</v>
+        <v>2655</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F21" s="9">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H21" s="9">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J21" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>106</v>
+        <v>160</v>
       </c>
       <c r="L21" s="9">
-        <v>792</v>
+        <v>832</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>300</v>
+        <v>187</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
@@ -4287,70 +4284,70 @@
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>206</v>
+        <v>136</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AP21" s="9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AQ21" s="10" t="s">
         <v>302</v>
@@ -4359,69 +4356,69 @@
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="AT21" s="9">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="AU21" s="10" t="s">
         <v>303</v>
       </c>
       <c r="AV21" s="9">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AW21" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="AX21" s="9">
+        <v>905</v>
+      </c>
+      <c r="AY21" s="10" t="s">
         <v>304</v>
-      </c>
-      <c r="AX21" s="9">
-        <v>864</v>
-      </c>
-      <c r="AY21" s="10" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>306</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>307</v>
-      </c>
       <c r="C22" s="12">
-        <v>137675</v>
+        <v>144340</v>
       </c>
       <c r="D22" s="12">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>27506</v>
+        <v>28573</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2167</v>
+        <v>2063</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>57903</v>
+        <v>62588</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12494</v>
+        <v>12488</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
@@ -4433,7 +4430,7 @@
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>10494</v>
+        <v>11218</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4442,97 +4439,97 @@
         <v>98</v>
       </c>
       <c r="U22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="V22" s="12">
+        <v>11</v>
+      </c>
+      <c r="W22" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="V22" s="12">
+      <c r="X22" s="12">
+        <v>227</v>
+      </c>
+      <c r="Y22" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z22" s="12">
+        <v>33</v>
+      </c>
+      <c r="AA22" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB22" s="12">
         <v>19</v>
       </c>
-      <c r="W22" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="X22" s="12">
-        <v>213</v>
-      </c>
-      <c r="Y22" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="Z22" s="12">
-        <v>26</v>
-      </c>
-      <c r="AA22" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="AB22" s="12">
-        <v>18</v>
-      </c>
       <c r="AC22" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AD22" s="12">
         <v>97</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AF22" s="12">
         <v>4</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="AH22" s="12">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="AJ22" s="12">
-        <v>329</v>
+        <v>345</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AL22" s="12">
         <v>38</v>
       </c>
       <c r="AM22" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="AN22" s="12">
+        <v>66</v>
+      </c>
+      <c r="AO22" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="AP22" s="12">
+        <v>775</v>
+      </c>
+      <c r="AQ22" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="AN22" s="12">
-        <v>72</v>
-      </c>
-      <c r="AO22" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="AP22" s="12">
-        <v>739</v>
-      </c>
-      <c r="AQ22" s="13" t="s">
-        <v>122</v>
       </c>
       <c r="AR22" s="12">
         <v>118</v>
       </c>
       <c r="AS22" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="AT22" s="12">
+        <v>1016</v>
+      </c>
+      <c r="AU22" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="AV22" s="12">
+        <v>6769</v>
+      </c>
+      <c r="AW22" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="AT22" s="12">
-        <v>1048</v>
-      </c>
-      <c r="AU22" s="13" t="s">
+      <c r="AX22" s="12">
+        <v>15973</v>
+      </c>
+      <c r="AY22" s="13" t="s">
         <v>124</v>
-      </c>
-      <c r="AV22" s="12">
-        <v>6519</v>
-      </c>
-      <c r="AW22" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="AX22" s="12">
-        <v>15934</v>
-      </c>
-      <c r="AY22" s="13" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 15/09/2026  6:38:59,63
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="305">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 13 Sep 2026, 14.36</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 15 Sep 2026, 06.36</t>
   </si>
   <si>
     <t>Kode</t>
@@ -331,33 +331,39 @@
     <t>LAMPUNG</t>
   </si>
   <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>19,77</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>1,31</t>
+  </si>
+  <si>
+    <t>44,08</t>
+  </si>
+  <si>
+    <t>8,42</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>7,84</t>
+  </si>
+  <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>19,8</t>
-  </si>
-  <si>
-    <t>1,02</t>
-  </si>
-  <si>
-    <t>1,43</t>
-  </si>
-  <si>
-    <t>43,36</t>
-  </si>
-  <si>
-    <t>8,65</t>
+    <t>0,01</t>
   </si>
   <si>
     <t>0,16</t>
   </si>
   <si>
-    <t>7,77</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
     <t>0,02</t>
   </si>
   <si>
@@ -370,562 +376,550 @@
     <t>0,03</t>
   </si>
   <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,53</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>4,67</t>
+  </si>
+  <si>
+    <t>10,89</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>19,29</t>
+  </si>
+  <si>
+    <t>0,92</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>47,07</t>
+  </si>
+  <si>
+    <t>5,16</t>
+  </si>
+  <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>0,54</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
     <t>4,69</t>
   </si>
   <si>
-    <t>11,07</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>1,2</t>
+  </si>
+  <si>
+    <t>3,73</t>
+  </si>
+  <si>
+    <t>16,37</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>14,05</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>27,88</t>
+  </si>
+  <si>
+    <t>29,95</t>
+  </si>
+  <si>
+    <t>6,76</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>4,57</t>
+  </si>
+  <si>
+    <t>15,36</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>15,44</t>
+  </si>
+  <si>
+    <t>1,6</t>
+  </si>
+  <si>
+    <t>53,3</t>
+  </si>
+  <si>
+    <t>7,45</t>
+  </si>
+  <si>
+    <t>10,44</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>3,47</t>
+  </si>
+  <si>
+    <t>6,17</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>24,68</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>7,01</t>
+  </si>
+  <si>
+    <t>34,59</t>
+  </si>
+  <si>
+    <t>11,79</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>7,24</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>19,16</t>
-  </si>
-  <si>
-    <t>0,93</t>
-  </si>
-  <si>
-    <t>0,81</t>
-  </si>
-  <si>
-    <t>47,6</t>
-  </si>
-  <si>
-    <t>4,25</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>4,49</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>2,38</t>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>2,01</t>
+  </si>
+  <si>
+    <t>8,52</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,69</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>0,52</t>
+  </si>
+  <si>
+    <t>51,38</t>
+  </si>
+  <si>
+    <t>3,3</t>
+  </si>
+  <si>
+    <t>12,16</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>2,86</t>
+  </si>
+  <si>
+    <t>9,77</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>17,73</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>44,16</t>
+  </si>
+  <si>
+    <t>12,12</t>
+  </si>
+  <si>
+    <t>7,03</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>6,27</t>
+  </si>
+  <si>
+    <t>9,15</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>18,19</t>
+  </si>
+  <si>
+    <t>43,46</t>
+  </si>
+  <si>
+    <t>17,07</t>
+  </si>
+  <si>
+    <t>6,74</t>
+  </si>
+  <si>
+    <t>0,77</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>4,24</t>
+  </si>
+  <si>
+    <t>6,63</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>20,99</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>35,49</t>
+  </si>
+  <si>
+    <t>16,06</t>
+  </si>
+  <si>
+    <t>5,86</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>7,12</t>
+  </si>
+  <si>
+    <t>12,54</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>30,11</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>32,46</t>
+  </si>
+  <si>
+    <t>1,35</t>
+  </si>
+  <si>
+    <t>5,87</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>8,19</t>
+  </si>
+  <si>
+    <t>19,91</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,24</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>36,55</t>
+  </si>
+  <si>
+    <t>4,59</t>
+  </si>
+  <si>
+    <t>5,18</t>
+  </si>
+  <si>
+    <t>7,74</t>
+  </si>
+  <si>
+    <t>26,42</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>28,55</t>
+  </si>
+  <si>
+    <t>2,13</t>
+  </si>
+  <si>
+    <t>1,21</t>
+  </si>
+  <si>
+    <t>40,97</t>
+  </si>
+  <si>
+    <t>6,41</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>4,52</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>2,56</t>
+  </si>
+  <si>
+    <t>7,4</t>
+  </si>
+  <si>
+    <t>4,72</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>20,22</t>
+  </si>
+  <si>
+    <t>1,4</t>
+  </si>
+  <si>
+    <t>35,8</t>
+  </si>
+  <si>
+    <t>14,42</t>
+  </si>
+  <si>
+    <t>6,58</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>62,1</t>
+  </si>
+  <si>
+    <t>6,15</t>
+  </si>
+  <si>
+    <t>10,21</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>5,05</t>
+  </si>
+  <si>
+    <t>3,28</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>14,97</t>
+  </si>
+  <si>
+    <t>0,51</t>
+  </si>
+  <si>
+    <t>2,12</t>
+  </si>
+  <si>
+    <t>37,39</t>
+  </si>
+  <si>
+    <t>4,23</t>
+  </si>
+  <si>
+    <t>14,55</t>
+  </si>
+  <si>
+    <t>1,52</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>0,85</t>
+  </si>
+  <si>
+    <t>3,81</t>
+  </si>
+  <si>
+    <t>17,34</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>16,03</t>
+  </si>
+  <si>
+    <t>5,57</t>
+  </si>
+  <si>
+    <t>31,34</t>
+  </si>
+  <si>
+    <t>3,84</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>2,97</t>
+  </si>
+  <si>
+    <t>0,71</t>
   </si>
   <si>
     <t>3,65</t>
   </si>
   <si>
-    <t>15,31</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>13,72</t>
-  </si>
-  <si>
-    <t>0,49</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>27,3</t>
-  </si>
-  <si>
-    <t>30,13</t>
-  </si>
-  <si>
-    <t>6,54</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>4,59</t>
-  </si>
-  <si>
-    <t>15,67</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>15,51</t>
-  </si>
-  <si>
-    <t>1,71</t>
-  </si>
-  <si>
-    <t>52,77</t>
-  </si>
-  <si>
-    <t>7,63</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>10,08</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>0,97</t>
-  </si>
-  <si>
-    <t>3,61</t>
-  </si>
-  <si>
-    <t>6,47</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>24,71</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>7,02</t>
-  </si>
-  <si>
-    <t>34,49</t>
-  </si>
-  <si>
-    <t>11,86</t>
-  </si>
-  <si>
-    <t>0,6</t>
-  </si>
-  <si>
-    <t>7,2</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>1,81</t>
-  </si>
-  <si>
-    <t>2,02</t>
-  </si>
-  <si>
-    <t>8,55</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>16,6</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>51,11</t>
-  </si>
-  <si>
-    <t>3,37</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>12,01</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>2,84</t>
-  </si>
-  <si>
-    <t>9,47</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>17,68</t>
-  </si>
-  <si>
-    <t>0,87</t>
-  </si>
-  <si>
-    <t>43,95</t>
-  </si>
-  <si>
-    <t>12,15</t>
-  </si>
-  <si>
-    <t>6,92</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>6,32</t>
-  </si>
-  <si>
-    <t>9,12</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>17,99</t>
-  </si>
-  <si>
-    <t>43,11</t>
-  </si>
-  <si>
-    <t>17,02</t>
-  </si>
-  <si>
-    <t>6,81</t>
-  </si>
-  <si>
-    <t>0,78</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>4,31</t>
-  </si>
-  <si>
-    <t>6,66</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>22,2</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>31,04</t>
-  </si>
-  <si>
-    <t>17,3</t>
-  </si>
-  <si>
-    <t>6,26</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>7,33</t>
-  </si>
-  <si>
-    <t>13,45</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,21</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>32,12</t>
-  </si>
-  <si>
-    <t>1,5</t>
-  </si>
-  <si>
-    <t>5,9</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>8,2</t>
-  </si>
-  <si>
-    <t>20,04</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,33</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>35,07</t>
-  </si>
-  <si>
-    <t>5,03</t>
-  </si>
-  <si>
-    <t>5,17</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>7,85</t>
-  </si>
-  <si>
-    <t>27,17</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>28,57</t>
-  </si>
-  <si>
-    <t>2,21</t>
-  </si>
-  <si>
-    <t>1,24</t>
-  </si>
-  <si>
-    <t>40,77</t>
-  </si>
-  <si>
-    <t>6,48</t>
-  </si>
-  <si>
-    <t>4,42</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>2,57</t>
-  </si>
-  <si>
-    <t>7,45</t>
-  </si>
-  <si>
-    <t>4,77</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>20,22</t>
-  </si>
-  <si>
-    <t>1,4</t>
-  </si>
-  <si>
-    <t>35,8</t>
-  </si>
-  <si>
-    <t>14,42</t>
-  </si>
-  <si>
-    <t>6,58</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>4,09</t>
-  </si>
-  <si>
-    <t>16,37</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>11,63</t>
-  </si>
-  <si>
-    <t>61,46</t>
-  </si>
-  <si>
-    <t>7,12</t>
-  </si>
-  <si>
-    <t>10,39</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>5,07</t>
-  </si>
-  <si>
-    <t>3,67</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>15,06</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>2,13</t>
-  </si>
-  <si>
-    <t>37,19</t>
-  </si>
-  <si>
-    <t>4,26</t>
-  </si>
-  <si>
-    <t>14,64</t>
-  </si>
-  <si>
-    <t>0,77</t>
-  </si>
-  <si>
-    <t>1,53</t>
-  </si>
-  <si>
-    <t>3,83</t>
-  </si>
-  <si>
-    <t>17,45</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>16,05</t>
-  </si>
-  <si>
-    <t>5,57</t>
-  </si>
-  <si>
-    <t>31,34</t>
-  </si>
-  <si>
-    <t>3,84</t>
-  </si>
-  <si>
-    <t>2,98</t>
-  </si>
-  <si>
-    <t>0,72</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>34,09</t>
+    <t>34,05</t>
   </si>
   <si>
     <t/>
@@ -1905,52 +1899,52 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>144340</v>
+        <v>149053</v>
       </c>
       <c r="D6" s="6">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>28573</v>
+        <v>29475</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1470</v>
+        <v>1485</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>2063</v>
+        <v>1948</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>62588</v>
+        <v>65700</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12488</v>
+        <v>12552</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>236</v>
+        <v>193</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>11218</v>
+        <v>11681</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
@@ -1959,463 +1953,463 @@
         <v>98</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="Z6" s="6">
         <v>33</v>
       </c>
       <c r="AA6" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AB6" s="6">
+        <v>16</v>
+      </c>
+      <c r="AC6" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="AB6" s="6">
-        <v>19</v>
-      </c>
-      <c r="AC6" s="7" t="s">
+      <c r="AD6" s="6">
+        <v>104</v>
+      </c>
+      <c r="AE6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="AD6" s="6">
-        <v>97</v>
-      </c>
-      <c r="AE6" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="AF6" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH6" s="6">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ6" s="6">
-        <v>345</v>
+        <v>356</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="AL6" s="6">
         <v>38</v>
       </c>
       <c r="AM6" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AO6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AP6" s="6">
+        <v>788</v>
+      </c>
+      <c r="AQ6" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR6" s="6">
         <v>119</v>
       </c>
-      <c r="AP6" s="6">
-        <v>775</v>
-      </c>
-      <c r="AQ6" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR6" s="6">
-        <v>118</v>
-      </c>
       <c r="AS6" s="7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AT6" s="6">
-        <v>1016</v>
+        <v>848</v>
       </c>
       <c r="AU6" s="7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AV6" s="6">
-        <v>6769</v>
+        <v>6962</v>
       </c>
       <c r="AW6" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>15973</v>
+        <v>16238</v>
       </c>
       <c r="AY6" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>7950</v>
+        <v>8331</v>
       </c>
       <c r="D7" s="9">
         <v>7</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F7" s="9">
-        <v>1523</v>
+        <v>1607</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H7" s="9">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J7" s="9">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L7" s="9">
-        <v>3784</v>
+        <v>3921</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N7" s="9">
-        <v>338</v>
+        <v>430</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P7" s="9">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R7" s="9">
-        <v>357</v>
+        <v>391</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="T7" s="9">
         <v>2</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V7" s="9">
         <v>0</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X7" s="9">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Z7" s="9">
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AB7" s="9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="AD7" s="9">
         <v>9</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AF7" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AH7" s="9">
         <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ7" s="9">
         <v>16</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AN7" s="9">
         <v>1</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AP7" s="9">
         <v>38</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="AR7" s="9">
         <v>7</v>
       </c>
       <c r="AS7" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="AT7" s="9">
-        <v>189</v>
+        <v>100</v>
       </c>
       <c r="AU7" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AV7" s="9">
-        <v>290</v>
+        <v>311</v>
       </c>
       <c r="AW7" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="AX7" s="9">
-        <v>1217</v>
+        <v>1364</v>
       </c>
       <c r="AY7" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C8" s="9">
-        <v>3439</v>
+        <v>3522</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F8" s="9">
-        <v>472</v>
+        <v>495</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H8" s="9">
         <v>17</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J8" s="9">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="L8" s="9">
-        <v>939</v>
+        <v>982</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="N8" s="9">
-        <v>1036</v>
+        <v>1055</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P8" s="9">
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="R8" s="9">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X8" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>151</v>
+        <v>106</v>
       </c>
       <c r="AT8" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="AV8" s="9">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AX8" s="9">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C9" s="9">
-        <v>11136</v>
+        <v>11729</v>
       </c>
       <c r="D9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F9" s="9">
-        <v>1727</v>
+        <v>1811</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H9" s="9">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J9" s="9">
         <v>7</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>151</v>
+        <v>106</v>
       </c>
       <c r="L9" s="9">
-        <v>5876</v>
+        <v>6252</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N9" s="9">
-        <v>850</v>
+        <v>874</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P9" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>160</v>
+        <v>115</v>
       </c>
       <c r="R9" s="9">
-        <v>1123</v>
+        <v>1224</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>161</v>
@@ -2424,16 +2418,16 @@
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X9" s="9">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Y9" s="10" t="s">
         <v>162</v>
@@ -2442,34 +2436,34 @@
         <v>0</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD9" s="9">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ9" s="9">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AK9" s="10" t="s">
         <v>163</v>
@@ -2478,63 +2472,63 @@
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AN9" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AP9" s="9">
         <v>108</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AT9" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="AV9" s="9">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="AW9" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="AX9" s="9">
+        <v>724</v>
+      </c>
+      <c r="AY9" s="10" t="s">
         <v>165</v>
-      </c>
-      <c r="AX9" s="9">
-        <v>721</v>
-      </c>
-      <c r="AY9" s="10" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>168</v>
-      </c>
       <c r="C10" s="9">
-        <v>22513</v>
+        <v>22596</v>
       </c>
       <c r="D10" s="9">
         <v>46</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="F10" s="9">
-        <v>5563</v>
+        <v>5576</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>169</v>
@@ -2546,19 +2540,19 @@
         <v>170</v>
       </c>
       <c r="J10" s="9">
-        <v>1580</v>
+        <v>1584</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>171</v>
       </c>
       <c r="L10" s="9">
-        <v>7765</v>
+        <v>7815</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>172</v>
       </c>
       <c r="N10" s="9">
-        <v>2671</v>
+        <v>2665</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>173</v>
@@ -2570,7 +2564,7 @@
         <v>174</v>
       </c>
       <c r="R10" s="9">
-        <v>1620</v>
+        <v>1637</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>175</v>
@@ -2579,153 +2573,153 @@
         <v>2</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="V10" s="9">
         <v>1</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X10" s="9">
         <v>20</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="Z10" s="9">
         <v>6</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AB10" s="9">
         <v>9</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="AD10" s="9">
         <v>17</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH10" s="9">
         <v>8</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="AJ10" s="9">
         <v>16</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AL10" s="9">
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AN10" s="9">
         <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="AP10" s="9">
         <v>34</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="AT10" s="9">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AV10" s="9">
         <v>454</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AX10" s="9">
-        <v>1924</v>
+        <v>1926</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C11" s="9">
-        <v>16744</v>
+        <v>17070</v>
       </c>
       <c r="D11" s="9">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F11" s="9">
-        <v>2780</v>
+        <v>2849</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H11" s="9">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J11" s="9">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="L11" s="9">
-        <v>8558</v>
+        <v>8770</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N11" s="9">
         <v>564</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P11" s="9">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>187</v>
+        <v>137</v>
       </c>
       <c r="R11" s="9">
-        <v>2011</v>
+        <v>2076</v>
       </c>
       <c r="S11" s="10" t="s">
         <v>188</v>
@@ -2734,13 +2728,13 @@
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="V11" s="9">
         <v>5</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="X11" s="9">
         <v>17</v>
@@ -2752,52 +2746,52 @@
         <v>5</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AB11" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AD11" s="9">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="AE11" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG11" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI11" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AJ11" s="9">
+        <v>48</v>
+      </c>
+      <c r="AK11" s="10" t="s">
         <v>190</v>
-      </c>
-      <c r="AF11" s="9">
-        <v>0</v>
-      </c>
-      <c r="AG11" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AH11" s="9">
-        <v>5</v>
-      </c>
-      <c r="AI11" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AJ11" s="9">
-        <v>40</v>
-      </c>
-      <c r="AK11" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AN11" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AO11" s="10" t="s">
         <v>115</v>
       </c>
       <c r="AP11" s="9">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="AQ11" s="10" t="s">
         <v>191</v>
@@ -2806,22 +2800,22 @@
         <v>10</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>151</v>
+        <v>106</v>
       </c>
       <c r="AT11" s="9">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>137</v>
+        <v>106</v>
       </c>
       <c r="AV11" s="9">
-        <v>476</v>
+        <v>488</v>
       </c>
       <c r="AW11" s="10" t="s">
         <v>192</v>
       </c>
       <c r="AX11" s="9">
-        <v>1585</v>
+        <v>1667</v>
       </c>
       <c r="AY11" s="10" t="s">
         <v>193</v>
@@ -2835,16 +2829,16 @@
         <v>195</v>
       </c>
       <c r="C12" s="9">
-        <v>6000</v>
+        <v>6046</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F12" s="9">
-        <v>1061</v>
+        <v>1072</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>196</v>
@@ -2853,34 +2847,34 @@
         <v>39</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>163</v>
+        <v>197</v>
       </c>
       <c r="J12" s="9">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="L12" s="9">
-        <v>2637</v>
+        <v>2670</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>198</v>
       </c>
       <c r="N12" s="9">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="O12" s="10" t="s">
         <v>199</v>
       </c>
       <c r="P12" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="10" t="s">
         <v>118</v>
       </c>
       <c r="R12" s="9">
-        <v>415</v>
+        <v>425</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>200</v>
@@ -2889,120 +2883,120 @@
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V12" s="9">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X12" s="9">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>201</v>
+        <v>139</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD12" s="9">
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF12" s="9">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH12" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AJ12" s="9">
+        <v>35</v>
+      </c>
+      <c r="AK12" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="AF12" s="9">
-        <v>0</v>
-      </c>
-      <c r="AG12" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AH12" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AJ12" s="9">
-        <v>34</v>
-      </c>
-      <c r="AK12" s="10" t="s">
-        <v>203</v>
-      </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AN12" s="9">
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP12" s="9">
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AT12" s="9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="AV12" s="9">
         <v>379</v>
       </c>
       <c r="AW12" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="AX12" s="9">
+        <v>553</v>
+      </c>
+      <c r="AY12" s="10" t="s">
         <v>205</v>
-      </c>
-      <c r="AX12" s="9">
-        <v>547</v>
-      </c>
-      <c r="AY12" s="10" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="C13" s="9">
+        <v>5442</v>
+      </c>
+      <c r="D13" s="9">
+        <v>0</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F13" s="9">
+        <v>990</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>208</v>
-      </c>
-      <c r="C13" s="9">
-        <v>5358</v>
-      </c>
-      <c r="D13" s="9">
-        <v>5</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F13" s="9">
-        <v>964</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>209</v>
       </c>
       <c r="H13" s="9">
         <v>32</v>
@@ -3011,392 +3005,392 @@
         <v>174</v>
       </c>
       <c r="J13" s="9">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>187</v>
+        <v>106</v>
       </c>
       <c r="L13" s="9">
-        <v>2310</v>
+        <v>2365</v>
       </c>
       <c r="M13" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="N13" s="9">
+        <v>929</v>
+      </c>
+      <c r="O13" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="N13" s="9">
-        <v>912</v>
-      </c>
-      <c r="O13" s="10" t="s">
+      <c r="P13" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R13" s="9">
+        <v>367</v>
+      </c>
+      <c r="S13" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="P13" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="R13" s="9">
-        <v>365</v>
-      </c>
-      <c r="S13" s="10" t="s">
-        <v>212</v>
-      </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V13" s="9">
         <v>1</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="Z13" s="9">
         <v>3</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>151</v>
+        <v>106</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH13" s="9">
         <v>0</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ13" s="9">
         <v>42</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
       <c r="AN13" s="9">
         <v>0</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP13" s="9">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="AR13" s="9">
         <v>27</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="AT13" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="AV13" s="9">
         <v>231</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AX13" s="9">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" s="9">
+        <v>5798</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="9">
+        <v>1217</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="H14" s="9">
+        <v>23</v>
+      </c>
+      <c r="I14" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="C14" s="9">
-        <v>5225</v>
-      </c>
-      <c r="D14" s="9">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="F14" s="9">
-        <v>1160</v>
-      </c>
-      <c r="G14" s="10" t="s">
+      <c r="J14" s="9">
+        <v>3</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="L14" s="9">
+        <v>2058</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="H14" s="9">
-        <v>18</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="J14" s="9">
-        <v>14</v>
-      </c>
-      <c r="K14" s="10" t="s">
+      <c r="N14" s="9">
+        <v>931</v>
+      </c>
+      <c r="O14" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="L14" s="9">
-        <v>1622</v>
-      </c>
-      <c r="M14" s="10" t="s">
+      <c r="P14" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R14" s="9">
+        <v>340</v>
+      </c>
+      <c r="S14" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="N14" s="9">
-        <v>904</v>
-      </c>
-      <c r="O14" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="P14" s="9">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="R14" s="9">
-        <v>327</v>
-      </c>
-      <c r="S14" s="10" t="s">
-        <v>225</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X14" s="9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ14" s="9">
         <v>20</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AN14" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AP14" s="9">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AQ14" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="AR14" s="9">
+        <v>2</v>
+      </c>
+      <c r="AS14" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="AT14" s="9">
+        <v>4</v>
+      </c>
+      <c r="AU14" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="AV14" s="9">
+        <v>413</v>
+      </c>
+      <c r="AW14" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="AX14" s="9">
+        <v>727</v>
+      </c>
+      <c r="AY14" s="10" t="s">
         <v>227</v>
-      </c>
-      <c r="AR14" s="9">
-        <v>1</v>
-      </c>
-      <c r="AS14" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="AT14" s="9">
-        <v>14</v>
-      </c>
-      <c r="AU14" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="AV14" s="9">
-        <v>383</v>
-      </c>
-      <c r="AW14" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="AX14" s="9">
-        <v>703</v>
-      </c>
-      <c r="AY14" s="10" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C15" s="9">
+        <v>13132</v>
+      </c>
+      <c r="D15" s="9">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" s="9">
+        <v>3954</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>230</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="C15" s="9">
-        <v>13061</v>
-      </c>
-      <c r="D15" s="9">
-        <v>0</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="F15" s="9">
-        <v>3946</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>232</v>
       </c>
       <c r="H15" s="9">
         <v>52</v>
       </c>
       <c r="I15" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="J15" s="9">
+        <v>35</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="L15" s="9">
+        <v>4263</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="N15" s="9">
+        <v>177</v>
+      </c>
+      <c r="O15" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="J15" s="9">
-        <v>30</v>
-      </c>
-      <c r="K15" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="L15" s="9">
-        <v>4195</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="N15" s="9">
-        <v>196</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>235</v>
-      </c>
       <c r="P15" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R15" s="9">
         <v>771</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="T15" s="9">
         <v>41</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="V15" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="X15" s="9">
         <v>15</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH15" s="9">
         <v>0</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ15" s="9">
         <v>13</v>
@@ -3408,329 +3402,329 @@
         <v>2</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AN15" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AP15" s="9">
         <v>84</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AR15" s="9">
         <v>16</v>
       </c>
       <c r="AS15" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="AT15" s="9">
+        <v>11</v>
+      </c>
+      <c r="AU15" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="AV15" s="9">
+        <v>1076</v>
+      </c>
+      <c r="AW15" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="AX15" s="9">
+        <v>2615</v>
+      </c>
+      <c r="AY15" s="10" t="s">
         <v>239</v>
-      </c>
-      <c r="AT15" s="9">
-        <v>8</v>
-      </c>
-      <c r="AU15" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="AV15" s="9">
-        <v>1071</v>
-      </c>
-      <c r="AW15" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="AX15" s="9">
-        <v>2617</v>
-      </c>
-      <c r="AY15" s="10" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" s="9">
+        <v>5749</v>
+      </c>
+      <c r="D16" s="9">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F16" s="9">
+        <v>991</v>
+      </c>
+      <c r="G16" s="10" t="s">
         <v>242</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="C16" s="9">
-        <v>5551</v>
-      </c>
-      <c r="D16" s="9">
-        <v>0</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="F16" s="9">
-        <v>962</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>244</v>
       </c>
       <c r="H16" s="9">
         <v>32</v>
       </c>
       <c r="I16" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="J16" s="9">
+        <v>0</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="L16" s="9">
+        <v>2101</v>
+      </c>
+      <c r="M16" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="N16" s="9">
+        <v>264</v>
+      </c>
+      <c r="O16" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="J16" s="9">
-        <v>0</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="L16" s="9">
-        <v>1947</v>
-      </c>
-      <c r="M16" s="10" t="s">
+      <c r="P16" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R16" s="9">
+        <v>298</v>
+      </c>
+      <c r="S16" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="N16" s="9">
-        <v>279</v>
-      </c>
-      <c r="O16" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="P16" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="R16" s="9">
-        <v>287</v>
-      </c>
-      <c r="S16" s="10" t="s">
-        <v>248</v>
-      </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X16" s="9">
         <v>7</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>190</v>
+        <v>237</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="AB16" s="9">
         <v>0</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="AF16" s="9">
         <v>1</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ16" s="9">
         <v>30</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>120</v>
+        <v>185</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AN16" s="9">
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP16" s="9">
         <v>44</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>249</v>
+        <v>212</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>190</v>
+        <v>237</v>
       </c>
       <c r="AT16" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AV16" s="9">
-        <v>436</v>
+        <v>445</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="AX16" s="9">
-        <v>1508</v>
+        <v>1519</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C17" s="9">
+        <v>10622</v>
+      </c>
+      <c r="D17" s="9">
+        <v>33</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="F17" s="9">
+        <v>3033</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="H17" s="9">
+        <v>226</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="J17" s="9">
+        <v>128</v>
+      </c>
+      <c r="K17" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="C17" s="9">
-        <v>10503</v>
-      </c>
-      <c r="D17" s="9">
-        <v>32</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="F17" s="9">
-        <v>3001</v>
-      </c>
-      <c r="G17" s="10" t="s">
+      <c r="L17" s="9">
+        <v>4352</v>
+      </c>
+      <c r="M17" s="10" t="s">
         <v>254</v>
-      </c>
-      <c r="H17" s="9">
-        <v>232</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>255</v>
-      </c>
-      <c r="J17" s="9">
-        <v>130</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="L17" s="9">
-        <v>4282</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>257</v>
       </c>
       <c r="N17" s="9">
         <v>681</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="P17" s="9">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>135</v>
+        <v>256</v>
       </c>
       <c r="R17" s="9">
-        <v>464</v>
+        <v>480</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="V17" s="9">
         <v>4</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="X17" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="Z17" s="9">
         <v>4</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="AF17" s="9">
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AN17" s="9">
         <v>8</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
@@ -3739,30 +3733,30 @@
         <v>189</v>
       </c>
       <c r="AT17" s="9">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="AV17" s="9">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="AX17" s="9">
         <v>501</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C18" s="9">
         <v>11285</v>
@@ -3771,61 +3765,61 @@
         <v>0</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F18" s="9">
         <v>2282</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H18" s="9">
         <v>158</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="J18" s="9">
         <v>0</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L18" s="9">
         <v>4040</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="N18" s="9">
         <v>1627</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="P18" s="9">
         <v>0</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="R18" s="9">
         <v>743</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="T18" s="9">
         <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X18" s="9">
         <v>11</v>
@@ -3837,31 +3831,31 @@
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AB18" s="9">
         <v>0</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD18" s="9">
         <v>6</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
@@ -3873,305 +3867,305 @@
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="AN18" s="9">
         <v>0</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP18" s="9">
         <v>40</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="AT18" s="9">
         <v>0</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AV18" s="9">
         <v>462</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="AX18" s="9">
         <v>1847</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>273</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="C19" s="9">
+        <v>23891</v>
+      </c>
+      <c r="D19" s="9">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="9">
+        <v>2995</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H19" s="9">
+        <v>24</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="J19" s="9">
+        <v>13</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="L19" s="9">
+        <v>14836</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="N19" s="9">
+        <v>1470</v>
+      </c>
+      <c r="O19" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="P19" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="R19" s="9">
+        <v>2440</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="C19" s="9">
-        <v>21745</v>
-      </c>
-      <c r="D19" s="9">
-        <v>0</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="F19" s="9">
-        <v>2529</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="H19" s="9">
-        <v>15</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="J19" s="9">
-        <v>15</v>
-      </c>
-      <c r="K19" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="L19" s="9">
-        <v>13364</v>
-      </c>
-      <c r="M19" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="N19" s="9">
-        <v>1549</v>
-      </c>
-      <c r="O19" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="P19" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="R19" s="9">
-        <v>2259</v>
-      </c>
-      <c r="S19" s="10" t="s">
-        <v>279</v>
-      </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V19" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X19" s="9">
         <v>23</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>136</v>
+        <v>189</v>
       </c>
       <c r="Z19" s="9">
         <v>0</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD19" s="9">
         <v>0</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AF19" s="9">
         <v>3</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ19" s="9">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP19" s="9">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AT19" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AV19" s="9">
-        <v>1103</v>
+        <v>1207</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="AX19" s="9">
-        <v>797</v>
+        <v>783</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C20" s="9">
-        <v>1175</v>
+        <v>1182</v>
       </c>
       <c r="D20" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="F20" s="9">
         <v>177</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="J20" s="9">
         <v>25</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="L20" s="9">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="N20" s="9">
         <v>50</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="P20" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>201</v>
+        <v>224</v>
       </c>
       <c r="R20" s="9">
         <v>172</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>291</v>
+        <v>170</v>
       </c>
       <c r="Z20" s="9">
         <v>4</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>162</v>
+        <v>224</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH20" s="9">
         <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ20" s="9">
         <v>7</v>
@@ -4183,254 +4177,254 @@
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AN20" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="AP20" s="9">
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="AR20" s="9">
         <v>5</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>201</v>
+        <v>288</v>
       </c>
       <c r="AT20" s="9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>174</v>
+        <v>289</v>
       </c>
       <c r="AV20" s="9">
         <v>45</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="AX20" s="9">
         <v>205</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C21" s="9">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F21" s="9">
         <v>426</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="H21" s="9">
         <v>148</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="L21" s="9">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>187</v>
+        <v>298</v>
       </c>
       <c r="R21" s="9">
         <v>79</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AP21" s="9">
         <v>19</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="AT21" s="9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>303</v>
+        <v>236</v>
       </c>
       <c r="AV21" s="9">
         <v>97</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>139</v>
+        <v>301</v>
       </c>
       <c r="AX21" s="9">
         <v>905</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C22" s="12">
-        <v>144340</v>
+        <v>149053</v>
       </c>
       <c r="D22" s="12">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>28573</v>
+        <v>29475</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1470</v>
+        <v>1485</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>2063</v>
+        <v>1948</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>62588</v>
+        <v>65700</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12488</v>
+        <v>12552</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>236</v>
+        <v>193</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>11218</v>
+        <v>11681</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
@@ -4439,97 +4433,97 @@
         <v>98</v>
       </c>
       <c r="U22" s="13" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="W22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="Y22" s="13" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="Z22" s="12">
         <v>33</v>
       </c>
       <c r="AA22" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="AB22" s="12">
+        <v>16</v>
+      </c>
+      <c r="AC22" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="AB22" s="12">
-        <v>19</v>
-      </c>
-      <c r="AC22" s="13" t="s">
+      <c r="AD22" s="12">
+        <v>104</v>
+      </c>
+      <c r="AE22" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="AD22" s="12">
-        <v>97</v>
-      </c>
-      <c r="AE22" s="13" t="s">
-        <v>106</v>
-      </c>
       <c r="AF22" s="12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AH22" s="12">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AJ22" s="12">
-        <v>345</v>
+        <v>356</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="AL22" s="12">
         <v>38</v>
       </c>
       <c r="AM22" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AO22" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="AP22" s="12">
+        <v>788</v>
+      </c>
+      <c r="AQ22" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR22" s="12">
         <v>119</v>
       </c>
-      <c r="AP22" s="12">
-        <v>775</v>
-      </c>
-      <c r="AQ22" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR22" s="12">
-        <v>118</v>
-      </c>
       <c r="AS22" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AT22" s="12">
-        <v>1016</v>
+        <v>848</v>
       </c>
       <c r="AU22" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AV22" s="12">
-        <v>6769</v>
+        <v>6962</v>
       </c>
       <c r="AW22" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>15973</v>
+        <v>16238</v>
       </c>
       <c r="AY22" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 16/09/2026  8:58:14,59
</commit_message>
<xml_diff>
--- a/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
+++ b/data/20260823_125259_Radar_Anomali_Usaha_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Anomali_8_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="294">
   <si>
     <t>DATA RADAR ANOMALI USAHA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 15 Sep 2026, 06.36</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 16 Sep 2026, 08.57</t>
   </si>
   <si>
     <t>Kode</t>
@@ -334,592 +334,559 @@
     <t>0,06</t>
   </si>
   <si>
-    <t>19,77</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>1,31</t>
-  </si>
-  <si>
-    <t>44,08</t>
-  </si>
-  <si>
-    <t>8,42</t>
+    <t>19,69</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>1,16</t>
+  </si>
+  <si>
+    <t>44,7</t>
+  </si>
+  <si>
+    <t>8,27</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>7,88</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>0,01</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>0,52</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>4,63</t>
+  </si>
+  <si>
+    <t>10,77</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>19,27</t>
+  </si>
+  <si>
+    <t>1,1</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>46,88</t>
+  </si>
+  <si>
+    <t>5,26</t>
+  </si>
+  <si>
+    <t>4,71</t>
+  </si>
+  <si>
+    <t>0,21</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>0,57</t>
+  </si>
+  <si>
+    <t>3,75</t>
+  </si>
+  <si>
+    <t>17,15</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>14,4</t>
+  </si>
+  <si>
+    <t>32,59</t>
+  </si>
+  <si>
+    <t>27,11</t>
+  </si>
+  <si>
+    <t>6,38</t>
   </si>
   <si>
     <t>0,13</t>
   </si>
   <si>
-    <t>7,84</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>0,53</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>4,67</t>
-  </si>
-  <si>
-    <t>10,89</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>19,29</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>47,07</t>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>4,24</t>
+  </si>
+  <si>
+    <t>13,99</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>14,99</t>
+  </si>
+  <si>
+    <t>1,45</t>
+  </si>
+  <si>
+    <t>54,84</t>
+  </si>
+  <si>
+    <t>6,9</t>
+  </si>
+  <si>
+    <t>10,92</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>3,27</t>
+  </si>
+  <si>
+    <t>5,72</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>24,72</t>
+  </si>
+  <si>
+    <t>0,76</t>
+  </si>
+  <si>
+    <t>6,94</t>
+  </si>
+  <si>
+    <t>34,69</t>
+  </si>
+  <si>
+    <t>11,8</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>7,2</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>1,81</t>
+  </si>
+  <si>
+    <t>2,04</t>
+  </si>
+  <si>
+    <t>8,46</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>16,74</t>
+  </si>
+  <si>
+    <t>1,67</t>
+  </si>
+  <si>
+    <t>52,15</t>
+  </si>
+  <si>
+    <t>12,25</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>2,88</t>
+  </si>
+  <si>
+    <t>9,59</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>17,88</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>44,6</t>
+  </si>
+  <si>
+    <t>12,03</t>
+  </si>
+  <si>
+    <t>7,08</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>6,21</t>
+  </si>
+  <si>
+    <t>9,04</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>18,19</t>
+  </si>
+  <si>
+    <t>43,57</t>
+  </si>
+  <si>
+    <t>17,01</t>
+  </si>
+  <si>
+    <t>6,74</t>
+  </si>
+  <si>
+    <t>0,77</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>0,49</t>
+  </si>
+  <si>
+    <t>4,23</t>
+  </si>
+  <si>
+    <t>6,61</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>20,56</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>38,37</t>
+  </si>
+  <si>
+    <t>15,07</t>
+  </si>
+  <si>
+    <t>5,62</t>
+  </si>
+  <si>
+    <t>0,32</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>6,91</t>
+  </si>
+  <si>
+    <t>11,79</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>29,89</t>
+  </si>
+  <si>
+    <t>0,39</t>
+  </si>
+  <si>
+    <t>33,13</t>
+  </si>
+  <si>
+    <t>1,33</t>
+  </si>
+  <si>
+    <t>5,9</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>8,13</t>
+  </si>
+  <si>
+    <t>19,86</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>17,14</t>
+  </si>
+  <si>
+    <t>37,16</t>
+  </si>
+  <si>
+    <t>4,26</t>
   </si>
   <si>
     <t>5,16</t>
   </si>
   <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>4,69</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,19</t>
-  </si>
-  <si>
-    <t>0,46</t>
+    <t>7,7</t>
+  </si>
+  <si>
+    <t>26,29</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>28,52</t>
+  </si>
+  <si>
+    <t>2,11</t>
   </si>
   <si>
     <t>1,2</t>
   </si>
   <si>
+    <t>41,18</t>
+  </si>
+  <si>
+    <t>6,36</t>
+  </si>
+  <si>
+    <t>4,49</t>
+  </si>
+  <si>
+    <t>2,54</t>
+  </si>
+  <si>
+    <t>7,4</t>
+  </si>
+  <si>
+    <t>4,68</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>20,21</t>
+  </si>
+  <si>
+    <t>1,4</t>
+  </si>
+  <si>
+    <t>35,79</t>
+  </si>
+  <si>
+    <t>6,58</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>16,35</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>12,66</t>
+  </si>
+  <si>
+    <t>62,12</t>
+  </si>
+  <si>
+    <t>6,09</t>
+  </si>
+  <si>
+    <t>10,22</t>
+  </si>
+  <si>
+    <t>5,06</t>
+  </si>
+  <si>
+    <t>3,25</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>14,83</t>
+  </si>
+  <si>
+    <t>1,57</t>
+  </si>
+  <si>
+    <t>38,19</t>
+  </si>
+  <si>
+    <t>4,14</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>14,5</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>1,49</t>
+  </si>
+  <si>
     <t>3,73</t>
   </si>
   <si>
-    <t>16,37</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>14,05</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>27,88</t>
-  </si>
-  <si>
-    <t>29,95</t>
-  </si>
-  <si>
-    <t>6,76</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>4,57</t>
-  </si>
-  <si>
-    <t>15,36</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>15,44</t>
-  </si>
-  <si>
-    <t>1,6</t>
-  </si>
-  <si>
-    <t>53,3</t>
-  </si>
-  <si>
-    <t>7,45</t>
-  </si>
-  <si>
-    <t>10,44</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>0,62</t>
-  </si>
-  <si>
-    <t>3,47</t>
-  </si>
-  <si>
-    <t>6,17</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>24,68</t>
-  </si>
-  <si>
-    <t>0,76</t>
-  </si>
-  <si>
-    <t>7,01</t>
-  </si>
-  <si>
-    <t>34,59</t>
-  </si>
-  <si>
-    <t>11,79</t>
-  </si>
-  <si>
-    <t>0,59</t>
-  </si>
-  <si>
-    <t>7,24</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>1,82</t>
-  </si>
-  <si>
-    <t>2,01</t>
-  </si>
-  <si>
-    <t>8,52</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>16,69</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>0,52</t>
-  </si>
-  <si>
-    <t>51,38</t>
-  </si>
-  <si>
-    <t>3,3</t>
-  </si>
-  <si>
-    <t>12,16</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>2,86</t>
-  </si>
-  <si>
-    <t>9,77</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>17,73</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>44,16</t>
-  </si>
-  <si>
-    <t>12,12</t>
-  </si>
-  <si>
-    <t>7,03</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>6,27</t>
-  </si>
-  <si>
-    <t>9,15</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>18,19</t>
-  </si>
-  <si>
-    <t>43,46</t>
-  </si>
-  <si>
-    <t>17,07</t>
-  </si>
-  <si>
-    <t>6,74</t>
-  </si>
-  <si>
-    <t>0,77</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>4,24</t>
-  </si>
-  <si>
-    <t>6,63</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>20,99</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>35,49</t>
-  </si>
-  <si>
-    <t>16,06</t>
-  </si>
-  <si>
-    <t>5,86</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>0,69</t>
-  </si>
-  <si>
-    <t>7,12</t>
-  </si>
-  <si>
-    <t>12,54</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>30,11</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>32,46</t>
-  </si>
-  <si>
-    <t>1,35</t>
-  </si>
-  <si>
-    <t>5,87</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>8,19</t>
-  </si>
-  <si>
-    <t>19,91</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>17,24</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>36,55</t>
-  </si>
-  <si>
-    <t>4,59</t>
-  </si>
-  <si>
-    <t>5,18</t>
-  </si>
-  <si>
-    <t>7,74</t>
-  </si>
-  <si>
-    <t>26,42</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>28,55</t>
-  </si>
-  <si>
-    <t>2,13</t>
-  </si>
-  <si>
-    <t>1,21</t>
-  </si>
-  <si>
-    <t>40,97</t>
-  </si>
-  <si>
-    <t>6,41</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>4,52</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>2,56</t>
-  </si>
-  <si>
-    <t>7,4</t>
-  </si>
-  <si>
-    <t>4,72</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>20,22</t>
-  </si>
-  <si>
-    <t>1,4</t>
-  </si>
-  <si>
-    <t>35,8</t>
-  </si>
-  <si>
-    <t>14,42</t>
-  </si>
-  <si>
-    <t>6,58</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>4,09</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>62,1</t>
-  </si>
-  <si>
-    <t>6,15</t>
-  </si>
-  <si>
-    <t>10,21</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>5,05</t>
-  </si>
-  <si>
-    <t>3,28</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>14,97</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>2,12</t>
-  </si>
-  <si>
-    <t>37,39</t>
-  </si>
-  <si>
-    <t>4,23</t>
-  </si>
-  <si>
-    <t>14,55</t>
-  </si>
-  <si>
-    <t>1,52</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>3,81</t>
-  </si>
-  <si>
-    <t>17,34</t>
-  </si>
-  <si>
     <t>1872</t>
   </si>
   <si>
     <t>METRO</t>
   </si>
   <si>
-    <t>16,03</t>
-  </si>
-  <si>
-    <t>5,57</t>
-  </si>
-  <si>
-    <t>31,34</t>
-  </si>
-  <si>
-    <t>3,84</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>2,97</t>
-  </si>
-  <si>
-    <t>0,71</t>
-  </si>
-  <si>
-    <t>3,65</t>
-  </si>
-  <si>
-    <t>34,05</t>
+    <t>16</t>
+  </si>
+  <si>
+    <t>5,53</t>
+  </si>
+  <si>
+    <t>31,77</t>
+  </si>
+  <si>
+    <t>3,76</t>
+  </si>
+  <si>
+    <t>2,99</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>3,87</t>
+  </si>
+  <si>
+    <t>34,17</t>
   </si>
   <si>
     <t/>
@@ -1899,106 +1866,106 @@
         <v>105</v>
       </c>
       <c r="C6" s="6">
-        <v>149053</v>
+        <v>152452</v>
       </c>
       <c r="D6" s="6">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>106</v>
       </c>
       <c r="F6" s="6">
-        <v>29475</v>
+        <v>30019</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H6" s="6">
-        <v>1485</v>
+        <v>1503</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="6">
-        <v>1948</v>
+        <v>1763</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>109</v>
       </c>
       <c r="L6" s="6">
-        <v>65700</v>
+        <v>68151</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N6" s="6">
-        <v>12552</v>
+        <v>12602</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>111</v>
       </c>
       <c r="P6" s="6">
-        <v>193</v>
+        <v>167</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>112</v>
       </c>
       <c r="R6" s="6">
-        <v>11681</v>
+        <v>12014</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>113</v>
       </c>
       <c r="T6" s="6">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="U6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="V6" s="6">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>115</v>
       </c>
       <c r="X6" s="6">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>116</v>
       </c>
       <c r="Z6" s="6">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>117</v>
       </c>
       <c r="AB6" s="6">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AD6" s="6">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="AE6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="AF6" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH6" s="6">
         <v>10</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AJ6" s="6">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AK6" s="7" t="s">
         <v>119</v>
@@ -2010,37 +1977,37 @@
         <v>120</v>
       </c>
       <c r="AN6" s="6">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="AO6" s="7" t="s">
         <v>121</v>
       </c>
       <c r="AP6" s="6">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="AQ6" s="7" t="s">
         <v>122</v>
       </c>
       <c r="AR6" s="6">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="AS6" s="7" t="s">
         <v>123</v>
       </c>
       <c r="AT6" s="6">
-        <v>848</v>
+        <v>757</v>
       </c>
       <c r="AU6" s="7" t="s">
         <v>124</v>
       </c>
       <c r="AV6" s="6">
-        <v>6962</v>
+        <v>7066</v>
       </c>
       <c r="AW6" s="7" t="s">
         <v>125</v>
       </c>
       <c r="AX6" s="6">
-        <v>16238</v>
+        <v>16418</v>
       </c>
       <c r="AY6" s="7" t="s">
         <v>126</v>
@@ -2054,127 +2021,127 @@
         <v>128</v>
       </c>
       <c r="C7" s="9">
-        <v>8331</v>
+        <v>8541</v>
       </c>
       <c r="D7" s="9">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="F7" s="9">
-        <v>1607</v>
+        <v>1646</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>129</v>
       </c>
       <c r="H7" s="9">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>130</v>
       </c>
       <c r="J7" s="9">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>131</v>
       </c>
       <c r="L7" s="9">
-        <v>3921</v>
+        <v>4004</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>132</v>
       </c>
       <c r="N7" s="9">
-        <v>430</v>
+        <v>449</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>133</v>
       </c>
       <c r="P7" s="9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R7" s="9">
+        <v>402</v>
+      </c>
+      <c r="S7" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="R7" s="9">
-        <v>391</v>
-      </c>
-      <c r="S7" s="10" t="s">
-        <v>135</v>
-      </c>
       <c r="T7" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="V7" s="9">
         <v>0</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X7" s="9">
         <v>18</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Z7" s="9">
         <v>2</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AB7" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AD7" s="9">
         <v>9</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="AF7" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="AH7" s="9">
         <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ7" s="9">
         <v>16</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AL7" s="9">
         <v>1</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AN7" s="9">
         <v>1</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AP7" s="9">
         <v>38</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AR7" s="9">
         <v>7</v>
@@ -2183,257 +2150,257 @@
         <v>123</v>
       </c>
       <c r="AT7" s="9">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="AU7" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AV7" s="9">
+        <v>320</v>
+      </c>
+      <c r="AW7" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="AX7" s="9">
+        <v>1465</v>
+      </c>
+      <c r="AY7" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="AV7" s="9">
-        <v>311</v>
-      </c>
-      <c r="AW7" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>1364</v>
-      </c>
-      <c r="AY7" s="10" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" s="9">
+        <v>3888</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F8" s="9">
+        <v>560</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>143</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="C8" s="9">
-        <v>3522</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F8" s="9">
-        <v>495</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>145</v>
       </c>
       <c r="H8" s="9">
         <v>17</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="L8" s="9">
-        <v>982</v>
+        <v>1267</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="N8" s="9">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="P8" s="9">
         <v>0</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R8" s="9">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="T8" s="9">
         <v>0</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V8" s="9">
         <v>0</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X8" s="9">
         <v>8</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="Z8" s="9">
         <v>0</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AB8" s="9">
         <v>0</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD8" s="9">
         <v>1</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="AF8" s="9">
         <v>0</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH8" s="9">
         <v>0</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ8" s="9">
         <v>5</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="AL8" s="9">
         <v>0</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP8" s="9">
         <v>16</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="AT8" s="9">
         <v>0</v>
       </c>
       <c r="AU8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AV8" s="9">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="AW8" s="10" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="AX8" s="9">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="AY8" s="10" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C9" s="9">
+        <v>12734</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="9">
+        <v>1909</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="H9" s="9">
+        <v>185</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="L9" s="9">
+        <v>6983</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="C9" s="9">
-        <v>11729</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F9" s="9">
-        <v>1811</v>
-      </c>
-      <c r="G9" s="10" t="s">
+      <c r="N9" s="9">
+        <v>879</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>157</v>
-      </c>
-      <c r="H9" s="9">
-        <v>188</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="J9" s="9">
-        <v>7</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="L9" s="9">
-        <v>6252</v>
-      </c>
-      <c r="M9" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="N9" s="9">
-        <v>874</v>
-      </c>
-      <c r="O9" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="P9" s="9">
         <v>1</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="R9" s="9">
-        <v>1224</v>
+        <v>1391</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="T9" s="9">
         <v>1</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="V9" s="9">
         <v>0</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X9" s="9">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="Z9" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA9" s="10" t="s">
         <v>118</v>
@@ -2442,156 +2409,156 @@
         <v>0</v>
       </c>
       <c r="AC9" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD9" s="9">
         <v>13</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="AF9" s="9">
         <v>0</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ9" s="9">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AL9" s="9">
         <v>0</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
         <v>115</v>
       </c>
       <c r="AP9" s="9">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>130</v>
+        <v>162</v>
       </c>
       <c r="AR9" s="9">
         <v>2</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AT9" s="9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AU9" s="10" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AV9" s="9">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="AW9" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="AX9" s="9">
+        <v>729</v>
+      </c>
+      <c r="AY9" s="10" t="s">
         <v>164</v>
-      </c>
-      <c r="AX9" s="9">
-        <v>724</v>
-      </c>
-      <c r="AY9" s="10" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>167</v>
-      </c>
       <c r="C10" s="9">
-        <v>22596</v>
+        <v>22762</v>
       </c>
       <c r="D10" s="9">
         <v>46</v>
       </c>
       <c r="E10" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="F10" s="9">
+        <v>5626</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>168</v>
-      </c>
-      <c r="F10" s="9">
-        <v>5576</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>169</v>
       </c>
       <c r="H10" s="9">
         <v>172</v>
       </c>
       <c r="I10" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="J10" s="9">
+        <v>1579</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="J10" s="9">
-        <v>1584</v>
-      </c>
-      <c r="K10" s="10" t="s">
+      <c r="L10" s="9">
+        <v>7896</v>
+      </c>
+      <c r="M10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="L10" s="9">
-        <v>7815</v>
-      </c>
-      <c r="M10" s="10" t="s">
+      <c r="N10" s="9">
+        <v>2687</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>172</v>
-      </c>
-      <c r="N10" s="9">
-        <v>2665</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>173</v>
       </c>
       <c r="P10" s="9">
         <v>134</v>
       </c>
       <c r="Q10" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="R10" s="9">
+        <v>1639</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>174</v>
-      </c>
-      <c r="R10" s="9">
-        <v>1637</v>
-      </c>
-      <c r="S10" s="10" t="s">
-        <v>175</v>
       </c>
       <c r="T10" s="9">
         <v>2</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="V10" s="9">
         <v>1</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X10" s="9">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>176</v>
+        <v>112</v>
       </c>
       <c r="Z10" s="9">
         <v>6</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="AB10" s="9">
         <v>9</v>
@@ -2603,13 +2570,13 @@
         <v>17</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="AF10" s="9">
         <v>0</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH10" s="9">
         <v>8</v>
@@ -2627,19 +2594,19 @@
         <v>1</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN10" s="9">
         <v>52</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="AP10" s="9">
         <v>34</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AR10" s="9">
         <v>10</v>
@@ -2651,150 +2618,150 @@
         <v>411</v>
       </c>
       <c r="AU10" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AV10" s="9">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="AW10" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="AX10" s="9">
         <v>1926</v>
       </c>
       <c r="AY10" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C11" s="9">
+        <v>17501</v>
+      </c>
+      <c r="D11" s="9">
+        <v>0</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" s="9">
+        <v>2930</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="H11" s="9">
+        <v>293</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="C11" s="9">
-        <v>17070</v>
-      </c>
-      <c r="D11" s="9">
-        <v>3</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F11" s="9">
-        <v>2849</v>
-      </c>
-      <c r="G11" s="10" t="s">
+      <c r="J11" s="9">
+        <v>1</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="L11" s="9">
+        <v>9127</v>
+      </c>
+      <c r="M11" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="H11" s="9">
-        <v>291</v>
-      </c>
-      <c r="I11" s="10" t="s">
+      <c r="N11" s="9">
+        <v>573</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="P11" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R11" s="9">
+        <v>2143</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>184</v>
-      </c>
-      <c r="J11" s="9">
-        <v>88</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="L11" s="9">
-        <v>8770</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="N11" s="9">
-        <v>564</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="P11" s="9">
-        <v>19</v>
-      </c>
-      <c r="Q11" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="R11" s="9">
-        <v>2076</v>
-      </c>
-      <c r="S11" s="10" t="s">
-        <v>188</v>
       </c>
       <c r="T11" s="9">
         <v>18</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="V11" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="X11" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="Z11" s="9">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="AB11" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AD11" s="9">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>177</v>
+        <v>136</v>
       </c>
       <c r="AF11" s="9">
         <v>0</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH11" s="9">
         <v>0</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ11" s="9">
         <v>48</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="AL11" s="9">
         <v>3</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AN11" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AP11" s="9">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="AR11" s="9">
         <v>10</v>
@@ -2803,248 +2770,248 @@
         <v>106</v>
       </c>
       <c r="AT11" s="9">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AU11" s="10" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="AV11" s="9">
-        <v>488</v>
+        <v>504</v>
       </c>
       <c r="AW11" s="10" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="AX11" s="9">
-        <v>1667</v>
+        <v>1679</v>
       </c>
       <c r="AY11" s="10" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C12" s="9">
+        <v>6117</v>
+      </c>
+      <c r="D12" s="9">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12" s="9">
+        <v>1094</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="H12" s="9">
+        <v>38</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="J12" s="9">
+        <v>18</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="L12" s="9">
+        <v>2728</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="N12" s="9">
+        <v>736</v>
+      </c>
+      <c r="O12" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="P12" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R12" s="9">
+        <v>433</v>
+      </c>
+      <c r="S12" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="C12" s="9">
-        <v>6046</v>
-      </c>
-      <c r="D12" s="9">
-        <v>0</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F12" s="9">
-        <v>1072</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="H12" s="9">
-        <v>39</v>
-      </c>
-      <c r="I12" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="J12" s="9">
-        <v>38</v>
-      </c>
-      <c r="K12" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="L12" s="9">
-        <v>2670</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="N12" s="9">
-        <v>733</v>
-      </c>
-      <c r="O12" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="P12" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R12" s="9">
-        <v>425</v>
-      </c>
-      <c r="S12" s="10" t="s">
-        <v>200</v>
-      </c>
       <c r="T12" s="9">
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V12" s="9">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X12" s="9">
         <v>28</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>139</v>
+        <v>196</v>
       </c>
       <c r="Z12" s="9">
         <v>2</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD12" s="9">
         <v>10</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>201</v>
+        <v>116</v>
       </c>
       <c r="AF12" s="9">
         <v>0</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH12" s="9">
         <v>0</v>
       </c>
       <c r="AI12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ12" s="9">
         <v>35</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>202</v>
+        <v>138</v>
       </c>
       <c r="AL12" s="9">
         <v>0</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN12" s="9">
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP12" s="9">
         <v>60</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="AR12" s="9">
         <v>1</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AT12" s="9">
         <v>1</v>
       </c>
       <c r="AU12" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AV12" s="9">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AW12" s="10" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="AX12" s="9">
         <v>553</v>
       </c>
       <c r="AY12" s="10" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C13" s="9">
-        <v>5442</v>
+        <v>5460</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F13" s="9">
-        <v>990</v>
+        <v>993</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="H13" s="9">
         <v>32</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J13" s="9">
         <v>3</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="L13" s="9">
-        <v>2365</v>
+        <v>2379</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="N13" s="9">
         <v>929</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="P13" s="9">
         <v>0</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R13" s="9">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="T13" s="9">
         <v>0</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V13" s="9">
         <v>1</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="X13" s="9">
         <v>4</v>
@@ -3056,502 +3023,502 @@
         <v>3</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="AB13" s="9">
         <v>0</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD13" s="9">
         <v>8</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AF13" s="9">
         <v>0</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH13" s="9">
         <v>0</v>
       </c>
       <c r="AI13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ13" s="9">
         <v>42</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="AL13" s="9">
         <v>11</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AN13" s="9">
         <v>0</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP13" s="9">
         <v>65</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="AR13" s="9">
         <v>27</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="AT13" s="9">
         <v>3</v>
       </c>
       <c r="AU13" s="10" t="s">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="AV13" s="9">
         <v>231</v>
       </c>
       <c r="AW13" s="10" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="AX13" s="9">
         <v>361</v>
       </c>
       <c r="AY13" s="10" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C14" s="9">
-        <v>5798</v>
+        <v>6211</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F14" s="9">
-        <v>1217</v>
+        <v>1277</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="H14" s="9">
         <v>23</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="J14" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="L14" s="9">
-        <v>2058</v>
+        <v>2383</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="N14" s="9">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="P14" s="9">
         <v>0</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R14" s="9">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="T14" s="9">
         <v>3</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="V14" s="9">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X14" s="9">
         <v>10</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>201</v>
+        <v>116</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD14" s="9">
         <v>5</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>176</v>
+        <v>123</v>
       </c>
       <c r="AF14" s="9">
         <v>0</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ14" s="9">
         <v>20</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="AL14" s="9">
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AN14" s="9">
         <v>0</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP14" s="9">
         <v>40</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="AR14" s="9">
         <v>2</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="AT14" s="9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AU14" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AV14" s="9">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="AW14" s="10" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="AX14" s="9">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="AY14" s="10" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C15" s="9">
-        <v>13132</v>
+        <v>13298</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F15" s="9">
-        <v>3954</v>
+        <v>3975</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="H15" s="9">
         <v>52</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="J15" s="9">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>231</v>
+        <v>120</v>
       </c>
       <c r="L15" s="9">
-        <v>4263</v>
+        <v>4405</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N15" s="9">
         <v>177</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="P15" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="10" t="s">
         <v>115</v>
       </c>
       <c r="R15" s="9">
-        <v>771</v>
+        <v>784</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="T15" s="9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="V15" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W15" s="10" t="s">
         <v>115</v>
       </c>
       <c r="X15" s="9">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="Z15" s="9">
         <v>0</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD15" s="9">
         <v>3</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AF15" s="9">
         <v>0</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH15" s="9">
         <v>0</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ15" s="9">
         <v>13</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="AL15" s="9">
         <v>2</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AN15" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AO15" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AP15" s="9">
         <v>84</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="AR15" s="9">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="AT15" s="9">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="AU15" s="10" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="AV15" s="9">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="AW15" s="10" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="AX15" s="9">
-        <v>2615</v>
+        <v>2641</v>
       </c>
       <c r="AY15" s="10" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C16" s="9">
-        <v>5749</v>
+        <v>5777</v>
       </c>
       <c r="D16" s="9">
         <v>0</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F16" s="9">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="H16" s="9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>243</v>
+        <v>138</v>
       </c>
       <c r="J16" s="9">
         <v>0</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="L16" s="9">
-        <v>2101</v>
+        <v>2147</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="N16" s="9">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="P16" s="9">
         <v>0</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R16" s="9">
         <v>298</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="T16" s="9">
         <v>0</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X16" s="9">
         <v>7</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>237</v>
+        <v>131</v>
       </c>
       <c r="Z16" s="9">
         <v>3</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="AB16" s="9">
         <v>0</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD16" s="9">
         <v>3</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="AF16" s="9">
         <v>1</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AH16" s="9">
         <v>0</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ16" s="9">
         <v>30</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>185</v>
+        <v>122</v>
       </c>
       <c r="AL16" s="9">
         <v>4</v>
@@ -3563,102 +3530,102 @@
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP16" s="9">
         <v>44</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>212</v>
+        <v>169</v>
       </c>
       <c r="AR16" s="9">
         <v>7</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>237</v>
+        <v>131</v>
       </c>
       <c r="AT16" s="9">
         <v>0</v>
       </c>
       <c r="AU16" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AV16" s="9">
         <v>445</v>
       </c>
       <c r="AW16" s="10" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="AX16" s="9">
         <v>1519</v>
       </c>
       <c r="AY16" s="10" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C17" s="9">
-        <v>10622</v>
+        <v>10709</v>
       </c>
       <c r="D17" s="9">
         <v>33</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>235</v>
+        <v>159</v>
       </c>
       <c r="F17" s="9">
-        <v>3033</v>
+        <v>3054</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="H17" s="9">
         <v>226</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="J17" s="9">
         <v>128</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="L17" s="9">
-        <v>4352</v>
+        <v>4410</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="N17" s="9">
         <v>681</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="P17" s="9">
         <v>22</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>256</v>
+        <v>135</v>
       </c>
       <c r="R17" s="9">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="T17" s="9">
         <v>1</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="V17" s="9">
         <v>4</v>
@@ -3682,7 +3649,7 @@
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AD17" s="9">
         <v>4</v>
@@ -3694,490 +3661,490 @@
         <v>0</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH17" s="9">
         <v>2</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AJ17" s="9">
         <v>16</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AL17" s="9">
         <v>3</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="AN17" s="9">
         <v>8</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="AP17" s="9">
         <v>44</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>258</v>
+        <v>148</v>
       </c>
       <c r="AR17" s="9">
         <v>11</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="AT17" s="9">
         <v>272</v>
       </c>
       <c r="AU17" s="10" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="AV17" s="9">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="AW17" s="10" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="AX17" s="9">
         <v>501</v>
       </c>
       <c r="AY17" s="10" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="C18" s="9">
-        <v>11285</v>
+        <v>11299</v>
       </c>
       <c r="D18" s="9">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="F18" s="9">
-        <v>2282</v>
+        <v>2283</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="H18" s="9">
         <v>158</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="J18" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="10" t="s">
         <v>118</v>
       </c>
       <c r="L18" s="9">
-        <v>4040</v>
+        <v>4044</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="N18" s="9">
         <v>1627</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>267</v>
+        <v>143</v>
       </c>
       <c r="P18" s="9">
         <v>0</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R18" s="9">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="T18" s="9">
         <v>30</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>231</v>
+        <v>185</v>
       </c>
       <c r="V18" s="9">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X18" s="9">
         <v>11</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="Z18" s="9">
         <v>1</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AB18" s="9">
         <v>0</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD18" s="9">
         <v>6</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="AF18" s="9">
         <v>0</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH18" s="9">
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ18" s="9">
         <v>11</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="AL18" s="9">
         <v>10</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>176</v>
+        <v>258</v>
       </c>
       <c r="AN18" s="9">
         <v>0</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP18" s="9">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="AR18" s="9">
         <v>17</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AT18" s="9">
         <v>0</v>
       </c>
       <c r="AU18" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AV18" s="9">
         <v>462</v>
       </c>
       <c r="AW18" s="10" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="AX18" s="9">
         <v>1847</v>
       </c>
       <c r="AY18" s="10" t="s">
-        <v>142</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="C19" s="9">
-        <v>23891</v>
+        <v>24235</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F19" s="9">
-        <v>2995</v>
+        <v>3069</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>227</v>
+        <v>264</v>
       </c>
       <c r="H19" s="9">
         <v>24</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="J19" s="9">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="L19" s="9">
-        <v>14836</v>
+        <v>15055</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="N19" s="9">
-        <v>1470</v>
+        <v>1476</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="R19" s="9">
-        <v>2440</v>
+        <v>2478</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="T19" s="9">
         <v>0</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V19" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X19" s="9">
         <v>23</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>189</v>
+        <v>258</v>
       </c>
       <c r="Z19" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AB19" s="9">
         <v>0</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD19" s="9">
         <v>0</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AF19" s="9">
         <v>3</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AH19" s="9">
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ19" s="9">
         <v>21</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>176</v>
+        <v>258</v>
       </c>
       <c r="AL19" s="9">
         <v>0</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP19" s="9">
         <v>70</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>276</v>
+        <v>192</v>
       </c>
       <c r="AR19" s="9">
         <v>1</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AT19" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU19" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AV19" s="9">
-        <v>1207</v>
+        <v>1226</v>
       </c>
       <c r="AW19" s="10" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="AX19" s="9">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="AY19" s="10" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="C20" s="9">
-        <v>1182</v>
+        <v>1207</v>
       </c>
       <c r="D20" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F20" s="9">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>282</v>
+        <v>124</v>
       </c>
       <c r="J20" s="9">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="L20" s="9">
-        <v>442</v>
+        <v>461</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="N20" s="9">
         <v>50</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="P20" s="9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="R20" s="9">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="T20" s="9">
         <v>0</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V20" s="9">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X20" s="9">
         <v>9</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>170</v>
+        <v>278</v>
       </c>
       <c r="Z20" s="9">
         <v>4</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>224</v>
+        <v>279</v>
       </c>
       <c r="AB20" s="9">
         <v>0</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD20" s="9">
         <v>0</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AF20" s="9">
         <v>0</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH20" s="9">
         <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ20" s="9">
         <v>7</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="AL20" s="9">
         <v>2</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>201</v>
+        <v>276</v>
       </c>
       <c r="AN20" s="9">
         <v>1</v>
@@ -4189,60 +4156,60 @@
         <v>18</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="AR20" s="9">
         <v>5</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>288</v>
+        <v>148</v>
       </c>
       <c r="AT20" s="9">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="AU20" s="10" t="s">
-        <v>289</v>
+        <v>227</v>
       </c>
       <c r="AV20" s="9">
         <v>45</v>
       </c>
       <c r="AW20" s="10" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="AX20" s="9">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="AY20" s="10" t="s">
-        <v>291</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="C21" s="9">
-        <v>2658</v>
+        <v>2713</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F21" s="9">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="H21" s="9">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
@@ -4251,100 +4218,100 @@
         <v>121</v>
       </c>
       <c r="L21" s="9">
-        <v>833</v>
+        <v>862</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="N21" s="9">
         <v>102</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="P21" s="9">
         <v>8</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>298</v>
+        <v>192</v>
       </c>
       <c r="R21" s="9">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="T21" s="9">
         <v>0</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V21" s="9">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="X21" s="9">
         <v>17</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="Z21" s="9">
         <v>2</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="AB21" s="9">
         <v>0</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AD21" s="9">
         <v>0</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AF21" s="9">
         <v>0</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AJ21" s="9">
         <v>3</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="AL21" s="9">
         <v>0</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AP21" s="9">
         <v>19</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="AR21" s="9">
         <v>1</v>
@@ -4353,132 +4320,132 @@
         <v>121</v>
       </c>
       <c r="AT21" s="9">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AU21" s="10" t="s">
-        <v>236</v>
+        <v>121</v>
       </c>
       <c r="AV21" s="9">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="AW21" s="10" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="AX21" s="9">
-        <v>905</v>
+        <v>927</v>
       </c>
       <c r="AY21" s="10" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="C22" s="12">
-        <v>149053</v>
+        <v>152452</v>
       </c>
       <c r="D22" s="12">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="F22" s="12">
-        <v>29475</v>
+        <v>30019</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H22" s="12">
-        <v>1485</v>
+        <v>1503</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J22" s="12">
-        <v>1948</v>
+        <v>1763</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="L22" s="12">
-        <v>65700</v>
+        <v>68151</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>110</v>
       </c>
       <c r="N22" s="12">
-        <v>12552</v>
+        <v>12602</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>111</v>
       </c>
       <c r="P22" s="12">
-        <v>193</v>
+        <v>167</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R22" s="12">
-        <v>11681</v>
+        <v>12014</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>113</v>
       </c>
       <c r="T22" s="12">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="U22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="V22" s="12">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>115</v>
       </c>
       <c r="X22" s="12">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="Z22" s="12">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>117</v>
       </c>
       <c r="AB22" s="12">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AD22" s="12">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="AE22" s="13" t="s">
         <v>114</v>
       </c>
       <c r="AF22" s="12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AH22" s="12">
         <v>10</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="AJ22" s="12">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AK22" s="13" t="s">
         <v>119</v>
@@ -4490,37 +4457,37 @@
         <v>120</v>
       </c>
       <c r="AN22" s="12">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="AO22" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AP22" s="12">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="AQ22" s="13" t="s">
         <v>122</v>
       </c>
       <c r="AR22" s="12">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="AS22" s="13" t="s">
         <v>123</v>
       </c>
       <c r="AT22" s="12">
-        <v>848</v>
+        <v>757</v>
       </c>
       <c r="AU22" s="13" t="s">
         <v>124</v>
       </c>
       <c r="AV22" s="12">
-        <v>6962</v>
+        <v>7066</v>
       </c>
       <c r="AW22" s="13" t="s">
         <v>125</v>
       </c>
       <c r="AX22" s="12">
-        <v>16238</v>
+        <v>16418</v>
       </c>
       <c r="AY22" s="13" t="s">
         <v>126</v>

</xml_diff>